<commit_message>
Added new inventories for biogas purification technologies
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF8BD208-F231-4C2C-AD11-8661DC65CD46}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C3EF791-C10F-491E-BB03-3273FECC7A9E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1844" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2245" uniqueCount="290">
   <si>
     <t>Database</t>
   </si>
@@ -820,18 +820,6 @@
   </si>
   <si>
     <t>market for inorganic nitrogen fertiliser, as N</t>
-  </si>
-  <si>
-    <t>activity type</t>
-  </si>
-  <si>
-    <t>ordinary transforming activity</t>
-  </si>
-  <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>e413022065fd99c773b8664679178c5f_copy1</t>
   </si>
   <si>
     <t>The data presented is derived from information available from the manufacturer of biogas upgrading plants. The upgraded gas leaves the process with a pressure of 5 bar. For the composition of the product gas we assume a share of more than 96 Vol. % of methane.
@@ -840,18 +828,6 @@
 Technology:  Membrane technology</t>
   </si>
   <si>
-    <t>filename</t>
-  </si>
-  <si>
-    <t>75233bc2-3805-52eb-8459-4bf104a8a5dc_3f14ad74-3caf-4ddc-9155-c78e40f80a14.spold</t>
-  </si>
-  <si>
-    <t>flow</t>
-  </si>
-  <si>
-    <t>3f14ad74-3caf-4ddc-9155-c78e40f80a14</t>
-  </si>
-  <si>
     <t>biomethane, high pressure</t>
   </si>
   <si>
@@ -882,9 +858,6 @@
     <t>steel, chromium steel 18/8</t>
   </si>
   <si>
-    <t>biogas purification to biomethane by membrane</t>
-  </si>
-  <si>
     <t>market for biogas to biomethane, Tr2050</t>
   </si>
   <si>
@@ -895,17 +868,63 @@
   </si>
   <si>
     <t>nothing</t>
+  </si>
+  <si>
+    <t>biogas purification to biomethane by chemical scrubbing, Tr2050</t>
+  </si>
+  <si>
+    <t>market for monoethanolamine</t>
+  </si>
+  <si>
+    <t>monoethanolamine</t>
+  </si>
+  <si>
+    <t>market for charcoal</t>
+  </si>
+  <si>
+    <t>charcoal</t>
+  </si>
+  <si>
+    <t>market for chemical, organic</t>
+  </si>
+  <si>
+    <t>chemical, organic</t>
+  </si>
+  <si>
+    <t>market for potassium hydroxide</t>
+  </si>
+  <si>
+    <t>potassium hydroxide</t>
+  </si>
+  <si>
+    <t>market for sodium chloride, powder</t>
+  </si>
+  <si>
+    <t>sodium chloride, powder</t>
+  </si>
+  <si>
+    <t>Ammonia</t>
+  </si>
+  <si>
+    <t>biogas purification to biomethane by membrane, Tr2050</t>
+  </si>
+  <si>
+    <t>biogas purification to biomethane by water scrubbing, Tr2050</t>
+  </si>
+  <si>
+    <t>biogas purification to biomethane by PSA, Tr2050</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000E+00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000000000"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1024,13 +1043,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Consolas"/>
-      <family val="3"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1060,6 +1074,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1086,7 +1106,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1161,13 +1181,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
@@ -1456,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH436"/>
+  <dimension ref="A1:AH513"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="55.44140625" customWidth="1"/>
@@ -4955,7 +4974,7 @@
       <c r="I166" s="36"/>
     </row>
     <row r="167" spans="1:9">
-      <c r="A167" s="60"/>
+      <c r="A167" s="36"/>
       <c r="B167" s="36"/>
       <c r="C167" s="36"/>
       <c r="D167" s="36"/>
@@ -4970,7 +4989,7 @@
         <v>1</v>
       </c>
       <c r="B168" s="30" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -4986,7 +5005,7 @@
         <v>11</v>
       </c>
       <c r="B170" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -5008,7 +5027,7 @@
         <v>4</v>
       </c>
       <c r="B173" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -13099,174 +13118,226 @@
       <c r="AG398" s="41"/>
       <c r="AH398" s="41"/>
     </row>
-    <row r="399" spans="1:34" ht="15.6">
-      <c r="A399" s="30" t="s">
+    <row r="399" spans="1:34">
+      <c r="A399" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B399" s="30" t="s">
-        <v>279</v>
+      <c r="B399" s="43" t="s">
+        <v>287</v>
       </c>
       <c r="I399"/>
     </row>
     <row r="400" spans="1:34">
-      <c r="A400" t="s">
+      <c r="A400" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B400" s="59" t="s">
         <v>260</v>
       </c>
-      <c r="B400" t="s">
+      <c r="I400"/>
+    </row>
+    <row r="401" spans="1:9">
+      <c r="A401" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B401" t="s">
+        <v>29</v>
+      </c>
+      <c r="I401"/>
+    </row>
+    <row r="402" spans="1:9">
+      <c r="A402" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B402" s="47">
+        <v>1</v>
+      </c>
+      <c r="I402"/>
+    </row>
+    <row r="403" spans="1:9">
+      <c r="A403" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B403" t="s">
         <v>261</v>
       </c>
-      <c r="I400"/>
-    </row>
-    <row r="401" spans="1:9">
-      <c r="A401" t="s">
-        <v>262</v>
-      </c>
-      <c r="B401" t="s">
-        <v>263</v>
-      </c>
-      <c r="I401"/>
-    </row>
-    <row r="402" spans="1:9">
-      <c r="A402" t="s">
+      <c r="I403"/>
+    </row>
+    <row r="404" spans="1:9">
+      <c r="A404" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B404" t="s">
+        <v>128</v>
+      </c>
+      <c r="I404"/>
+    </row>
+    <row r="405" spans="1:9">
+      <c r="A405" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B405"/>
+      <c r="I405"/>
+    </row>
+    <row r="406" spans="1:9" ht="15.6">
+      <c r="A406" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B406"/>
+      <c r="I406"/>
+    </row>
+    <row r="407" spans="1:9" s="46" customFormat="1">
+      <c r="A407" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B407" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C407" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D407" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E407" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F407" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G407" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H407" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="I407" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="B402" t="s">
-        <v>264</v>
-      </c>
-      <c r="I402"/>
-    </row>
-    <row r="403" spans="1:9">
-      <c r="A403" t="s">
-        <v>265</v>
-      </c>
-      <c r="B403" t="s">
-        <v>266</v>
-      </c>
-      <c r="I403"/>
-    </row>
-    <row r="404" spans="1:9">
-      <c r="A404" t="s">
-        <v>267</v>
-      </c>
-      <c r="B404" t="s">
-        <v>268</v>
-      </c>
-      <c r="I404"/>
-    </row>
-    <row r="405" spans="1:9">
-      <c r="A405" t="s">
-        <v>2</v>
-      </c>
-      <c r="B405" t="s">
-        <v>29</v>
-      </c>
-      <c r="I405"/>
-    </row>
-    <row r="406" spans="1:9">
-      <c r="A406" t="s">
-        <v>3</v>
-      </c>
-      <c r="B406">
-        <v>1</v>
-      </c>
-      <c r="I406"/>
-    </row>
-    <row r="407" spans="1:9">
-      <c r="A407" t="s">
-        <v>4</v>
-      </c>
-      <c r="B407" t="s">
-        <v>269</v>
-      </c>
-      <c r="I407"/>
     </row>
     <row r="408" spans="1:9">
       <c r="A408" t="s">
-        <v>5</v>
+        <v>287</v>
       </c>
       <c r="B408" t="s">
-        <v>78</v>
-      </c>
-      <c r="I408"/>
+        <v>261</v>
+      </c>
+      <c r="C408">
+        <v>1</v>
+      </c>
+      <c r="D408" t="s">
+        <v>128</v>
+      </c>
+      <c r="E408" s="50"/>
+      <c r="G408" t="s">
+        <v>29</v>
+      </c>
+      <c r="H408" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="409" spans="1:9">
       <c r="A409" t="s">
+        <v>266</v>
+      </c>
+      <c r="B409" t="s">
+        <v>267</v>
+      </c>
+      <c r="C409">
+        <f>10.2555323734231/1000</f>
+        <v>1.0255532373423099E-2</v>
+      </c>
+      <c r="D409" t="s">
+        <v>13</v>
+      </c>
+      <c r="E409" t="s">
+        <v>211</v>
+      </c>
+      <c r="G409" t="s">
+        <v>140</v>
+      </c>
+      <c r="H409" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="410" spans="1:9">
+      <c r="A410" t="s">
+        <v>268</v>
+      </c>
+      <c r="B410" t="s">
+        <v>135</v>
+      </c>
+      <c r="C410">
+        <v>5.4000000000000001E-11</v>
+      </c>
+      <c r="D410" t="s">
         <v>6</v>
       </c>
-      <c r="B409" t="s">
-        <v>128</v>
-      </c>
-      <c r="I409"/>
-    </row>
-    <row r="410" spans="1:9" ht="15.6">
-      <c r="A410" s="30" t="s">
-        <v>7</v>
-      </c>
-      <c r="B410"/>
-      <c r="I410"/>
-    </row>
-    <row r="411" spans="1:9" s="46" customFormat="1">
-      <c r="A411" s="46" t="s">
-        <v>8</v>
-      </c>
-      <c r="B411" s="46" t="s">
-        <v>4</v>
-      </c>
-      <c r="C411" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="D411" s="46" t="s">
-        <v>6</v>
-      </c>
-      <c r="E411" s="46" t="s">
-        <v>106</v>
-      </c>
-      <c r="F411" s="46" t="s">
-        <v>10</v>
-      </c>
-      <c r="G411" s="46" t="s">
-        <v>2</v>
-      </c>
-      <c r="H411" s="46" t="s">
-        <v>5</v>
-      </c>
-      <c r="I411" s="46" t="s">
-        <v>11</v>
+      <c r="E410" t="s">
+        <v>211</v>
+      </c>
+      <c r="G410" t="s">
+        <v>140</v>
+      </c>
+      <c r="H410" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="411" spans="1:9">
+      <c r="A411" t="s">
+        <v>28</v>
+      </c>
+      <c r="B411" t="s">
+        <v>20</v>
+      </c>
+      <c r="C411">
+        <v>0.97686420144549235</v>
+      </c>
+      <c r="D411" t="s">
+        <v>19</v>
+      </c>
+      <c r="E411" t="s">
+        <v>211</v>
+      </c>
+      <c r="G411" t="s">
+        <v>27</v>
+      </c>
+      <c r="H411" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="412" spans="1:9">
       <c r="A412" t="s">
-        <v>279</v>
+        <v>180</v>
       </c>
       <c r="B412" t="s">
-        <v>269</v>
+        <v>181</v>
       </c>
       <c r="C412">
-        <v>1</v>
+        <v>1.1400000000000001E-4</v>
       </c>
       <c r="D412" t="s">
-        <v>128</v>
-      </c>
-      <c r="E412" s="50" t="s">
-        <v>198</v>
+        <v>13</v>
+      </c>
+      <c r="E412" t="s">
+        <v>211</v>
       </c>
       <c r="G412" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="H412" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="413" spans="1:9">
       <c r="A413" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B413" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C413">
-        <f>10.2555323734231/1000</f>
-        <v>1.0255532373423099E-2</v>
+        <v>1.01E-4</v>
       </c>
       <c r="D413" t="s">
         <v>13</v>
@@ -13283,22 +13354,19 @@
     </row>
     <row r="414" spans="1:9">
       <c r="A414" t="s">
-        <v>276</v>
-      </c>
-      <c r="B414" t="s">
-        <v>135</v>
+        <v>271</v>
+      </c>
+      <c r="B414" s="19" t="s">
+        <v>197</v>
       </c>
       <c r="C414">
-        <v>5.4000000000000001E-11</v>
-      </c>
-      <c r="D414" t="s">
-        <v>6</v>
-      </c>
-      <c r="E414" t="s">
-        <v>211</v>
-      </c>
-      <c r="G414" t="s">
-        <v>140</v>
+        <v>1.8841794028909846</v>
+      </c>
+      <c r="D414" s="45" t="s">
+        <v>128</v>
+      </c>
+      <c r="G414" s="50" t="s">
+        <v>29</v>
       </c>
       <c r="H414" t="s">
         <v>12</v>
@@ -13306,100 +13374,95 @@
     </row>
     <row r="415" spans="1:9">
       <c r="A415" t="s">
-        <v>28</v>
-      </c>
-      <c r="B415" t="s">
-        <v>20</v>
-      </c>
+        <v>218</v>
+      </c>
+      <c r="B415"/>
       <c r="C415">
-        <v>0.97686420144549235</v>
+        <v>1.7520580065460971</v>
       </c>
       <c r="D415" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E415" t="s">
-        <v>211</v>
-      </c>
-      <c r="G415" t="s">
-        <v>27</v>
+        <v>109</v>
+      </c>
+      <c r="F415" t="s">
+        <v>184</v>
       </c>
       <c r="H415" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="416" spans="1:9">
       <c r="A416" t="s">
-        <v>180</v>
-      </c>
-      <c r="B416" t="s">
-        <v>181</v>
-      </c>
+        <v>262</v>
+      </c>
+      <c r="B416"/>
       <c r="C416">
-        <v>1.1400000000000001E-4</v>
+        <v>1.28</v>
       </c>
       <c r="D416" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E416" t="s">
-        <v>211</v>
-      </c>
-      <c r="G416" t="s">
-        <v>49</v>
+        <v>109</v>
+      </c>
+      <c r="F416" t="s">
+        <v>184</v>
       </c>
       <c r="H416" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="417" spans="1:9">
       <c r="A417" t="s">
-        <v>277</v>
-      </c>
-      <c r="B417" t="s">
-        <v>278</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="B417"/>
       <c r="C417">
-        <v>1.01E-4</v>
+        <v>0</v>
       </c>
       <c r="D417" t="s">
         <v>13</v>
       </c>
       <c r="E417" t="s">
-        <v>211</v>
-      </c>
-      <c r="G417" t="s">
-        <v>140</v>
+        <v>109</v>
+      </c>
+      <c r="F417" t="s">
+        <v>184</v>
       </c>
       <c r="H417" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="418" spans="1:9">
-      <c r="A418" s="56" t="s">
-        <v>280</v>
-      </c>
-      <c r="B418" s="19" t="s">
-        <v>197</v>
-      </c>
+      <c r="A418" t="s">
+        <v>185</v>
+      </c>
+      <c r="B418"/>
       <c r="C418">
-        <v>1.8841794028909846</v>
-      </c>
-      <c r="D418" s="45" t="s">
-        <v>128</v>
-      </c>
-      <c r="G418" s="50" t="s">
-        <v>29</v>
+        <v>7.0244489999999995E-3</v>
+      </c>
+      <c r="D418" t="s">
+        <v>13</v>
+      </c>
+      <c r="E418" t="s">
+        <v>109</v>
+      </c>
+      <c r="F418" t="s">
+        <v>184</v>
       </c>
       <c r="H418" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="419" spans="1:9">
       <c r="A419" t="s">
-        <v>218</v>
+        <v>264</v>
       </c>
       <c r="B419"/>
       <c r="C419">
-        <v>1.7520580065460971</v>
+        <v>5.1560000000000002E-2</v>
       </c>
       <c r="D419" t="s">
         <v>13</v>
@@ -13408,7 +13471,7 @@
         <v>109</v>
       </c>
       <c r="F419" t="s">
-        <v>184</v>
+        <v>25</v>
       </c>
       <c r="H419" t="s">
         <v>15</v>
@@ -13416,154 +13479,1707 @@
     </row>
     <row r="420" spans="1:9">
       <c r="A420" t="s">
-        <v>270</v>
+        <v>125</v>
       </c>
       <c r="B420"/>
       <c r="C420">
-        <v>1.28</v>
+        <v>6.5989999999999998E-6</v>
       </c>
       <c r="D420" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="E420" t="s">
         <v>109</v>
       </c>
       <c r="F420" t="s">
-        <v>184</v>
+        <v>265</v>
       </c>
       <c r="H420" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="421" spans="1:9">
-      <c r="A421" t="s">
+    <row r="421" spans="1:9" s="56" customFormat="1">
+      <c r="B421" s="57"/>
+      <c r="I421" s="58"/>
+    </row>
+    <row r="422" spans="1:9">
+      <c r="A422" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B422" s="43" t="s">
+        <v>275</v>
+      </c>
+      <c r="I422"/>
+    </row>
+    <row r="423" spans="1:9">
+      <c r="A423" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B423" s="59"/>
+      <c r="I423"/>
+    </row>
+    <row r="424" spans="1:9">
+      <c r="A424" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B424" t="s">
+        <v>29</v>
+      </c>
+      <c r="I424"/>
+    </row>
+    <row r="425" spans="1:9">
+      <c r="A425" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B425" s="47">
+        <v>1</v>
+      </c>
+      <c r="I425"/>
+    </row>
+    <row r="426" spans="1:9">
+      <c r="A426" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B426" t="s">
+        <v>261</v>
+      </c>
+      <c r="I426"/>
+    </row>
+    <row r="427" spans="1:9">
+      <c r="A427" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B427" t="s">
+        <v>128</v>
+      </c>
+      <c r="I427"/>
+    </row>
+    <row r="428" spans="1:9">
+      <c r="A428" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B428"/>
+      <c r="I428"/>
+    </row>
+    <row r="429" spans="1:9" ht="15.6">
+      <c r="A429" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B429"/>
+      <c r="I429"/>
+    </row>
+    <row r="430" spans="1:9" s="46" customFormat="1">
+      <c r="A430" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B430" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C430" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D430" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E430" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F430" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G430" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H430" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="I430" s="46" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="431" spans="1:9">
+      <c r="A431" t="s">
+        <v>275</v>
+      </c>
+      <c r="B431" t="s">
+        <v>261</v>
+      </c>
+      <c r="C431">
+        <v>1</v>
+      </c>
+      <c r="D431" t="s">
+        <v>128</v>
+      </c>
+      <c r="E431" s="50"/>
+      <c r="G431" t="s">
+        <v>29</v>
+      </c>
+      <c r="H431" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="432" spans="1:9">
+      <c r="A432" t="s">
+        <v>266</v>
+      </c>
+      <c r="B432" t="s">
+        <v>267</v>
+      </c>
+      <c r="C432">
+        <v>1.0255532373423097E-2</v>
+      </c>
+      <c r="D432" t="s">
+        <v>13</v>
+      </c>
+      <c r="E432" t="s">
+        <v>211</v>
+      </c>
+      <c r="G432" t="s">
+        <v>140</v>
+      </c>
+      <c r="H432" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="433" spans="1:8">
+      <c r="A433" t="s">
+        <v>268</v>
+      </c>
+      <c r="B433" t="s">
+        <v>135</v>
+      </c>
+      <c r="C433">
+        <v>5.4000000000000001E-11</v>
+      </c>
+      <c r="D433" t="s">
+        <v>6</v>
+      </c>
+      <c r="E433" t="s">
+        <v>211</v>
+      </c>
+      <c r="G433" t="s">
+        <v>140</v>
+      </c>
+      <c r="H433" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="434" spans="1:8">
+      <c r="A434" t="s">
+        <v>28</v>
+      </c>
+      <c r="B434" t="s">
+        <v>20</v>
+      </c>
+      <c r="C434">
+        <v>0.75934029794307212</v>
+      </c>
+      <c r="D434" t="s">
+        <v>19</v>
+      </c>
+      <c r="E434" t="s">
+        <v>211</v>
+      </c>
+      <c r="G434" t="s">
+        <v>27</v>
+      </c>
+      <c r="H434" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="435" spans="1:8">
+      <c r="A435" t="s">
+        <v>180</v>
+      </c>
+      <c r="B435" t="s">
+        <v>181</v>
+      </c>
+      <c r="C435">
+        <v>1.1400000000000001E-4</v>
+      </c>
+      <c r="D435" t="s">
+        <v>13</v>
+      </c>
+      <c r="E435" t="s">
+        <v>211</v>
+      </c>
+      <c r="G435" t="s">
+        <v>49</v>
+      </c>
+      <c r="H435" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="436" spans="1:8">
+      <c r="A436" t="s">
+        <v>269</v>
+      </c>
+      <c r="B436" t="s">
+        <v>270</v>
+      </c>
+      <c r="C436">
+        <v>1.01E-4</v>
+      </c>
+      <c r="D436" t="s">
+        <v>13</v>
+      </c>
+      <c r="E436" t="s">
+        <v>211</v>
+      </c>
+      <c r="G436" t="s">
+        <v>140</v>
+      </c>
+      <c r="H436" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="437" spans="1:8">
+      <c r="A437" t="s">
         <v>271</v>
       </c>
-      <c r="B421"/>
-      <c r="C421">
+      <c r="B437" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C437">
+        <v>1.9058925655516348</v>
+      </c>
+      <c r="D437" s="45" t="s">
+        <v>128</v>
+      </c>
+      <c r="G437" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="H437" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="438" spans="1:8">
+      <c r="A438" t="s">
+        <v>218</v>
+      </c>
+      <c r="B438"/>
+      <c r="C438">
+        <v>1.8087898191725484</v>
+      </c>
+      <c r="D438" t="s">
+        <v>13</v>
+      </c>
+      <c r="E438" t="s">
+        <v>109</v>
+      </c>
+      <c r="F438" t="s">
+        <v>184</v>
+      </c>
+      <c r="H438" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="439" spans="1:8">
+      <c r="A439" t="s">
+        <v>262</v>
+      </c>
+      <c r="B439"/>
+      <c r="C439">
+        <v>1.28</v>
+      </c>
+      <c r="D439" t="s">
+        <v>46</v>
+      </c>
+      <c r="E439" t="s">
+        <v>109</v>
+      </c>
+      <c r="F439" t="s">
+        <v>184</v>
+      </c>
+      <c r="H439" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="440" spans="1:8">
+      <c r="A440" t="s">
+        <v>263</v>
+      </c>
+      <c r="B440"/>
+      <c r="C440">
         <v>0</v>
       </c>
-      <c r="D421" t="s">
-        <v>13</v>
-      </c>
-      <c r="E421" t="s">
+      <c r="D440" t="s">
+        <v>13</v>
+      </c>
+      <c r="E440" t="s">
         <v>109</v>
       </c>
-      <c r="F421" t="s">
+      <c r="F440" t="s">
         <v>184</v>
       </c>
-      <c r="H421" t="s">
+      <c r="H440" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="422" spans="1:9">
-      <c r="A422" t="s">
+    <row r="441" spans="1:8">
+      <c r="A441" t="s">
         <v>185</v>
       </c>
-      <c r="B422"/>
-      <c r="C422">
-        <v>7.0244489999999995E-3</v>
-      </c>
-      <c r="D422" t="s">
-        <v>13</v>
-      </c>
-      <c r="E422" t="s">
+      <c r="B441"/>
+      <c r="C441">
+        <v>7.1053982999999977E-4</v>
+      </c>
+      <c r="D441" t="s">
+        <v>13</v>
+      </c>
+      <c r="E441" t="s">
         <v>109</v>
       </c>
-      <c r="F422" t="s">
+      <c r="F441" t="s">
         <v>184</v>
       </c>
-      <c r="H422" t="s">
+      <c r="H441" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="423" spans="1:9">
-      <c r="A423" t="s">
-        <v>272</v>
-      </c>
-      <c r="B423"/>
-      <c r="C423">
+    <row r="442" spans="1:8">
+      <c r="A442" t="s">
+        <v>264</v>
+      </c>
+      <c r="B442"/>
+      <c r="C442">
         <v>5.1560000000000002E-2</v>
       </c>
-      <c r="D423" t="s">
-        <v>13</v>
-      </c>
-      <c r="E423" t="s">
+      <c r="D442" t="s">
+        <v>13</v>
+      </c>
+      <c r="E442" t="s">
         <v>109</v>
       </c>
-      <c r="F423" t="s">
+      <c r="F442" t="s">
         <v>25</v>
       </c>
-      <c r="H423" t="s">
+      <c r="H442" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="424" spans="1:9">
-      <c r="A424" t="s">
+    <row r="443" spans="1:8">
+      <c r="A443" t="s">
         <v>125</v>
       </c>
-      <c r="B424"/>
-      <c r="C424">
+      <c r="B443"/>
+      <c r="C443">
         <v>6.5989999999999998E-6</v>
       </c>
-      <c r="D424" t="s">
-        <v>13</v>
-      </c>
-      <c r="E424" t="s">
+      <c r="D443" t="s">
+        <v>13</v>
+      </c>
+      <c r="E443" t="s">
         <v>109</v>
       </c>
-      <c r="F424" t="s">
-        <v>273</v>
-      </c>
-      <c r="H424" t="s">
+      <c r="F443" t="s">
+        <v>265</v>
+      </c>
+      <c r="H443" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="425" spans="1:9" s="57" customFormat="1">
-      <c r="B425" s="58"/>
-      <c r="I425" s="59"/>
-    </row>
-    <row r="426" spans="1:9" ht="15.6">
-      <c r="A426" s="30"/>
-      <c r="B426" s="30"/>
-    </row>
-    <row r="427" spans="1:9">
-      <c r="B427"/>
-    </row>
-    <row r="428" spans="1:9">
-      <c r="B428"/>
-    </row>
-    <row r="429" spans="1:9">
-      <c r="B429"/>
-    </row>
-    <row r="430" spans="1:9">
-      <c r="B430"/>
-    </row>
-    <row r="431" spans="1:9">
-      <c r="B431"/>
-    </row>
-    <row r="432" spans="1:9">
-      <c r="B432"/>
-    </row>
-    <row r="433" spans="1:8">
-      <c r="B433" s="36"/>
-    </row>
-    <row r="434" spans="1:8" ht="15.6">
-      <c r="A434" s="30"/>
-      <c r="B434"/>
-    </row>
-    <row r="435" spans="1:8" ht="15.6">
-      <c r="A435" s="30"/>
-      <c r="B435" s="30"/>
-      <c r="C435" s="30"/>
-      <c r="D435" s="30"/>
-      <c r="E435" s="30"/>
-      <c r="F435" s="30"/>
-      <c r="G435" s="30"/>
-      <c r="H435" s="30"/>
-    </row>
-    <row r="436" spans="1:8">
-      <c r="B436"/>
+    <row r="444" spans="1:8">
+      <c r="A444" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B444" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="C444" s="60">
+        <v>0</v>
+      </c>
+      <c r="D444" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E444" t="s">
+        <v>211</v>
+      </c>
+      <c r="G444" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H444" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="445" spans="1:8">
+      <c r="A445" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B445" s="50" t="s">
+        <v>277</v>
+      </c>
+      <c r="C445">
+        <v>0</v>
+      </c>
+      <c r="D445" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E445" t="s">
+        <v>211</v>
+      </c>
+      <c r="G445" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H445" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="446" spans="1:8">
+      <c r="A446" s="50" t="s">
+        <v>278</v>
+      </c>
+      <c r="B446" s="50" t="s">
+        <v>279</v>
+      </c>
+      <c r="C446">
+        <v>0</v>
+      </c>
+      <c r="D446" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E446" t="s">
+        <v>211</v>
+      </c>
+      <c r="G446" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H446" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="447" spans="1:8">
+      <c r="A447" t="s">
+        <v>280</v>
+      </c>
+      <c r="B447" t="s">
+        <v>281</v>
+      </c>
+      <c r="C447">
+        <v>0</v>
+      </c>
+      <c r="D447" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E447" t="s">
+        <v>211</v>
+      </c>
+      <c r="G447" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H447" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="448" spans="1:8">
+      <c r="A448" s="50" t="s">
+        <v>282</v>
+      </c>
+      <c r="B448" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="C448">
+        <v>0</v>
+      </c>
+      <c r="D448" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E448" t="s">
+        <v>211</v>
+      </c>
+      <c r="G448" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H448" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="449" spans="1:9">
+      <c r="A449" s="50" t="s">
+        <v>284</v>
+      </c>
+      <c r="B449" s="51" t="s">
+        <v>285</v>
+      </c>
+      <c r="C449">
+        <v>0</v>
+      </c>
+      <c r="D449" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E449" t="s">
+        <v>211</v>
+      </c>
+      <c r="G449" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H449" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="450" spans="1:9">
+      <c r="A450" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B450" s="51"/>
+      <c r="C450">
+        <v>1.3341247958861444E-2</v>
+      </c>
+      <c r="D450" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E450" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F450" t="s">
+        <v>184</v>
+      </c>
+      <c r="H450" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="451" spans="1:9">
+      <c r="A451" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B451" s="50"/>
+      <c r="C451">
+        <v>0.35068423206150079</v>
+      </c>
+      <c r="D451" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E451" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F451" t="s">
+        <v>184</v>
+      </c>
+      <c r="H451" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="452" spans="1:9" s="56" customFormat="1">
+      <c r="B452" s="57"/>
+      <c r="I452" s="58"/>
+    </row>
+    <row r="453" spans="1:9">
+      <c r="A453" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B453" s="43" t="s">
+        <v>288</v>
+      </c>
+      <c r="I453"/>
+    </row>
+    <row r="454" spans="1:9">
+      <c r="A454" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B454" s="59"/>
+      <c r="I454"/>
+    </row>
+    <row r="455" spans="1:9">
+      <c r="A455" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B455" t="s">
+        <v>29</v>
+      </c>
+      <c r="I455"/>
+    </row>
+    <row r="456" spans="1:9">
+      <c r="A456" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B456" s="47">
+        <v>1</v>
+      </c>
+      <c r="I456"/>
+    </row>
+    <row r="457" spans="1:9">
+      <c r="A457" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B457" t="s">
+        <v>261</v>
+      </c>
+      <c r="I457"/>
+    </row>
+    <row r="458" spans="1:9">
+      <c r="A458" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B458" t="s">
+        <v>128</v>
+      </c>
+      <c r="I458"/>
+    </row>
+    <row r="459" spans="1:9">
+      <c r="A459" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B459"/>
+      <c r="I459"/>
+    </row>
+    <row r="460" spans="1:9" ht="15.6">
+      <c r="A460" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B460"/>
+      <c r="I460"/>
+    </row>
+    <row r="461" spans="1:9" s="46" customFormat="1">
+      <c r="A461" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B461" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C461" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D461" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E461" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F461" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G461" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H461" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="I461" s="46" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="462" spans="1:9">
+      <c r="A462" t="s">
+        <v>288</v>
+      </c>
+      <c r="B462" t="s">
+        <v>261</v>
+      </c>
+      <c r="C462">
+        <v>1</v>
+      </c>
+      <c r="D462" t="s">
+        <v>128</v>
+      </c>
+      <c r="E462" s="50"/>
+      <c r="G462" t="s">
+        <v>29</v>
+      </c>
+      <c r="H462" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="463" spans="1:9">
+      <c r="A463" t="s">
+        <v>266</v>
+      </c>
+      <c r="B463" t="s">
+        <v>267</v>
+      </c>
+      <c r="C463">
+        <v>1.0255532373423097E-2</v>
+      </c>
+      <c r="D463" t="s">
+        <v>13</v>
+      </c>
+      <c r="E463" t="s">
+        <v>211</v>
+      </c>
+      <c r="G463" t="s">
+        <v>140</v>
+      </c>
+      <c r="H463" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="464" spans="1:9">
+      <c r="A464" t="s">
+        <v>268</v>
+      </c>
+      <c r="B464" t="s">
+        <v>135</v>
+      </c>
+      <c r="C464">
+        <v>5.4000000000000001E-11</v>
+      </c>
+      <c r="D464" t="s">
+        <v>6</v>
+      </c>
+      <c r="E464" t="s">
+        <v>211</v>
+      </c>
+      <c r="G464" t="s">
+        <v>140</v>
+      </c>
+      <c r="H464" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="465" spans="1:8">
+      <c r="A465" t="s">
+        <v>28</v>
+      </c>
+      <c r="B465" t="s">
+        <v>20</v>
+      </c>
+      <c r="C465">
+        <v>0.63128239335113012</v>
+      </c>
+      <c r="D465" t="s">
+        <v>19</v>
+      </c>
+      <c r="E465" t="s">
+        <v>211</v>
+      </c>
+      <c r="G465" t="s">
+        <v>27</v>
+      </c>
+      <c r="H465" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="466" spans="1:8">
+      <c r="A466" t="s">
+        <v>180</v>
+      </c>
+      <c r="B466" t="s">
+        <v>181</v>
+      </c>
+      <c r="C466">
+        <v>1.1400000000000001E-4</v>
+      </c>
+      <c r="D466" t="s">
+        <v>13</v>
+      </c>
+      <c r="E466" t="s">
+        <v>211</v>
+      </c>
+      <c r="G466" t="s">
+        <v>49</v>
+      </c>
+      <c r="H466" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="467" spans="1:8">
+      <c r="A467" t="s">
+        <v>269</v>
+      </c>
+      <c r="B467" t="s">
+        <v>270</v>
+      </c>
+      <c r="C467">
+        <v>1.01E-4</v>
+      </c>
+      <c r="D467" t="s">
+        <v>13</v>
+      </c>
+      <c r="E467" t="s">
+        <v>211</v>
+      </c>
+      <c r="G467" t="s">
+        <v>140</v>
+      </c>
+      <c r="H467" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="468" spans="1:8">
+      <c r="A468" t="s">
+        <v>271</v>
+      </c>
+      <c r="B468" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C468">
+        <v>1.9028346445037665</v>
+      </c>
+      <c r="D468" s="45" t="s">
+        <v>128</v>
+      </c>
+      <c r="G468" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="H468" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="469" spans="1:8">
+      <c r="A469" t="s">
+        <v>218</v>
+      </c>
+      <c r="B469"/>
+      <c r="C469">
+        <v>1.7694051155218009</v>
+      </c>
+      <c r="D469" t="s">
+        <v>13</v>
+      </c>
+      <c r="E469" t="s">
+        <v>109</v>
+      </c>
+      <c r="F469" t="s">
+        <v>184</v>
+      </c>
+      <c r="H469" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="470" spans="1:8">
+      <c r="A470" t="s">
+        <v>262</v>
+      </c>
+      <c r="B470"/>
+      <c r="C470">
+        <v>1.28</v>
+      </c>
+      <c r="D470" t="s">
+        <v>46</v>
+      </c>
+      <c r="E470" t="s">
+        <v>109</v>
+      </c>
+      <c r="F470" t="s">
+        <v>184</v>
+      </c>
+      <c r="H470" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="471" spans="1:8">
+      <c r="A471" t="s">
+        <v>263</v>
+      </c>
+      <c r="B471"/>
+      <c r="C471">
+        <v>0</v>
+      </c>
+      <c r="D471" t="s">
+        <v>13</v>
+      </c>
+      <c r="E471" t="s">
+        <v>109</v>
+      </c>
+      <c r="F471" t="s">
+        <v>184</v>
+      </c>
+      <c r="H471" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="472" spans="1:8">
+      <c r="A472" t="s">
+        <v>185</v>
+      </c>
+      <c r="B472"/>
+      <c r="C472">
+        <v>1.4187996E-2</v>
+      </c>
+      <c r="D472" t="s">
+        <v>13</v>
+      </c>
+      <c r="E472" t="s">
+        <v>109</v>
+      </c>
+      <c r="F472" t="s">
+        <v>184</v>
+      </c>
+      <c r="H472" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="473" spans="1:8">
+      <c r="A473" t="s">
+        <v>264</v>
+      </c>
+      <c r="B473"/>
+      <c r="C473">
+        <v>5.1560000000000002E-2</v>
+      </c>
+      <c r="D473" t="s">
+        <v>13</v>
+      </c>
+      <c r="E473" t="s">
+        <v>109</v>
+      </c>
+      <c r="F473" t="s">
+        <v>25</v>
+      </c>
+      <c r="H473" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="474" spans="1:8">
+      <c r="A474" t="s">
+        <v>125</v>
+      </c>
+      <c r="B474"/>
+      <c r="C474">
+        <v>6.5989999999999998E-6</v>
+      </c>
+      <c r="D474" t="s">
+        <v>13</v>
+      </c>
+      <c r="E474" t="s">
+        <v>109</v>
+      </c>
+      <c r="F474" t="s">
+        <v>265</v>
+      </c>
+      <c r="H474" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="475" spans="1:8">
+      <c r="A475" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B475" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="C475" s="60">
+        <v>0.19028346445037667</v>
+      </c>
+      <c r="D475" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E475" t="s">
+        <v>211</v>
+      </c>
+      <c r="G475" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H475" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="476" spans="1:8">
+      <c r="A476" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B476" s="50" t="s">
+        <v>277</v>
+      </c>
+      <c r="C476">
+        <v>0</v>
+      </c>
+      <c r="D476" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E476" t="s">
+        <v>211</v>
+      </c>
+      <c r="G476" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H476" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="477" spans="1:8">
+      <c r="A477" s="50" t="s">
+        <v>278</v>
+      </c>
+      <c r="B477" s="50" t="s">
+        <v>279</v>
+      </c>
+      <c r="C477">
+        <v>0</v>
+      </c>
+      <c r="D477" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E477" t="s">
+        <v>211</v>
+      </c>
+      <c r="G477" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H477" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="478" spans="1:8">
+      <c r="A478" t="s">
+        <v>280</v>
+      </c>
+      <c r="B478" t="s">
+        <v>281</v>
+      </c>
+      <c r="C478">
+        <v>0</v>
+      </c>
+      <c r="D478" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E478" t="s">
+        <v>211</v>
+      </c>
+      <c r="G478" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H478" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="479" spans="1:8">
+      <c r="A479" s="50" t="s">
+        <v>282</v>
+      </c>
+      <c r="B479" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="C479">
+        <v>0</v>
+      </c>
+      <c r="D479" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E479" t="s">
+        <v>211</v>
+      </c>
+      <c r="G479" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H479" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="480" spans="1:8">
+      <c r="A480" s="50" t="s">
+        <v>284</v>
+      </c>
+      <c r="B480" s="51" t="s">
+        <v>285</v>
+      </c>
+      <c r="C480">
+        <v>0</v>
+      </c>
+      <c r="D480" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E480" t="s">
+        <v>211</v>
+      </c>
+      <c r="G480" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H480" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="481" spans="1:9">
+      <c r="A481" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B481" s="51"/>
+      <c r="C481">
+        <v>0</v>
+      </c>
+      <c r="D481" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E481" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F481" t="s">
+        <v>184</v>
+      </c>
+      <c r="H481" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="482" spans="1:9">
+      <c r="A482" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B482" s="50"/>
+      <c r="C482">
+        <v>0</v>
+      </c>
+      <c r="D482" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E482" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F482" t="s">
+        <v>184</v>
+      </c>
+      <c r="H482" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="483" spans="1:9" s="56" customFormat="1">
+      <c r="B483" s="57"/>
+      <c r="I483" s="58"/>
+    </row>
+    <row r="484" spans="1:9">
+      <c r="A484" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B484" s="43" t="s">
+        <v>289</v>
+      </c>
+      <c r="I484"/>
+    </row>
+    <row r="485" spans="1:9">
+      <c r="A485" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B485" s="59"/>
+      <c r="I485"/>
+    </row>
+    <row r="486" spans="1:9">
+      <c r="A486" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B486" t="s">
+        <v>29</v>
+      </c>
+      <c r="I486"/>
+    </row>
+    <row r="487" spans="1:9">
+      <c r="A487" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B487" s="47">
+        <v>1</v>
+      </c>
+      <c r="I487"/>
+    </row>
+    <row r="488" spans="1:9">
+      <c r="A488" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B488" t="s">
+        <v>261</v>
+      </c>
+      <c r="I488"/>
+    </row>
+    <row r="489" spans="1:9">
+      <c r="A489" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B489" t="s">
+        <v>128</v>
+      </c>
+      <c r="I489"/>
+    </row>
+    <row r="490" spans="1:9">
+      <c r="A490" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B490"/>
+      <c r="I490"/>
+    </row>
+    <row r="491" spans="1:9" ht="15.6">
+      <c r="A491" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B491"/>
+      <c r="I491"/>
+    </row>
+    <row r="492" spans="1:9" s="46" customFormat="1">
+      <c r="A492" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B492" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C492" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D492" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E492" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F492" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G492" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H492" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="I492" s="46" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="493" spans="1:9">
+      <c r="A493" t="s">
+        <v>289</v>
+      </c>
+      <c r="B493" t="s">
+        <v>261</v>
+      </c>
+      <c r="C493">
+        <v>1</v>
+      </c>
+      <c r="D493" t="s">
+        <v>128</v>
+      </c>
+      <c r="E493" s="50"/>
+      <c r="G493" t="s">
+        <v>29</v>
+      </c>
+      <c r="H493" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="494" spans="1:9">
+      <c r="A494" t="s">
+        <v>266</v>
+      </c>
+      <c r="B494" t="s">
+        <v>267</v>
+      </c>
+      <c r="C494">
+        <v>1.0255532373423097E-2</v>
+      </c>
+      <c r="D494" t="s">
+        <v>13</v>
+      </c>
+      <c r="E494" t="s">
+        <v>211</v>
+      </c>
+      <c r="G494" t="s">
+        <v>140</v>
+      </c>
+      <c r="H494" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="495" spans="1:9">
+      <c r="A495" t="s">
+        <v>268</v>
+      </c>
+      <c r="B495" t="s">
+        <v>135</v>
+      </c>
+      <c r="C495">
+        <v>5.4000000000000001E-11</v>
+      </c>
+      <c r="D495" t="s">
+        <v>6</v>
+      </c>
+      <c r="E495" t="s">
+        <v>211</v>
+      </c>
+      <c r="G495" t="s">
+        <v>140</v>
+      </c>
+      <c r="H495" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="496" spans="1:9">
+      <c r="A496" t="s">
+        <v>28</v>
+      </c>
+      <c r="B496" t="s">
+        <v>20</v>
+      </c>
+      <c r="C496">
+        <v>0.67375221360986193</v>
+      </c>
+      <c r="D496" t="s">
+        <v>19</v>
+      </c>
+      <c r="E496" t="s">
+        <v>211</v>
+      </c>
+      <c r="G496" t="s">
+        <v>27</v>
+      </c>
+      <c r="H496" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8">
+      <c r="A497" t="s">
+        <v>180</v>
+      </c>
+      <c r="B497" t="s">
+        <v>181</v>
+      </c>
+      <c r="C497">
+        <v>1.1400000000000001E-4</v>
+      </c>
+      <c r="D497" t="s">
+        <v>13</v>
+      </c>
+      <c r="E497" t="s">
+        <v>211</v>
+      </c>
+      <c r="G497" t="s">
+        <v>49</v>
+      </c>
+      <c r="H497" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8">
+      <c r="A498" t="s">
+        <v>269</v>
+      </c>
+      <c r="B498" t="s">
+        <v>270</v>
+      </c>
+      <c r="C498">
+        <v>1.01E-4</v>
+      </c>
+      <c r="D498" t="s">
+        <v>13</v>
+      </c>
+      <c r="E498" t="s">
+        <v>211</v>
+      </c>
+      <c r="G498" t="s">
+        <v>140</v>
+      </c>
+      <c r="H498" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8">
+      <c r="A499" t="s">
+        <v>271</v>
+      </c>
+      <c r="B499" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C499">
+        <v>1.9016807120328729</v>
+      </c>
+      <c r="D499" s="45" t="s">
+        <v>128</v>
+      </c>
+      <c r="G499" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="H499" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8">
+      <c r="A500" t="s">
+        <v>218</v>
+      </c>
+      <c r="B500"/>
+      <c r="C500">
+        <v>1.7501018706524611</v>
+      </c>
+      <c r="D500" t="s">
+        <v>13</v>
+      </c>
+      <c r="E500" t="s">
+        <v>109</v>
+      </c>
+      <c r="F500" t="s">
+        <v>184</v>
+      </c>
+      <c r="H500" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8">
+      <c r="A501" t="s">
+        <v>262</v>
+      </c>
+      <c r="B501"/>
+      <c r="C501">
+        <v>1.28</v>
+      </c>
+      <c r="D501" t="s">
+        <v>46</v>
+      </c>
+      <c r="E501" t="s">
+        <v>109</v>
+      </c>
+      <c r="F501" t="s">
+        <v>184</v>
+      </c>
+      <c r="H501" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="502" spans="1:8">
+      <c r="A502" t="s">
+        <v>263</v>
+      </c>
+      <c r="B502"/>
+      <c r="C502">
+        <v>0</v>
+      </c>
+      <c r="D502" t="s">
+        <v>13</v>
+      </c>
+      <c r="E502" t="s">
+        <v>109</v>
+      </c>
+      <c r="F502" t="s">
+        <v>184</v>
+      </c>
+      <c r="H502" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="503" spans="1:8">
+      <c r="A503" t="s">
+        <v>185</v>
+      </c>
+      <c r="B503"/>
+      <c r="C503">
+        <v>2.1269087999999998E-2</v>
+      </c>
+      <c r="D503" t="s">
+        <v>13</v>
+      </c>
+      <c r="E503" t="s">
+        <v>109</v>
+      </c>
+      <c r="F503" t="s">
+        <v>184</v>
+      </c>
+      <c r="H503" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="504" spans="1:8">
+      <c r="A504" t="s">
+        <v>264</v>
+      </c>
+      <c r="B504"/>
+      <c r="C504">
+        <v>5.1560000000000002E-2</v>
+      </c>
+      <c r="D504" t="s">
+        <v>13</v>
+      </c>
+      <c r="E504" t="s">
+        <v>109</v>
+      </c>
+      <c r="F504" t="s">
+        <v>25</v>
+      </c>
+      <c r="H504" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="505" spans="1:8">
+      <c r="A505" t="s">
+        <v>125</v>
+      </c>
+      <c r="B505"/>
+      <c r="C505">
+        <v>6.5989999999999998E-6</v>
+      </c>
+      <c r="D505" t="s">
+        <v>13</v>
+      </c>
+      <c r="E505" t="s">
+        <v>109</v>
+      </c>
+      <c r="F505" t="s">
+        <v>265</v>
+      </c>
+      <c r="H505" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="506" spans="1:8">
+      <c r="A506" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B506" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="C506" s="61">
+        <v>0</v>
+      </c>
+      <c r="D506" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E506" t="s">
+        <v>211</v>
+      </c>
+      <c r="G506" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H506" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="507" spans="1:8">
+      <c r="A507" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B507" s="50" t="s">
+        <v>277</v>
+      </c>
+      <c r="C507">
+        <v>0</v>
+      </c>
+      <c r="D507" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E507" t="s">
+        <v>211</v>
+      </c>
+      <c r="G507" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H507" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="508" spans="1:8">
+      <c r="A508" s="50" t="s">
+        <v>278</v>
+      </c>
+      <c r="B508" s="50" t="s">
+        <v>279</v>
+      </c>
+      <c r="C508">
+        <v>0</v>
+      </c>
+      <c r="D508" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E508" t="s">
+        <v>211</v>
+      </c>
+      <c r="G508" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H508" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="509" spans="1:8">
+      <c r="A509" t="s">
+        <v>280</v>
+      </c>
+      <c r="B509" t="s">
+        <v>281</v>
+      </c>
+      <c r="C509">
+        <v>0</v>
+      </c>
+      <c r="D509" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E509" t="s">
+        <v>211</v>
+      </c>
+      <c r="G509" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H509" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="510" spans="1:8">
+      <c r="A510" s="50" t="s">
+        <v>282</v>
+      </c>
+      <c r="B510" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="C510">
+        <v>0</v>
+      </c>
+      <c r="D510" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E510" t="s">
+        <v>211</v>
+      </c>
+      <c r="G510" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H510" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="511" spans="1:8">
+      <c r="A511" s="50" t="s">
+        <v>284</v>
+      </c>
+      <c r="B511" s="51" t="s">
+        <v>285</v>
+      </c>
+      <c r="C511">
+        <v>0</v>
+      </c>
+      <c r="D511" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E511" t="s">
+        <v>211</v>
+      </c>
+      <c r="G511" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H511" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="512" spans="1:8">
+      <c r="A512" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B512" s="51"/>
+      <c r="C512">
+        <v>0</v>
+      </c>
+      <c r="D512" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E512" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F512" t="s">
+        <v>184</v>
+      </c>
+      <c r="H512" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="513" spans="1:8">
+      <c r="A513" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B513" s="50"/>
+      <c r="C513">
+        <v>0</v>
+      </c>
+      <c r="D513" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E513" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F513" t="s">
+        <v>184</v>
+      </c>
+      <c r="H513" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added cryogenic separation simplified LCI
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="242" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C3EF791-C10F-491E-BB03-3273FECC7A9E}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B80BF9B0-457C-49AA-B771-15865184CE48}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2245" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2382" uniqueCount="291">
   <si>
     <t>Database</t>
   </si>
@@ -913,6 +913,9 @@
   </si>
   <si>
     <t>biogas purification to biomethane by PSA, Tr2050</t>
+  </si>
+  <si>
+    <t>biogas purification to biomethane by cryogenic separation, Tr2050</t>
   </si>
 </sst>
 </file>
@@ -1475,7 +1478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH513"/>
+  <dimension ref="A1:AH544"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="55.44140625" customWidth="1"/>
@@ -15160,7 +15163,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="513" spans="1:8">
+    <row r="513" spans="1:9">
       <c r="A513" s="15" t="s">
         <v>108</v>
       </c>
@@ -15178,6 +15181,574 @@
         <v>184</v>
       </c>
       <c r="H513" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="514" spans="1:9">
+      <c r="A514" s="56"/>
+      <c r="B514" s="57"/>
+      <c r="C514" s="56"/>
+      <c r="D514" s="56"/>
+      <c r="E514" s="56"/>
+      <c r="F514" s="56"/>
+      <c r="G514" s="56"/>
+      <c r="H514" s="56"/>
+      <c r="I514" s="58"/>
+    </row>
+    <row r="515" spans="1:9">
+      <c r="A515" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B515" s="43" t="s">
+        <v>290</v>
+      </c>
+      <c r="I515"/>
+    </row>
+    <row r="516" spans="1:9">
+      <c r="A516" s="46" t="s">
+        <v>11</v>
+      </c>
+      <c r="B516" s="59"/>
+      <c r="I516"/>
+    </row>
+    <row r="517" spans="1:9">
+      <c r="A517" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B517" t="s">
+        <v>29</v>
+      </c>
+      <c r="I517"/>
+    </row>
+    <row r="518" spans="1:9">
+      <c r="A518" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B518" s="47">
+        <v>1</v>
+      </c>
+      <c r="I518"/>
+    </row>
+    <row r="519" spans="1:9">
+      <c r="A519" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B519" t="s">
+        <v>261</v>
+      </c>
+      <c r="I519"/>
+    </row>
+    <row r="520" spans="1:9">
+      <c r="A520" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="B520" t="s">
+        <v>128</v>
+      </c>
+      <c r="I520"/>
+    </row>
+    <row r="521" spans="1:9">
+      <c r="A521" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B521"/>
+      <c r="I521"/>
+    </row>
+    <row r="522" spans="1:9" ht="15.6">
+      <c r="A522" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B522"/>
+      <c r="I522"/>
+    </row>
+    <row r="523" spans="1:9">
+      <c r="A523" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="B523" s="46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C523" s="46" t="s">
+        <v>9</v>
+      </c>
+      <c r="D523" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="E523" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F523" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G523" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H523" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="I523" s="46" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="524" spans="1:9">
+      <c r="A524" t="s">
+        <v>290</v>
+      </c>
+      <c r="B524" t="s">
+        <v>261</v>
+      </c>
+      <c r="C524">
+        <v>1</v>
+      </c>
+      <c r="D524" t="s">
+        <v>128</v>
+      </c>
+      <c r="E524" s="50"/>
+      <c r="G524" t="s">
+        <v>29</v>
+      </c>
+      <c r="H524" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="525" spans="1:9">
+      <c r="A525" t="s">
+        <v>266</v>
+      </c>
+      <c r="B525" t="s">
+        <v>267</v>
+      </c>
+      <c r="C525">
+        <v>0.14950127537864799</v>
+      </c>
+      <c r="D525" t="s">
+        <v>13</v>
+      </c>
+      <c r="E525" t="s">
+        <v>211</v>
+      </c>
+      <c r="G525" t="s">
+        <v>140</v>
+      </c>
+      <c r="H525" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="526" spans="1:9">
+      <c r="A526" t="s">
+        <v>268</v>
+      </c>
+      <c r="B526" t="s">
+        <v>135</v>
+      </c>
+      <c r="C526">
+        <v>0</v>
+      </c>
+      <c r="D526" t="s">
+        <v>6</v>
+      </c>
+      <c r="E526" t="s">
+        <v>211</v>
+      </c>
+      <c r="G526" t="s">
+        <v>140</v>
+      </c>
+      <c r="H526" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="527" spans="1:9">
+      <c r="A527" t="s">
+        <v>28</v>
+      </c>
+      <c r="B527" t="s">
+        <v>20</v>
+      </c>
+      <c r="C527">
+        <v>0.65406807978158488</v>
+      </c>
+      <c r="D527" t="s">
+        <v>19</v>
+      </c>
+      <c r="E527" t="s">
+        <v>211</v>
+      </c>
+      <c r="G527" t="s">
+        <v>27</v>
+      </c>
+      <c r="H527" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="528" spans="1:9">
+      <c r="A528" t="s">
+        <v>180</v>
+      </c>
+      <c r="B528" t="s">
+        <v>181</v>
+      </c>
+      <c r="C528">
+        <v>0</v>
+      </c>
+      <c r="D528" t="s">
+        <v>13</v>
+      </c>
+      <c r="E528" t="s">
+        <v>211</v>
+      </c>
+      <c r="G528" t="s">
+        <v>49</v>
+      </c>
+      <c r="H528" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="529" spans="1:8">
+      <c r="A529" t="s">
+        <v>269</v>
+      </c>
+      <c r="B529" t="s">
+        <v>270</v>
+      </c>
+      <c r="C529">
+        <v>0</v>
+      </c>
+      <c r="D529" t="s">
+        <v>13</v>
+      </c>
+      <c r="E529" t="s">
+        <v>211</v>
+      </c>
+      <c r="G529" t="s">
+        <v>140</v>
+      </c>
+      <c r="H529" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="530" spans="1:8">
+      <c r="A530" t="s">
+        <v>271</v>
+      </c>
+      <c r="B530" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="C530">
+        <v>1.8687659422330998</v>
+      </c>
+      <c r="D530" s="45" t="s">
+        <v>128</v>
+      </c>
+      <c r="G530" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="H530" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="531" spans="1:8">
+      <c r="A531" t="s">
+        <v>218</v>
+      </c>
+      <c r="B531"/>
+      <c r="C531">
+        <v>1.7398751234684424</v>
+      </c>
+      <c r="D531" t="s">
+        <v>13</v>
+      </c>
+      <c r="E531" t="s">
+        <v>109</v>
+      </c>
+      <c r="F531" t="s">
+        <v>184</v>
+      </c>
+      <c r="H531" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="532" spans="1:8">
+      <c r="A532" t="s">
+        <v>262</v>
+      </c>
+      <c r="B532"/>
+      <c r="C532">
+        <v>0</v>
+      </c>
+      <c r="D532" t="s">
+        <v>46</v>
+      </c>
+      <c r="E532" t="s">
+        <v>109</v>
+      </c>
+      <c r="F532" t="s">
+        <v>184</v>
+      </c>
+      <c r="H532" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="533" spans="1:8">
+      <c r="A533" t="s">
+        <v>263</v>
+      </c>
+      <c r="B533"/>
+      <c r="C533">
+        <v>0</v>
+      </c>
+      <c r="D533" t="s">
+        <v>13</v>
+      </c>
+      <c r="E533" t="s">
+        <v>109</v>
+      </c>
+      <c r="F533" t="s">
+        <v>184</v>
+      </c>
+      <c r="H533" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="534" spans="1:8">
+      <c r="A534" t="s">
+        <v>185</v>
+      </c>
+      <c r="B534"/>
+      <c r="C534">
+        <v>3.4834928759999994E-4</v>
+      </c>
+      <c r="D534" t="s">
+        <v>13</v>
+      </c>
+      <c r="E534" t="s">
+        <v>109</v>
+      </c>
+      <c r="F534" t="s">
+        <v>184</v>
+      </c>
+      <c r="H534" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="535" spans="1:8">
+      <c r="A535" t="s">
+        <v>264</v>
+      </c>
+      <c r="B535"/>
+      <c r="C535">
+        <v>0</v>
+      </c>
+      <c r="D535" t="s">
+        <v>13</v>
+      </c>
+      <c r="E535" t="s">
+        <v>109</v>
+      </c>
+      <c r="F535" t="s">
+        <v>25</v>
+      </c>
+      <c r="H535" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="536" spans="1:8">
+      <c r="A536" t="s">
+        <v>125</v>
+      </c>
+      <c r="B536"/>
+      <c r="C536">
+        <v>0</v>
+      </c>
+      <c r="D536" t="s">
+        <v>13</v>
+      </c>
+      <c r="E536" t="s">
+        <v>109</v>
+      </c>
+      <c r="F536" t="s">
+        <v>265</v>
+      </c>
+      <c r="H536" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="537" spans="1:8">
+      <c r="A537" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="B537" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="C537" s="61">
+        <v>0</v>
+      </c>
+      <c r="D537" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E537" t="s">
+        <v>211</v>
+      </c>
+      <c r="G537" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="H537" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="538" spans="1:8">
+      <c r="A538" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="B538" s="50" t="s">
+        <v>277</v>
+      </c>
+      <c r="C538">
+        <v>0</v>
+      </c>
+      <c r="D538" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E538" t="s">
+        <v>211</v>
+      </c>
+      <c r="G538" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H538" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="539" spans="1:8">
+      <c r="A539" s="50" t="s">
+        <v>278</v>
+      </c>
+      <c r="B539" s="50" t="s">
+        <v>279</v>
+      </c>
+      <c r="C539">
+        <v>0</v>
+      </c>
+      <c r="D539" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E539" t="s">
+        <v>211</v>
+      </c>
+      <c r="G539" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H539" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="540" spans="1:8">
+      <c r="A540" t="s">
+        <v>280</v>
+      </c>
+      <c r="B540" t="s">
+        <v>281</v>
+      </c>
+      <c r="C540">
+        <v>0</v>
+      </c>
+      <c r="D540" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E540" t="s">
+        <v>211</v>
+      </c>
+      <c r="G540" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H540" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="541" spans="1:8">
+      <c r="A541" s="50" t="s">
+        <v>282</v>
+      </c>
+      <c r="B541" s="51" t="s">
+        <v>283</v>
+      </c>
+      <c r="C541">
+        <v>0</v>
+      </c>
+      <c r="D541" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E541" t="s">
+        <v>211</v>
+      </c>
+      <c r="G541" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H541" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="542" spans="1:8">
+      <c r="A542" s="50" t="s">
+        <v>284</v>
+      </c>
+      <c r="B542" s="51" t="s">
+        <v>285</v>
+      </c>
+      <c r="C542">
+        <v>0</v>
+      </c>
+      <c r="D542" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E542" t="s">
+        <v>211</v>
+      </c>
+      <c r="G542" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="H542" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="543" spans="1:8">
+      <c r="A543" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B543" s="51"/>
+      <c r="C543">
+        <v>0</v>
+      </c>
+      <c r="D543" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E543" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F543" t="s">
+        <v>184</v>
+      </c>
+      <c r="H543" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="544" spans="1:8">
+      <c r="A544" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B544" s="50"/>
+      <c r="C544">
+        <v>0</v>
+      </c>
+      <c r="D544" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E544" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F544" t="s">
+        <v>184</v>
+      </c>
+      <c r="H544" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
change elec from CH to elec from FR
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\ADEME_scenarios_premise_gas\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="511" documentId="13_ncr:1_{1521C391-BCF6-4923-B754-ECBD64DA2349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A179A91-8BC3-4719-BFAE-9B973199E214}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -1491,7 +1491,7 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
+    <cellStyle name="Neutre" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 11 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -1508,10 +1508,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1778,17 +1774,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH656"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="73.109375" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="99.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="73.08984375" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="17.08984375" customWidth="1"/>
+    <col min="4" max="4" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.36328125" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="99.08984375" style="3" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1840,7 +1836,7 @@
       <c r="I4" s="11"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5" spans="1:14" ht="15.6">
+    <row r="5" spans="1:14" ht="15.5">
       <c r="A5" s="30" t="s">
         <v>1</v>
       </c>
@@ -1930,7 +1926,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.6">
+    <row r="13" spans="1:14" ht="15.5">
       <c r="A13" s="30" t="s">
         <v>7</v>
       </c>
@@ -1940,7 +1936,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15.6">
+    <row r="14" spans="1:14" ht="15.5">
       <c r="A14" s="30" t="s">
         <v>8</v>
       </c>
@@ -2603,7 +2599,7 @@
       <c r="B49"/>
       <c r="I49"/>
     </row>
-    <row r="50" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="50" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A50" s="4" t="s">
         <v>1</v>
       </c>
@@ -2623,7 +2619,7 @@
       <c r="O50" s="26"/>
       <c r="P50" s="26"/>
     </row>
-    <row r="51" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="51" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A51" s="4" t="s">
         <v>3</v>
       </c>
@@ -2643,7 +2639,7 @@
       <c r="O51" s="26"/>
       <c r="P51" s="26"/>
     </row>
-    <row r="52" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="52" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A52" s="4" t="s">
         <v>11</v>
       </c>
@@ -2663,7 +2659,7 @@
       <c r="O52" s="26"/>
       <c r="P52" s="26"/>
     </row>
-    <row r="53" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="53" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A53" s="4" t="s">
         <v>4</v>
       </c>
@@ -2683,7 +2679,7 @@
       <c r="O53" s="26"/>
       <c r="P53" s="26"/>
     </row>
-    <row r="54" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="54" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A54" s="4" t="s">
         <v>2</v>
       </c>
@@ -2703,7 +2699,7 @@
       <c r="O54" s="26"/>
       <c r="P54" s="26"/>
     </row>
-    <row r="55" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="55" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A55" s="4" t="s">
         <v>6</v>
       </c>
@@ -2725,7 +2721,7 @@
       <c r="O55" s="26"/>
       <c r="P55" s="26"/>
     </row>
-    <row r="56" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="56" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A56" s="4" t="s">
         <v>7</v>
       </c>
@@ -2745,7 +2741,7 @@
       <c r="O56" s="26"/>
       <c r="P56" s="26"/>
     </row>
-    <row r="57" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="57" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A57" s="4" t="s">
         <v>8</v>
       </c>
@@ -2783,7 +2779,7 @@
       <c r="S57" s="29"/>
       <c r="T57" s="30"/>
     </row>
-    <row r="58" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="58" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A58" t="s">
         <v>73</v>
       </c>
@@ -2815,7 +2811,7 @@
       <c r="P58" s="26"/>
       <c r="T58"/>
     </row>
-    <row r="59" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="59" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A59" t="s">
         <v>71</v>
       </c>
@@ -2849,7 +2845,7 @@
       <c r="Q59"/>
       <c r="R59"/>
     </row>
-    <row r="60" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="60" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A60" t="s">
         <v>72</v>
       </c>
@@ -2883,7 +2879,7 @@
       <c r="Q60"/>
       <c r="R60"/>
     </row>
-    <row r="61" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="61" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -2917,7 +2913,7 @@
       <c r="Q61"/>
       <c r="R61"/>
     </row>
-    <row r="62" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="62" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -2951,7 +2947,7 @@
       <c r="Q62"/>
       <c r="R62"/>
     </row>
-    <row r="63" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="63" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A63" t="s">
         <v>28</v>
       </c>
@@ -2984,7 +2980,7 @@
       <c r="Q63"/>
       <c r="R63"/>
     </row>
-    <row r="64" spans="1:20" s="25" customFormat="1" ht="15.6">
+    <row r="64" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A64" t="s">
         <v>21</v>
       </c>
@@ -3017,7 +3013,7 @@
       <c r="Q64"/>
       <c r="R64"/>
     </row>
-    <row r="65" spans="1:18" s="25" customFormat="1" ht="15.6">
+    <row r="65" spans="1:18" s="25" customFormat="1" ht="15.5">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -3046,7 +3042,7 @@
       <c r="Q65" s="32"/>
       <c r="R65"/>
     </row>
-    <row r="66" spans="1:18" s="25" customFormat="1" ht="15.6">
+    <row r="66" spans="1:18" s="25" customFormat="1" ht="15.5">
       <c r="A66" t="s">
         <v>70</v>
       </c>
@@ -3076,7 +3072,7 @@
       <c r="Q66" s="32"/>
       <c r="R66"/>
     </row>
-    <row r="67" spans="1:18" s="25" customFormat="1" ht="15">
+    <row r="67" spans="1:18" s="25" customFormat="1" ht="15.5">
       <c r="K67" s="26"/>
       <c r="L67" s="26"/>
       <c r="M67" s="26"/>
@@ -3084,7 +3080,7 @@
       <c r="O67" s="26"/>
       <c r="P67" s="26"/>
     </row>
-    <row r="70" spans="1:18" ht="15.6">
+    <row r="70" spans="1:18" ht="15.5">
       <c r="A70" s="35" t="s">
         <v>1</v>
       </c>
@@ -3174,7 +3170,7 @@
       <c r="H75" s="36"/>
       <c r="I75" s="36"/>
     </row>
-    <row r="76" spans="1:18" ht="15.6">
+    <row r="76" spans="1:18" ht="15.5">
       <c r="A76" s="35" t="s">
         <v>7</v>
       </c>
@@ -5286,7 +5282,7 @@
       <c r="H167" s="36"/>
       <c r="I167" s="36"/>
     </row>
-    <row r="168" spans="1:9" ht="15.6">
+    <row r="168" spans="1:9" ht="15.5">
       <c r="A168" s="30" t="s">
         <v>1</v>
       </c>
@@ -5348,13 +5344,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="15.6">
+    <row r="176" spans="1:9" ht="15.5">
       <c r="A176" s="30" t="s">
         <v>7</v>
       </c>
       <c r="B176"/>
     </row>
-    <row r="177" spans="1:34" ht="15.6">
+    <row r="177" spans="1:34" ht="15.5">
       <c r="A177" s="30" t="s">
         <v>8</v>
       </c>
@@ -13860,7 +13856,7 @@
       <c r="AG416" s="41"/>
       <c r="AH416" s="41"/>
     </row>
-    <row r="417" spans="1:9" ht="15.6">
+    <row r="417" spans="1:9" ht="15.5">
       <c r="A417" s="30" t="s">
         <v>1</v>
       </c>
@@ -13932,7 +13928,7 @@
       </c>
       <c r="I424"/>
     </row>
-    <row r="425" spans="1:9" ht="15.6">
+    <row r="425" spans="1:9" ht="15.5">
       <c r="A425" s="30" t="s">
         <v>7</v>
       </c>
@@ -14266,7 +14262,7 @@
         <v>211</v>
       </c>
       <c r="G438" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H438" t="s">
         <v>12</v>
@@ -15722,7 +15718,7 @@
       <c r="B501"/>
       <c r="I501"/>
     </row>
-    <row r="502" spans="1:9" ht="15.6">
+    <row r="502" spans="1:9" ht="15.5">
       <c r="A502" s="30" t="s">
         <v>7</v>
       </c>
@@ -15843,7 +15839,7 @@
         <v>211</v>
       </c>
       <c r="G507" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H507" t="s">
         <v>12</v>
@@ -16104,7 +16100,7 @@
       <c r="B524"/>
       <c r="I524"/>
     </row>
-    <row r="525" spans="1:9" ht="15.6">
+    <row r="525" spans="1:9" ht="15.5">
       <c r="A525" s="30" t="s">
         <v>7</v>
       </c>
@@ -16224,7 +16220,7 @@
         <v>211</v>
       </c>
       <c r="G530" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H530" t="s">
         <v>12</v>
@@ -16665,7 +16661,7 @@
       <c r="B555"/>
       <c r="I555"/>
     </row>
-    <row r="556" spans="1:9" ht="15.6">
+    <row r="556" spans="1:9" ht="15.5">
       <c r="A556" s="30" t="s">
         <v>7</v>
       </c>
@@ -16785,7 +16781,7 @@
         <v>211</v>
       </c>
       <c r="G561" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H561" t="s">
         <v>12</v>
@@ -17226,7 +17222,7 @@
       <c r="B586"/>
       <c r="I586"/>
     </row>
-    <row r="587" spans="1:9" ht="15.6">
+    <row r="587" spans="1:9" ht="15.5">
       <c r="A587" s="30" t="s">
         <v>7</v>
       </c>
@@ -17346,7 +17342,7 @@
         <v>211</v>
       </c>
       <c r="G592" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H592" t="s">
         <v>12</v>
@@ -17794,7 +17790,7 @@
       <c r="B617"/>
       <c r="I617"/>
     </row>
-    <row r="618" spans="1:9" ht="15.6">
+    <row r="618" spans="1:9" ht="15.5">
       <c r="A618" s="30" t="s">
         <v>7</v>
       </c>
@@ -17914,7 +17910,7 @@
         <v>211</v>
       </c>
       <c r="G623" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H623" t="s">
         <v>12</v>
@@ -18367,7 +18363,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F633916-1C4C-4A86-8A8C-AB33DBD5A2E2}">
   <dimension ref="A1:K57"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
@@ -18439,7 +18435,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:11" ht="16.350000000000001" customHeight="1">
+    <row r="7" spans="1:11" ht="16.399999999999999" customHeight="1">
       <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
@@ -18703,7 +18699,7 @@
       <c r="H21" s="9"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" spans="1:11" ht="16.350000000000001" customHeight="1">
+    <row r="22" spans="1:11" ht="16.399999999999999" customHeight="1">
       <c r="A22" s="6" t="s">
         <v>2</v>
       </c>
@@ -19348,7 +19344,7 @@
       <c r="I56" s="3"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" spans="1:11" ht="15.6">
+    <row r="57" spans="1:11" ht="15.5">
       <c r="A57" s="28" t="s">
         <v>73</v>
       </c>

</xml_diff>

<commit_message>
Adapted anaerobic digestion inventories to new methane leaks values
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="348" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3859A26C-1B39-4317-828B-F7D7B9FDA0F6}"/>
+  <xr:revisionPtr revIDLastSave="409" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{301C550D-A113-4C7A-AF75-8514A9FBF668}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3807" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3849" uniqueCount="458">
   <si>
     <t>Database</t>
   </si>
@@ -1341,9 +1341,6 @@
     <t>Scaled from the inventory in premise, based on the same source. Considering 1kg methane = 1.39 Nm3</t>
   </si>
   <si>
-    <t>carbon dioxide capture, chemical absorption, with transport and storage, 200 km pipeline sotage 1000m</t>
-  </si>
-  <si>
     <t>market for sodium hydroxide, without water, in 50% solution state</t>
   </si>
   <si>
@@ -1383,9 +1380,6 @@
     <t>Monoethanolamine</t>
   </si>
   <si>
-    <t>carbon dioxide capture, chemical absorption</t>
-  </si>
-  <si>
     <t>Life cycle assessment of carbon capture and storage in power generation and industry in Europe, Volkart et al., 2013, International Journal of Greenhouse Gas Control</t>
   </si>
   <si>
@@ -1402,6 +1396,24 @@
   </si>
   <si>
     <t>biogas purification to biomethane by cryogenic separation with CCS, Tr2050</t>
+  </si>
+  <si>
+    <t>carbon dioxide capture and storage, chemical absorption</t>
+  </si>
+  <si>
+    <t>This activity represents post-combustion CO2 capture using chemical absorption with MEA. The transport has been removed from the original activity since methanation units are assumed to be coupled on-site with anaerobic digestion installations.</t>
+  </si>
+  <si>
+    <t>carbon dioxide storage in plant</t>
+  </si>
+  <si>
+    <t>CO2 storage at 22 bar in steel tank. No electricity is included for compression since the methanation process is assumed to be ran at 20 bar with CO2 capture happening on-site.</t>
+  </si>
+  <si>
+    <t>Based on 8322 operating hours and 20 years of lifetime, considering theorethical CO2 for methanation. Factor = 5.23E-07</t>
+  </si>
+  <si>
+    <t>CO2 storage at 22 bar</t>
   </si>
 </sst>
 </file>
@@ -1613,7 +1625,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1702,6 +1714,10 @@
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
@@ -1723,10 +1739,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1992,7 +2004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH863"/>
+  <dimension ref="A1:AH876"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -2003,7 +2015,7 @@
     <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="99.140625" customWidth="1"/>
+    <col min="9" max="9" width="109.7109375" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7634,7 +7646,7 @@
         <v>209</v>
       </c>
       <c r="C227" s="42">
-        <v>23.580792502540895</v>
+        <v>21.366271416169667</v>
       </c>
       <c r="D227" s="43" t="s">
         <v>13</v>
@@ -7686,7 +7698,7 @@
         <v>20</v>
       </c>
       <c r="C228" s="42">
-        <v>0.15104669391800005</v>
+        <v>0.13686158590383854</v>
       </c>
       <c r="D228" s="43" t="s">
         <v>19</v>
@@ -7736,7 +7748,7 @@
         <v>213</v>
       </c>
       <c r="C229" s="42">
-        <v>3.5844417588325009E-7</v>
+        <v>3.2478194058327522E-7</v>
       </c>
       <c r="D229" s="43" t="s">
         <v>6</v>
@@ -7786,7 +7798,7 @@
         <v>216</v>
       </c>
       <c r="C230" s="42">
-        <v>1.3087058134680292E-6</v>
+        <v>1.1858025387172218E-6</v>
       </c>
       <c r="D230" s="43" t="s">
         <v>6</v>
@@ -7834,7 +7846,7 @@
       </c>
       <c r="B231" s="43"/>
       <c r="C231" s="42">
-        <v>2.4549395159034604</v>
+        <v>2.2243910590121834</v>
       </c>
       <c r="D231" s="43" t="s">
         <v>13</v>
@@ -7884,7 +7896,7 @@
       </c>
       <c r="B232" s="48"/>
       <c r="C232" s="42">
-        <v>0.43565097472690606</v>
+        <v>0.2632929400988413</v>
       </c>
       <c r="D232" s="43" t="s">
         <v>13</v>
@@ -7934,7 +7946,7 @@
       </c>
       <c r="B233" s="48"/>
       <c r="C233" s="42">
-        <v>6.7703710782341719E-2</v>
+        <v>1.3939813637531055E-2</v>
       </c>
       <c r="D233" s="43" t="s">
         <v>13</v>
@@ -7984,7 +7996,7 @@
       </c>
       <c r="B234" s="48"/>
       <c r="C234" s="42">
-        <v>1.3812769695999995E-4</v>
+        <v>1.2515583871999998E-4</v>
       </c>
       <c r="D234" s="43" t="s">
         <v>13</v>
@@ -8034,7 +8046,7 @@
       </c>
       <c r="B235" s="48"/>
       <c r="C235" s="42">
-        <v>7.1938555222999971E-6</v>
+        <v>6.5182656435999982E-6</v>
       </c>
       <c r="D235" s="43" t="s">
         <v>13</v>
@@ -8084,7 +8096,7 @@
       </c>
       <c r="B236" s="48"/>
       <c r="C236" s="42">
-        <v>4.3162373633999985E-5</v>
+        <v>3.9108905687999992E-5</v>
       </c>
       <c r="D236" s="43" t="s">
         <v>13</v>
@@ -8134,7 +8146,7 @@
       </c>
       <c r="B237" s="48"/>
       <c r="C237" s="42">
-        <v>7.1938555222999983E-5</v>
+        <v>6.5182656435999986E-5</v>
       </c>
       <c r="D237" s="43" t="s">
         <v>13</v>
@@ -8184,7 +8196,7 @@
       </c>
       <c r="B238" s="48"/>
       <c r="C238" s="42">
-        <v>5.7551097344999977E-6</v>
+        <v>5.2146354539999984E-6</v>
       </c>
       <c r="D238" s="43" t="s">
         <v>13</v>
@@ -8234,7 +8246,7 @@
       </c>
       <c r="B239" s="48"/>
       <c r="C239" s="42">
-        <v>2.0143200528999993E-11</v>
+        <v>1.8251510827999994E-11</v>
       </c>
       <c r="D239" s="43" t="s">
         <v>13</v>
@@ -8501,7 +8513,7 @@
         <v>227</v>
       </c>
       <c r="C251" s="49">
-        <v>8.8211924785338294</v>
+        <v>8.5232248605658256</v>
       </c>
       <c r="D251" s="43" t="s">
         <v>13</v>
@@ -8529,7 +8541,7 @@
         <v>20</v>
       </c>
       <c r="C252" s="49">
-        <v>0.14643742546928246</v>
+        <v>0.14149097282644188</v>
       </c>
       <c r="D252" s="43" t="s">
         <v>19</v>
@@ -8579,7 +8591,7 @@
         <v>213</v>
       </c>
       <c r="C253" s="42">
-        <v>3.361361524898938E-7</v>
+        <v>3.2478194058327522E-7</v>
       </c>
       <c r="D253" s="43" t="s">
         <v>6</v>
@@ -8629,7 +8641,7 @@
         <v>216</v>
       </c>
       <c r="C254" s="42">
-        <v>1.2687699747005407E-6</v>
+        <v>1.2259126889049042E-6</v>
       </c>
       <c r="D254" s="43" t="s">
         <v>6</v>
@@ -8679,7 +8691,7 @@
       </c>
       <c r="B255" s="43"/>
       <c r="C255" s="49">
-        <v>2.3292600281428992</v>
+        <v>2.2505808627236248</v>
       </c>
       <c r="D255" s="43" t="s">
         <v>13</v>
@@ -8729,7 +8741,7 @@
       </c>
       <c r="B256" s="48"/>
       <c r="C256" s="49">
-        <v>0.32025391175564871</v>
+        <v>0.26554760117984672</v>
       </c>
       <c r="D256" s="43" t="s">
         <v>13</v>
@@ -8779,7 +8791,7 @@
       </c>
       <c r="B257" s="48"/>
       <c r="C257" s="49">
-        <v>3.2023771337382226E-2</v>
+        <v>1.4411332292900546E-2</v>
       </c>
       <c r="D257" s="43" t="s">
         <v>13</v>
@@ -8829,7 +8841,7 @@
       </c>
       <c r="B258" s="48"/>
       <c r="C258" s="42">
-        <v>1.2953122335999999E-4</v>
+        <v>1.2515583872E-4</v>
       </c>
       <c r="D258" s="43" t="s">
         <v>13</v>
@@ -8879,7 +8891,7 @@
       </c>
       <c r="B259" s="48"/>
       <c r="C259" s="42">
-        <v>6.7461409042999994E-6</v>
+        <v>6.5182656435999991E-6</v>
       </c>
       <c r="D259" s="43" t="s">
         <v>13</v>
@@ -8929,7 +8941,7 @@
       </c>
       <c r="B260" s="48"/>
       <c r="C260" s="42">
-        <v>4.0476133193999995E-5</v>
+        <v>3.9108905687999992E-5</v>
       </c>
       <c r="D260" s="43" t="s">
         <v>13</v>
@@ -8979,7 +8991,7 @@
       </c>
       <c r="B261" s="48"/>
       <c r="C261" s="42">
-        <v>6.7461409043000002E-5</v>
+        <v>6.5182656435999999E-5</v>
       </c>
       <c r="D261" s="43" t="s">
         <v>13</v>
@@ -9029,7 +9041,7 @@
       </c>
       <c r="B262" s="48"/>
       <c r="C262" s="42">
-        <v>5.3969364644999994E-6</v>
+        <v>5.2146354539999992E-6</v>
       </c>
       <c r="D262" s="43" t="s">
         <v>13</v>
@@ -9079,7 +9091,7 @@
       </c>
       <c r="B263" s="48"/>
       <c r="C263" s="42">
-        <v>1.8889574388999996E-11</v>
+        <v>1.8251510827999997E-11</v>
       </c>
       <c r="D263" s="43" t="s">
         <v>13</v>
@@ -9587,7 +9599,7 @@
         <v>233</v>
       </c>
       <c r="C275" s="49">
-        <v>7.3642594776735102</v>
+        <v>7.1155050309249033</v>
       </c>
       <c r="D275" s="43" t="s">
         <v>13</v>
@@ -9639,7 +9651,7 @@
         <v>20</v>
       </c>
       <c r="C276" s="49">
-        <v>0.14755967936260125</v>
+        <v>0.14257531854349526</v>
       </c>
       <c r="D276" s="43" t="s">
         <v>19</v>
@@ -9689,7 +9701,7 @@
         <v>213</v>
       </c>
       <c r="C277" s="42">
-        <v>3.361361524898938E-7</v>
+        <v>3.2478194058327522E-7</v>
       </c>
       <c r="D277" s="43" t="s">
         <v>6</v>
@@ -9739,7 +9751,7 @@
         <v>216</v>
       </c>
       <c r="C278" s="42">
-        <v>1.278493459248774E-6</v>
+        <v>1.2353077276634966E-6</v>
       </c>
       <c r="D278" s="43" t="s">
         <v>6</v>
@@ -9789,7 +9801,7 @@
       </c>
       <c r="B279" s="43"/>
       <c r="C279" s="49">
-        <v>2.3298053529472447</v>
+        <v>2.2511077672142359</v>
       </c>
       <c r="D279" s="43" t="s">
         <v>13</v>
@@ -9814,7 +9826,7 @@
       </c>
       <c r="B280" s="51"/>
       <c r="C280" s="49">
-        <v>0.31967459976937124</v>
+        <v>0.2653153277009781</v>
       </c>
       <c r="D280" s="43" t="s">
         <v>13</v>
@@ -9839,7 +9851,7 @@
       </c>
       <c r="B281" s="48"/>
       <c r="C281" s="49">
-        <v>3.2269192219011061E-2</v>
+        <v>1.4521776557553446E-2</v>
       </c>
       <c r="D281" s="43" t="s">
         <v>13</v>
@@ -9864,7 +9876,7 @@
       </c>
       <c r="B282" s="48"/>
       <c r="C282" s="42">
-        <v>1.2953122335999999E-4</v>
+        <v>1.2515583872E-4</v>
       </c>
       <c r="D282" s="43" t="s">
         <v>13</v>
@@ -9914,7 +9926,7 @@
       </c>
       <c r="B283" s="48"/>
       <c r="C283" s="42">
-        <v>6.7461409042999994E-6</v>
+        <v>6.5182656435999991E-6</v>
       </c>
       <c r="D283" s="43" t="s">
         <v>13</v>
@@ -9964,7 +9976,7 @@
       </c>
       <c r="B284" s="48"/>
       <c r="C284" s="42">
-        <v>4.0476133193999995E-5</v>
+        <v>3.9108905687999992E-5</v>
       </c>
       <c r="D284" s="43" t="s">
         <v>13</v>
@@ -10014,7 +10026,7 @@
       </c>
       <c r="B285" s="48"/>
       <c r="C285" s="42">
-        <v>6.7461409043000002E-5</v>
+        <v>6.5182656435999999E-5</v>
       </c>
       <c r="D285" s="43" t="s">
         <v>13</v>
@@ -10064,7 +10076,7 @@
       </c>
       <c r="B286" s="48"/>
       <c r="C286" s="42">
-        <v>5.3969364644999994E-6</v>
+        <v>5.2146354539999992E-6</v>
       </c>
       <c r="D286" s="43" t="s">
         <v>13</v>
@@ -10114,7 +10126,7 @@
       </c>
       <c r="B287" s="48"/>
       <c r="C287" s="42">
-        <v>1.8889574388999996E-11</v>
+        <v>1.8251510827999997E-11</v>
       </c>
       <c r="D287" s="43" t="s">
         <v>13</v>
@@ -10619,7 +10631,7 @@
         <v>237</v>
       </c>
       <c r="C299" s="49">
-        <v>8.600396986554621</v>
+        <v>8.3098875333373829</v>
       </c>
       <c r="D299" s="43" t="s">
         <v>13</v>
@@ -10669,7 +10681,7 @@
         <v>20</v>
       </c>
       <c r="C300" s="49">
-        <v>0.14704987784003279</v>
+        <v>0.14208273740759059</v>
       </c>
       <c r="D300" s="43" t="s">
         <v>19</v>
@@ -10695,7 +10707,7 @@
         <v>213</v>
       </c>
       <c r="C301" s="42">
-        <v>3.361361524898938E-7</v>
+        <v>3.2478194058327522E-7</v>
       </c>
       <c r="D301" s="43" t="s">
         <v>6</v>
@@ -10721,7 +10733,7 @@
         <v>216</v>
       </c>
       <c r="C302" s="42">
-        <v>1.274076413108973E-6</v>
+        <v>1.2310398832013525E-6</v>
       </c>
       <c r="D302" s="43" t="s">
         <v>6</v>
@@ -10747,7 +10759,7 @@
       </c>
       <c r="B303" s="43"/>
       <c r="C303" s="49">
-        <v>2.3289945729253771</v>
+        <v>2.2503243742142924</v>
       </c>
       <c r="D303" s="43" t="s">
         <v>13</v>
@@ -10772,7 +10784,7 @@
       </c>
       <c r="B304" s="51"/>
       <c r="C304" s="49">
-        <v>0.31983905736853946</v>
+        <v>0.26534706999299229</v>
       </c>
       <c r="D304" s="43" t="s">
         <v>13</v>
@@ -10797,7 +10809,7 @@
       </c>
       <c r="B305" s="48"/>
       <c r="C305" s="49">
-        <v>3.2157705914646832E-2</v>
+        <v>1.4471605509260181E-2</v>
       </c>
       <c r="D305" s="43" t="s">
         <v>13</v>
@@ -10822,7 +10834,7 @@
       </c>
       <c r="B306" s="48"/>
       <c r="C306" s="42">
-        <v>1.2953122335999996E-4</v>
+        <v>1.2515583871999998E-4</v>
       </c>
       <c r="D306" s="43" t="s">
         <v>13</v>
@@ -10848,7 +10860,7 @@
       </c>
       <c r="B307" s="48"/>
       <c r="C307" s="42">
-        <v>6.7461409042999986E-6</v>
+        <v>6.5182656435999982E-6</v>
       </c>
       <c r="D307" s="43" t="s">
         <v>13</v>
@@ -10874,7 +10886,7 @@
       </c>
       <c r="B308" s="48"/>
       <c r="C308" s="42">
-        <v>4.0476133193999988E-5</v>
+        <v>3.9108905687999992E-5</v>
       </c>
       <c r="D308" s="43" t="s">
         <v>13</v>
@@ -10900,7 +10912,7 @@
       </c>
       <c r="B309" s="48"/>
       <c r="C309" s="42">
-        <v>6.7461409042999989E-5</v>
+        <v>6.5182656435999986E-5</v>
       </c>
       <c r="D309" s="43" t="s">
         <v>13</v>
@@ -10926,7 +10938,7 @@
       </c>
       <c r="B310" s="48"/>
       <c r="C310" s="42">
-        <v>5.3969364644999985E-6</v>
+        <v>5.2146354539999984E-6</v>
       </c>
       <c r="D310" s="43" t="s">
         <v>13</v>
@@ -10952,7 +10964,7 @@
       </c>
       <c r="B311" s="48"/>
       <c r="C311" s="42">
-        <v>1.8889574388999996E-11</v>
+        <v>1.8251510827999994E-11</v>
       </c>
       <c r="D311" s="43" t="s">
         <v>13</v>
@@ -11436,7 +11448,7 @@
         <v>240</v>
       </c>
       <c r="C323" s="49">
-        <v>12.2842813266157</v>
+        <v>11.869335382034194</v>
       </c>
       <c r="D323" s="43" t="s">
         <v>13</v>
@@ -11488,7 +11500,7 @@
         <v>20</v>
       </c>
       <c r="C324" s="49">
-        <v>0.14683967094502717</v>
+        <v>0.14187963100925111</v>
       </c>
       <c r="D324" s="43" t="s">
         <v>19</v>
@@ -11514,7 +11526,7 @@
         <v>213</v>
       </c>
       <c r="C325" s="42">
-        <v>3.361361524898938E-7</v>
+        <v>3.2478194058327522E-7</v>
       </c>
       <c r="D325" s="43" t="s">
         <v>6</v>
@@ -11540,7 +11552,7 @@
         <v>216</v>
       </c>
       <c r="C326" s="42">
-        <v>1.2722551287207543E-6</v>
+        <v>1.2292801192676664E-6</v>
       </c>
       <c r="D326" s="43" t="s">
         <v>6</v>
@@ -11566,7 +11578,7 @@
       </c>
       <c r="B327" s="43"/>
       <c r="C327" s="49">
-        <v>2.3281445513202397</v>
+        <v>2.2495030651572057</v>
       </c>
       <c r="D327" s="43" t="s">
         <v>13</v>
@@ -11591,7 +11603,7 @@
       </c>
       <c r="B328" s="51"/>
       <c r="C328" s="42">
-        <v>0.3198164639983479</v>
+        <v>0.26529258993003446</v>
       </c>
       <c r="D328" s="43" t="s">
         <v>13</v>
@@ -11616,7 +11628,7 @@
       </c>
       <c r="B329" s="48"/>
       <c r="C329" s="42">
-        <v>3.2111736672032598E-2</v>
+        <v>1.4450918438284459E-2</v>
       </c>
       <c r="D329" s="43" t="s">
         <v>13</v>
@@ -11641,7 +11653,7 @@
       </c>
       <c r="B330" s="48"/>
       <c r="C330" s="42">
-        <v>1.2953122335999999E-4</v>
+        <v>1.2515583872E-4</v>
       </c>
       <c r="D330" s="43" t="s">
         <v>13</v>
@@ -11667,7 +11679,7 @@
       </c>
       <c r="B331" s="48"/>
       <c r="C331" s="42">
-        <v>6.7461409042999994E-6</v>
+        <v>6.5182656435999991E-6</v>
       </c>
       <c r="D331" s="43" t="s">
         <v>13</v>
@@ -11693,7 +11705,7 @@
       </c>
       <c r="B332" s="48"/>
       <c r="C332" s="42">
-        <v>4.0476133193999995E-5</v>
+        <v>3.9108905687999992E-5</v>
       </c>
       <c r="D332" s="43" t="s">
         <v>13</v>
@@ -11719,7 +11731,7 @@
       </c>
       <c r="B333" s="48"/>
       <c r="C333" s="42">
-        <v>6.7461409043000002E-5</v>
+        <v>6.5182656435999999E-5</v>
       </c>
       <c r="D333" s="43" t="s">
         <v>13</v>
@@ -11745,7 +11757,7 @@
       </c>
       <c r="B334" s="48"/>
       <c r="C334" s="42">
-        <v>5.3969364644999994E-6</v>
+        <v>5.2146354539999992E-6</v>
       </c>
       <c r="D334" s="43" t="s">
         <v>13</v>
@@ -11771,7 +11783,7 @@
       </c>
       <c r="B335" s="48"/>
       <c r="C335" s="42">
-        <v>1.8889574388999996E-11</v>
+        <v>1.8251510827999997E-11</v>
       </c>
       <c r="D335" s="43" t="s">
         <v>13</v>
@@ -18362,7 +18374,7 @@
         <v>1</v>
       </c>
       <c r="B651" s="41" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="652" spans="1:8">
@@ -18446,7 +18458,7 @@
     </row>
     <row r="660" spans="1:9">
       <c r="A660" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B660" t="s">
         <v>259</v>
@@ -18734,7 +18746,7 @@
         <v>1</v>
       </c>
       <c r="B674" s="41" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="675" spans="1:9">
@@ -18818,7 +18830,7 @@
     </row>
     <row r="683" spans="1:9">
       <c r="A683" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B683" t="s">
         <v>259</v>
@@ -19286,7 +19298,7 @@
         <v>1</v>
       </c>
       <c r="B705" s="41" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="706" spans="1:9">
@@ -19370,7 +19382,7 @@
     </row>
     <row r="714" spans="1:9">
       <c r="A714" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B714" t="s">
         <v>259</v>
@@ -19838,7 +19850,7 @@
         <v>1</v>
       </c>
       <c r="B736" s="41" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="737" spans="1:9">
@@ -19922,7 +19934,7 @@
     </row>
     <row r="745" spans="1:9">
       <c r="A745" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B745" t="s">
         <v>259</v>
@@ -20398,7 +20410,7 @@
         <v>1</v>
       </c>
       <c r="B767" s="41" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="768" spans="1:9">
@@ -20482,7 +20494,7 @@
     </row>
     <row r="776" spans="1:9">
       <c r="A776" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B776" t="s">
         <v>259</v>
@@ -21176,10 +21188,10 @@
     </row>
     <row r="809" spans="1:21">
       <c r="A809" s="48" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="B809" s="48" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="C809">
         <v>1.9717499999999999</v>
@@ -21188,7 +21200,7 @@
         <v>13</v>
       </c>
       <c r="G809" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="H809" t="s">
         <v>12</v>
@@ -22121,7 +22133,7 @@
         <v>1</v>
       </c>
       <c r="B841" s="41" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="C841" s="42"/>
     </row>
@@ -22129,6 +22141,9 @@
       <c r="A842" s="41" t="s">
         <v>11</v>
       </c>
+      <c r="B842" s="43" t="s">
+        <v>453</v>
+      </c>
       <c r="C842" s="42"/>
     </row>
     <row r="843" spans="1:21" s="43" customFormat="1">
@@ -22136,7 +22151,7 @@
         <v>2</v>
       </c>
       <c r="B843" s="43" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="C843" s="42"/>
     </row>
@@ -22145,7 +22160,7 @@
         <v>4</v>
       </c>
       <c r="B844" s="48" t="s">
-        <v>433</v>
+        <v>452</v>
       </c>
       <c r="C844" s="42"/>
     </row>
@@ -22174,7 +22189,7 @@
         <v>76</v>
       </c>
       <c r="B847" s="43" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C847" s="42"/>
       <c r="D847" s="46"/>
@@ -22216,10 +22231,10 @@
     </row>
     <row r="850" spans="1:11" s="43" customFormat="1">
       <c r="A850" s="48" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="B850" s="48" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="C850" s="65">
         <v>1</v>
@@ -22230,7 +22245,7 @@
       <c r="E850" s="48"/>
       <c r="F850" s="48"/>
       <c r="G850" s="48" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="H850" s="48" t="s">
         <v>18</v>
@@ -22241,50 +22256,50 @@
     </row>
     <row r="851" spans="1:11" s="43" customFormat="1">
       <c r="A851" s="48" t="s">
-        <v>45</v>
+        <v>454</v>
       </c>
       <c r="B851" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="C851" s="66">
-        <v>0.38400000000000001</v>
-      </c>
-      <c r="D851" t="s">
-        <v>19</v>
-      </c>
-      <c r="E851" t="s">
-        <v>211</v>
-      </c>
-      <c r="F851"/>
-      <c r="G851" t="s">
+        <v>454</v>
+      </c>
+      <c r="C851" s="65">
+        <v>1</v>
+      </c>
+      <c r="D851" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E851" s="48"/>
+      <c r="F851" s="48"/>
+      <c r="G851" s="48" t="s">
         <v>29</v>
       </c>
       <c r="H851" t="s">
         <v>12</v>
       </c>
-      <c r="I851"/>
+      <c r="I851" s="48" t="s">
+        <v>457</v>
+      </c>
       <c r="J851" s="48"/>
       <c r="K851" s="48"/>
     </row>
     <row r="852" spans="1:11" s="43" customFormat="1">
-      <c r="A852" t="s">
-        <v>274</v>
-      </c>
-      <c r="B852" t="s">
-        <v>275</v>
-      </c>
-      <c r="C852" s="18">
-        <v>2.8400000000000002E-4</v>
+      <c r="A852" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="B852" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C852" s="66">
+        <v>0.38400000000000001</v>
       </c>
       <c r="D852" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E852" t="s">
         <v>211</v>
       </c>
       <c r="F852"/>
       <c r="G852" t="s">
-        <v>140</v>
+        <v>29</v>
       </c>
       <c r="H852" t="s">
         <v>12</v>
@@ -22295,13 +22310,13 @@
     </row>
     <row r="853" spans="1:11" s="43" customFormat="1">
       <c r="A853" t="s">
-        <v>434</v>
+        <v>274</v>
       </c>
       <c r="B853" t="s">
-        <v>435</v>
+        <v>275</v>
       </c>
       <c r="C853" s="18">
-        <v>3.0400000000000002E-4</v>
+        <v>2.8400000000000002E-4</v>
       </c>
       <c r="D853" t="s">
         <v>13</v>
@@ -22322,13 +22337,13 @@
     </row>
     <row r="854" spans="1:11" s="43" customFormat="1">
       <c r="A854" t="s">
-        <v>276</v>
+        <v>433</v>
       </c>
       <c r="B854" t="s">
-        <v>277</v>
+        <v>434</v>
       </c>
       <c r="C854" s="18">
-        <v>8.2600000000000002E-5</v>
+        <v>3.0400000000000002E-4</v>
       </c>
       <c r="D854" t="s">
         <v>13</v>
@@ -22349,23 +22364,23 @@
     </row>
     <row r="855" spans="1:11" s="43" customFormat="1">
       <c r="A855" t="s">
-        <v>436</v>
+        <v>276</v>
       </c>
       <c r="B855" t="s">
-        <v>437</v>
+        <v>277</v>
       </c>
       <c r="C855" s="18">
-        <v>8.2699999999999996E-11</v>
+        <v>8.2600000000000002E-5</v>
       </c>
       <c r="D855" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E855" t="s">
         <v>211</v>
       </c>
       <c r="F855"/>
       <c r="G855" t="s">
-        <v>49</v>
+        <v>140</v>
       </c>
       <c r="H855" t="s">
         <v>12</v>
@@ -22376,13 +22391,13 @@
     </row>
     <row r="856" spans="1:11" s="43" customFormat="1">
       <c r="A856" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B856" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C856" s="18">
-        <v>7.4400000000000002E-10</v>
+        <v>8.2699999999999996E-11</v>
       </c>
       <c r="D856" t="s">
         <v>6</v>
@@ -22392,7 +22407,7 @@
       </c>
       <c r="F856"/>
       <c r="G856" t="s">
-        <v>140</v>
+        <v>49</v>
       </c>
       <c r="H856" t="s">
         <v>12</v>
@@ -22403,13 +22418,13 @@
     </row>
     <row r="857" spans="1:11" s="43" customFormat="1">
       <c r="A857" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B857" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C857" s="18">
-        <v>3.3099999999999999E-10</v>
+        <v>7.4400000000000002E-10</v>
       </c>
       <c r="D857" t="s">
         <v>6</v>
@@ -22430,13 +22445,13 @@
     </row>
     <row r="858" spans="1:11" s="43" customFormat="1">
       <c r="A858" t="s">
-        <v>144</v>
+        <v>439</v>
       </c>
       <c r="B858" t="s">
-        <v>145</v>
+        <v>440</v>
       </c>
       <c r="C858" s="18">
-        <v>5.1400000000000003E-12</v>
+        <v>3.3099999999999999E-10</v>
       </c>
       <c r="D858" t="s">
         <v>6</v>
@@ -22457,13 +22472,13 @@
     </row>
     <row r="859" spans="1:11" s="43" customFormat="1">
       <c r="A859" t="s">
-        <v>442</v>
+        <v>144</v>
       </c>
       <c r="B859" t="s">
-        <v>443</v>
+        <v>145</v>
       </c>
       <c r="C859" s="18">
-        <v>5.7899999999999997E-10</v>
+        <v>5.1400000000000003E-12</v>
       </c>
       <c r="D859" t="s">
         <v>6</v>
@@ -22484,23 +22499,23 @@
     </row>
     <row r="860" spans="1:11" s="43" customFormat="1">
       <c r="A860" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B860" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="C860" s="18">
-        <v>-2.2699999999999999E-4</v>
+        <v>5.7899999999999997E-10</v>
       </c>
       <c r="D860" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E860" t="s">
         <v>211</v>
       </c>
       <c r="F860"/>
       <c r="G860" t="s">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="H860" t="s">
         <v>12</v>
@@ -22510,64 +22525,66 @@
       <c r="K860" s="48"/>
     </row>
     <row r="861" spans="1:11" s="43" customFormat="1">
-      <c r="A861" s="48" t="s">
-        <v>127</v>
-      </c>
-      <c r="B861" s="48"/>
-      <c r="C861" s="67">
-        <v>8.3199999999999996E-2</v>
-      </c>
-      <c r="D861" s="43" t="s">
-        <v>128</v>
-      </c>
-      <c r="E861" s="48" t="s">
-        <v>109</v>
-      </c>
-      <c r="F861" s="43" t="s">
-        <v>129</v>
-      </c>
-      <c r="G861"/>
+      <c r="A861" t="s">
+        <v>443</v>
+      </c>
+      <c r="B861" t="s">
+        <v>444</v>
+      </c>
+      <c r="C861" s="18">
+        <v>-2.2699999999999999E-4</v>
+      </c>
+      <c r="D861" t="s">
+        <v>13</v>
+      </c>
+      <c r="E861" t="s">
+        <v>211</v>
+      </c>
+      <c r="F861"/>
+      <c r="G861" t="s">
+        <v>22</v>
+      </c>
       <c r="H861" t="s">
-        <v>15</v>
-      </c>
-      <c r="I861" s="48"/>
+        <v>12</v>
+      </c>
+      <c r="I861"/>
       <c r="J861" s="48"/>
       <c r="K861" s="48"/>
     </row>
     <row r="862" spans="1:11" s="43" customFormat="1">
-      <c r="A862" t="s">
-        <v>284</v>
-      </c>
-      <c r="B862"/>
-      <c r="C862" s="18">
-        <v>1.2300000000000001E-4</v>
-      </c>
-      <c r="D862" t="s">
-        <v>13</v>
+      <c r="A862" s="48" t="s">
+        <v>127</v>
+      </c>
+      <c r="B862" s="48"/>
+      <c r="C862" s="67">
+        <v>8.3199999999999996E-2</v>
+      </c>
+      <c r="D862" s="43" t="s">
+        <v>128</v>
       </c>
       <c r="E862" s="48" t="s">
         <v>109</v>
       </c>
-      <c r="F862" s="45" t="s">
-        <v>184</v>
+      <c r="F862" s="43" t="s">
+        <v>129</v>
       </c>
       <c r="G862"/>
       <c r="H862" t="s">
         <v>15</v>
       </c>
-      <c r="I862"/>
+      <c r="I862" s="48"/>
       <c r="J862" s="48"/>
       <c r="K862" s="48"/>
     </row>
     <row r="863" spans="1:11" s="43" customFormat="1">
-      <c r="A863" s="48" t="s">
-        <v>446</v>
-      </c>
-      <c r="B863" s="48"/>
-      <c r="C863" s="46">
-        <v>6.0000000000000002E-6</v>
-      </c>
-      <c r="D863" s="43" t="s">
+      <c r="A863" t="s">
+        <v>284</v>
+      </c>
+      <c r="B863"/>
+      <c r="C863" s="18">
+        <v>1.2300000000000001E-4</v>
+      </c>
+      <c r="D863" t="s">
         <v>13</v>
       </c>
       <c r="E863" s="48" t="s">
@@ -22580,9 +22597,195 @@
       <c r="H863" t="s">
         <v>15</v>
       </c>
-      <c r="I863" s="48"/>
+      <c r="I863"/>
       <c r="J863" s="48"/>
       <c r="K863" s="48"/>
+    </row>
+    <row r="864" spans="1:11" s="43" customFormat="1">
+      <c r="A864" s="48" t="s">
+        <v>445</v>
+      </c>
+      <c r="B864" s="48"/>
+      <c r="C864" s="46">
+        <v>6.0000000000000002E-6</v>
+      </c>
+      <c r="D864" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E864" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="F864" s="45" t="s">
+        <v>184</v>
+      </c>
+      <c r="G864"/>
+      <c r="H864" t="s">
+        <v>15</v>
+      </c>
+      <c r="I864" s="48"/>
+      <c r="J864" s="48"/>
+      <c r="K864" s="48"/>
+    </row>
+    <row r="865" spans="1:11">
+      <c r="A865" s="53"/>
+      <c r="B865" s="54"/>
+      <c r="C865" s="53"/>
+      <c r="D865" s="53"/>
+      <c r="E865" s="53"/>
+      <c r="F865" s="53"/>
+      <c r="G865" s="53"/>
+      <c r="H865" s="53"/>
+      <c r="I865" s="53"/>
+    </row>
+    <row r="866" spans="1:11" s="43" customFormat="1">
+      <c r="A866" s="41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B866" s="68" t="s">
+        <v>454</v>
+      </c>
+      <c r="C866" s="42"/>
+    </row>
+    <row r="867" spans="1:11" s="43" customFormat="1">
+      <c r="A867" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B867" s="48" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="868" spans="1:11" s="43" customFormat="1">
+      <c r="A868" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="B868" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="C868" s="42"/>
+    </row>
+    <row r="869" spans="1:11" s="43" customFormat="1">
+      <c r="A869" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="B869" s="48" t="s">
+        <v>454</v>
+      </c>
+      <c r="C869" s="42"/>
+    </row>
+    <row r="870" spans="1:11" s="43" customFormat="1">
+      <c r="A870" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="B870" s="45">
+        <v>1</v>
+      </c>
+      <c r="C870" s="42"/>
+      <c r="D870" s="46"/>
+    </row>
+    <row r="871" spans="1:11" s="43" customFormat="1">
+      <c r="A871" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B871" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="C871" s="42"/>
+      <c r="D871" s="46"/>
+    </row>
+    <row r="872" spans="1:11" s="43" customFormat="1">
+      <c r="A872" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B872" s="43" t="s">
+        <v>403</v>
+      </c>
+      <c r="C872" s="42"/>
+      <c r="D872" s="46"/>
+    </row>
+    <row r="873" spans="1:11" s="43" customFormat="1">
+      <c r="A873" s="41" t="s">
+        <v>7</v>
+      </c>
+      <c r="C873" s="42"/>
+    </row>
+    <row r="874" spans="1:11" s="43" customFormat="1">
+      <c r="A874" s="41" t="s">
+        <v>8</v>
+      </c>
+      <c r="B874" s="41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C874" s="47" t="s">
+        <v>9</v>
+      </c>
+      <c r="D874" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="E874" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="F874" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G874" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="H874" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="I874" s="41" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="875" spans="1:11" s="43" customFormat="1">
+      <c r="A875" s="48" t="s">
+        <v>454</v>
+      </c>
+      <c r="B875" s="48" t="s">
+        <v>454</v>
+      </c>
+      <c r="C875" s="65">
+        <v>1</v>
+      </c>
+      <c r="D875" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E875" s="48"/>
+      <c r="F875" s="48"/>
+      <c r="G875" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="H875" t="s">
+        <v>18</v>
+      </c>
+      <c r="J875" s="48"/>
+      <c r="K875" s="48"/>
+    </row>
+    <row r="876" spans="1:11" s="43" customFormat="1">
+      <c r="A876" s="43" t="s">
+        <v>267</v>
+      </c>
+      <c r="B876" s="43" t="s">
+        <v>268</v>
+      </c>
+      <c r="C876" s="69">
+        <v>1.3129534488582797E-3</v>
+      </c>
+      <c r="D876" s="43" t="s">
+        <v>13</v>
+      </c>
+      <c r="E876" t="s">
+        <v>211</v>
+      </c>
+      <c r="G876" s="43" t="s">
+        <v>140</v>
+      </c>
+      <c r="H876" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="I876" s="43" t="s">
+        <v>456</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Modified biowaste collection value (cut-off)
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="409" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{301C550D-A113-4C7A-AF75-8514A9FBF668}"/>
+  <xr:revisionPtr revIDLastSave="414" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B73EFCCE-38DB-4B53-B421-30AADF34CEC4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -6078,7 +6078,7 @@
         <v>291</v>
       </c>
       <c r="C190" s="49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D190" s="43" t="s">
         <v>13</v>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="B191" s="43"/>
       <c r="C191" s="49">
-        <v>2.4324509555475786</v>
+        <v>2.2403011395943495</v>
       </c>
       <c r="D191" s="43" t="s">
         <v>13</v>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="B203" s="43"/>
       <c r="C203" s="49">
-        <v>2.4411239472074011</v>
+        <v>2.2482890141514411</v>
       </c>
       <c r="D203" s="43" t="s">
         <v>13</v>
@@ -7138,7 +7138,7 @@
       </c>
       <c r="B215" s="43"/>
       <c r="C215" s="49">
-        <v>2.4264812291656459</v>
+        <v>2.2348029877051991</v>
       </c>
       <c r="D215" s="43" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Modified inventories to correct for biogas market as input in purification activities
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1290" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97970104-FA1D-4428-B530-8285CC28D1E0}"/>
+  <xr:revisionPtr revIDLastSave="1312" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{444287BB-FE43-4137-874D-06C43648E757}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -804,9 +804,6 @@
     <t>steel, chromium steel 18/8</t>
   </si>
   <si>
-    <t>market for biogas to biomethane, Tr2050</t>
-  </si>
-  <si>
     <t>empty activity, for market that does not exist any more in 2050, Tr2050</t>
   </si>
   <si>
@@ -1522,6 +1519,9 @@
   </si>
   <si>
     <t>Scaled to reference product based on ecoinvent Faist Emmenegger M., Del Duce A., Moreno Ruiz E., Brunner F., (2017). Update of the European natural gas supply chains. Ecoinvent, Zürich, Switzerland</t>
+  </si>
+  <si>
+    <t>market for biogas</t>
   </si>
 </sst>
 </file>
@@ -4457,7 +4457,7 @@
     </row>
     <row r="116" spans="1:9">
       <c r="A116" s="36" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B116" s="34">
         <v>4.3695687769999996</v>
@@ -5583,7 +5583,7 @@
     </row>
     <row r="166" spans="1:9">
       <c r="A166" s="36" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B166" s="34">
         <v>4.3011681309999998</v>
@@ -5622,7 +5622,7 @@
         <v>1</v>
       </c>
       <c r="B168" s="29" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -5638,7 +5638,7 @@
         <v>11</v>
       </c>
       <c r="B170" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="171" spans="1:9">
@@ -5660,7 +5660,7 @@
         <v>4</v>
       </c>
       <c r="B173" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="174" spans="1:9">
@@ -5815,7 +5815,7 @@
         <v>11</v>
       </c>
       <c r="B181" s="41" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C181" s="40"/>
       <c r="D181" s="41"/>
@@ -6192,10 +6192,10 @@
     </row>
     <row r="190" spans="1:34">
       <c r="A190" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="B190" s="46" t="s">
         <v>275</v>
-      </c>
-      <c r="B190" s="46" t="s">
-        <v>276</v>
       </c>
       <c r="C190" s="47">
         <v>0</v>
@@ -6921,7 +6921,7 @@
         <v>11</v>
       </c>
       <c r="B205" s="41" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C205" s="40"/>
       <c r="D205" s="41"/>
@@ -7977,7 +7977,7 @@
         <v>11</v>
       </c>
       <c r="B228" s="41" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C228" s="40"/>
       <c r="D228" s="41"/>
@@ -9033,7 +9033,7 @@
         <v>11</v>
       </c>
       <c r="B251" s="41" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C251" s="40"/>
       <c r="D251" s="41"/>
@@ -10117,7 +10117,7 @@
         <v>11</v>
       </c>
       <c r="B275" s="41" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C275" s="40"/>
       <c r="D275" s="41"/>
@@ -10986,7 +10986,7 @@
         <v>11</v>
       </c>
       <c r="B299" s="41" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C299" s="40"/>
       <c r="D299" s="41"/>
@@ -11363,10 +11363,10 @@
     </row>
     <row r="308" spans="1:34">
       <c r="A308" s="41" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B308" s="41" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C308" s="47">
         <v>7.1155050309249033</v>
@@ -12021,7 +12021,7 @@
         <v>11</v>
       </c>
       <c r="B323" s="41" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C323" s="40"/>
       <c r="D323" s="41"/>
@@ -12835,7 +12835,7 @@
         <v>11</v>
       </c>
       <c r="B347" s="41" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C347" s="40"/>
       <c r="D347" s="41"/>
@@ -13629,7 +13629,7 @@
         <v>11</v>
       </c>
       <c r="B371" s="41" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C371" s="40"/>
       <c r="D371" s="41"/>
@@ -13800,15 +13800,15 @@
         <v>12</v>
       </c>
       <c r="I380" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="381" spans="1:34">
       <c r="A381" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B381" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C381" s="47">
         <v>1</v>
@@ -13882,7 +13882,7 @@
         <v>11</v>
       </c>
       <c r="B384" s="41" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C384" s="40"/>
       <c r="D384" s="41"/>
@@ -14056,7 +14056,7 @@
         <v>12</v>
       </c>
       <c r="I393" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="394" spans="1:34">
@@ -14083,15 +14083,15 @@
         <v>12</v>
       </c>
       <c r="I394" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="395" spans="1:34">
       <c r="A395" s="46" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B395" s="46" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C395" s="47">
         <v>8.4999999999999995E-4</v>
@@ -14110,7 +14110,7 @@
         <v>12</v>
       </c>
       <c r="I395" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="396" spans="1:34" s="69" customFormat="1">
@@ -14169,7 +14169,7 @@
         <v>11</v>
       </c>
       <c r="B398" s="41" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C398" s="40"/>
       <c r="D398" s="41"/>
@@ -14244,7 +14244,7 @@
         <v>76</v>
       </c>
       <c r="B403" s="41" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C403" s="40"/>
       <c r="D403" s="44"/>
@@ -14345,7 +14345,7 @@
         <v>12</v>
       </c>
       <c r="I407" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="408" spans="1:34" s="69" customFormat="1">
@@ -14429,7 +14429,7 @@
         <v>11</v>
       </c>
       <c r="B410" s="41" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C410" s="40"/>
       <c r="D410" s="41"/>
@@ -14629,7 +14629,7 @@
         <v>76</v>
       </c>
       <c r="B415" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C415" s="40"/>
       <c r="D415" s="44"/>
@@ -14830,7 +14830,7 @@
         <v>12</v>
       </c>
       <c r="I419" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J419" s="46"/>
       <c r="K419" s="46"/>
@@ -14882,7 +14882,7 @@
         <v>12</v>
       </c>
       <c r="I420" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J420" s="46"/>
       <c r="K420" s="46"/>
@@ -14912,10 +14912,10 @@
     </row>
     <row r="421" spans="1:34">
       <c r="A421" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B421" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C421" s="54">
         <v>8.4999999999999995E-4</v>
@@ -14934,7 +14934,7 @@
         <v>12</v>
       </c>
       <c r="I421" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="422" spans="1:34" s="69" customFormat="1">
@@ -14978,7 +14978,7 @@
         <v>1</v>
       </c>
       <c r="B423" s="39" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C423" s="40"/>
       <c r="D423" s="41"/>
@@ -14993,7 +14993,7 @@
         <v>11</v>
       </c>
       <c r="B424" s="41" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C424" s="40"/>
       <c r="D424" s="41"/>
@@ -15023,7 +15023,7 @@
         <v>4</v>
       </c>
       <c r="B426" s="46" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C426" s="40"/>
       <c r="D426" s="44"/>
@@ -15068,7 +15068,7 @@
         <v>76</v>
       </c>
       <c r="B429" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C429" s="40"/>
       <c r="D429" s="44"/>
@@ -15122,10 +15122,10 @@
     </row>
     <row r="432" spans="1:34">
       <c r="A432" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="B432" s="46" t="s">
         <v>275</v>
-      </c>
-      <c r="B432" s="46" t="s">
-        <v>276</v>
       </c>
       <c r="C432" s="47">
         <v>1</v>
@@ -15147,10 +15147,10 @@
     </row>
     <row r="433" spans="1:34">
       <c r="A433" s="46" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B433" s="46" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C433" s="54">
         <v>0.1</v>
@@ -15169,7 +15169,7 @@
         <v>12</v>
       </c>
       <c r="I433" s="46" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="434" spans="1:34">
@@ -15196,15 +15196,15 @@
         <v>12</v>
       </c>
       <c r="I434" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="435" spans="1:34">
       <c r="A435" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B435" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C435" s="54">
         <v>8.4999999999999995E-4</v>
@@ -15223,7 +15223,7 @@
         <v>12</v>
       </c>
       <c r="I435" s="46" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="436" spans="1:34" s="69" customFormat="1">
@@ -15267,7 +15267,7 @@
         <v>1</v>
       </c>
       <c r="B437" s="39" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C437" s="40"/>
       <c r="D437" s="41"/>
@@ -15307,7 +15307,7 @@
         <v>11</v>
       </c>
       <c r="B438" s="41" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C438" s="40"/>
       <c r="D438" s="41"/>
@@ -15387,7 +15387,7 @@
         <v>4</v>
       </c>
       <c r="B440" s="41" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C440" s="40"/>
       <c r="D440" s="41"/>
@@ -15507,7 +15507,7 @@
         <v>76</v>
       </c>
       <c r="B443" s="41" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C443" s="40"/>
       <c r="D443" s="44"/>
@@ -15636,10 +15636,10 @@
     </row>
     <row r="446" spans="1:34">
       <c r="A446" s="46" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B446" s="46" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C446" s="47">
         <v>1</v>
@@ -15708,7 +15708,7 @@
         <v>12</v>
       </c>
       <c r="I447" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J447" s="46"/>
       <c r="K447" s="46"/>
@@ -15738,10 +15738,10 @@
     </row>
     <row r="448" spans="1:34">
       <c r="A448" s="46" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B448" s="46" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C448" s="47">
         <v>0.14285714285714285</v>
@@ -15788,10 +15788,10 @@
     </row>
     <row r="449" spans="1:34">
       <c r="A449" s="46" t="s">
+        <v>454</v>
+      </c>
+      <c r="B449" s="46" t="s">
         <v>455</v>
-      </c>
-      <c r="B449" s="46" t="s">
-        <v>456</v>
       </c>
       <c r="C449" s="47">
         <v>0.14285714285714285</v>
@@ -15838,10 +15838,10 @@
     </row>
     <row r="450" spans="1:34">
       <c r="A450" s="46" t="s">
+        <v>456</v>
+      </c>
+      <c r="B450" s="46" t="s">
         <v>457</v>
-      </c>
-      <c r="B450" s="46" t="s">
-        <v>458</v>
       </c>
       <c r="C450" s="47">
         <v>0.14285714285714285</v>
@@ -15888,10 +15888,10 @@
     </row>
     <row r="451" spans="1:34">
       <c r="A451" s="46" t="s">
+        <v>460</v>
+      </c>
+      <c r="B451" s="46" t="s">
         <v>461</v>
-      </c>
-      <c r="B451" s="46" t="s">
-        <v>462</v>
       </c>
       <c r="C451" s="47">
         <v>0.14285714285714285</v>
@@ -15938,10 +15938,10 @@
     </row>
     <row r="452" spans="1:34">
       <c r="A452" s="46" t="s">
+        <v>462</v>
+      </c>
+      <c r="B452" s="46" t="s">
         <v>463</v>
-      </c>
-      <c r="B452" s="46" t="s">
-        <v>464</v>
       </c>
       <c r="C452" s="47">
         <v>0.14285714285714285</v>
@@ -15988,10 +15988,10 @@
     </row>
     <row r="453" spans="1:34">
       <c r="A453" s="46" t="s">
+        <v>464</v>
+      </c>
+      <c r="B453" s="46" t="s">
         <v>465</v>
-      </c>
-      <c r="B453" s="46" t="s">
-        <v>466</v>
       </c>
       <c r="C453" s="47">
         <v>0.14285714285714285</v>
@@ -16010,7 +16010,7 @@
         <v>12</v>
       </c>
       <c r="I453" s="46" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="J453" s="46"/>
       <c r="K453" s="46"/>
@@ -16040,10 +16040,10 @@
     </row>
     <row r="454" spans="1:34">
       <c r="A454" s="46" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B454" s="46" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C454" s="47">
         <v>0.14285714285714285</v>
@@ -16129,7 +16129,7 @@
         <v>1</v>
       </c>
       <c r="B456" s="39" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C456" s="40"/>
       <c r="D456" s="41"/>
@@ -16169,7 +16169,7 @@
         <v>11</v>
       </c>
       <c r="B457" s="41" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C457" s="40"/>
       <c r="D457" s="41"/>
@@ -16249,7 +16249,7 @@
         <v>4</v>
       </c>
       <c r="B459" s="41" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C459" s="40"/>
       <c r="D459" s="41"/>
@@ -16369,7 +16369,7 @@
         <v>76</v>
       </c>
       <c r="B462" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C462" s="40"/>
       <c r="D462" s="44"/>
@@ -16498,10 +16498,10 @@
     </row>
     <row r="465" spans="1:34">
       <c r="A465" s="46" t="s">
+        <v>456</v>
+      </c>
+      <c r="B465" s="46" t="s">
         <v>457</v>
-      </c>
-      <c r="B465" s="46" t="s">
-        <v>458</v>
       </c>
       <c r="C465" s="47">
         <v>1</v>
@@ -16713,7 +16713,7 @@
         <v>1</v>
       </c>
       <c r="B470" s="37" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="471" spans="1:34">
@@ -16737,7 +16737,7 @@
         <v>4</v>
       </c>
       <c r="B473" s="55" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="474" spans="1:34">
@@ -16745,7 +16745,7 @@
         <v>76</v>
       </c>
       <c r="B474" s="18" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="475" spans="1:34">
@@ -16766,7 +16766,7 @@
     </row>
     <row r="477" spans="1:34">
       <c r="A477" s="42" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B477" s="31">
         <f>14.9/(1-B478)</f>
@@ -16775,7 +16775,7 @@
     </row>
     <row r="478" spans="1:34">
       <c r="A478" s="42" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B478" s="56">
         <v>0.14000000000000001</v>
@@ -16814,7 +16814,7 @@
     </row>
     <row r="481" spans="1:8" ht="15.75">
       <c r="A481" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B481" s="18">
         <v>1</v>
@@ -16826,7 +16826,7 @@
         <v>13</v>
       </c>
       <c r="E481" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F481" t="s">
         <v>18</v>
@@ -16835,7 +16835,7 @@
         <v>74</v>
       </c>
       <c r="H481" s="55" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="482" spans="1:8">
@@ -16855,7 +16855,7 @@
         <v>15</v>
       </c>
       <c r="G482" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="483" spans="1:8">
@@ -16875,12 +16875,12 @@
         <v>15</v>
       </c>
       <c r="G483" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="484" spans="1:8">
       <c r="A484" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B484" s="18">
         <v>8.9499999999999996E-3</v>
@@ -16892,21 +16892,21 @@
         <v>13</v>
       </c>
       <c r="E484" t="s">
+        <v>305</v>
+      </c>
+      <c r="F484" t="s">
+        <v>12</v>
+      </c>
+      <c r="G484" t="s">
         <v>306</v>
       </c>
-      <c r="F484" t="s">
-        <v>12</v>
-      </c>
-      <c r="G484" t="s">
+      <c r="H484" t="s">
         <v>307</v>
-      </c>
-      <c r="H484" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="485" spans="1:8">
       <c r="A485" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B485" s="18">
         <v>3.382384E-3</v>
@@ -16918,16 +16918,16 @@
         <v>13</v>
       </c>
       <c r="E485" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F485" t="s">
         <v>12</v>
       </c>
       <c r="G485" t="s">
+        <v>309</v>
+      </c>
+      <c r="H485" t="s">
         <v>310</v>
-      </c>
-      <c r="H485" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="486" spans="1:8">
@@ -16944,13 +16944,13 @@
         <v>13</v>
       </c>
       <c r="E486" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F486" t="s">
         <v>12</v>
       </c>
       <c r="G486" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H486" t="s">
         <v>234</v>
@@ -16958,7 +16958,7 @@
     </row>
     <row r="487" spans="1:8">
       <c r="A487" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B487" s="18">
         <f>0.00179/1000</f>
@@ -16971,21 +16971,21 @@
         <v>13</v>
       </c>
       <c r="E487" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F487" t="s">
         <v>12</v>
       </c>
       <c r="G487" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H487" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="488" spans="1:8">
       <c r="A488" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B488" s="18">
         <f>986/1000000</f>
@@ -17001,15 +17001,15 @@
         <v>12</v>
       </c>
       <c r="G488" t="s">
+        <v>314</v>
+      </c>
+      <c r="H488" t="s">
         <v>315</v>
-      </c>
-      <c r="H488" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="489" spans="1:8">
       <c r="A489" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B489" s="18">
         <v>5.3699999999999989E-3</v>
@@ -17021,21 +17021,21 @@
         <v>13</v>
       </c>
       <c r="E489" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F489" t="s">
         <v>12</v>
       </c>
       <c r="G489" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H489" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="490" spans="1:8">
       <c r="A490" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B490" s="18">
         <v>5.3699999999999989E-3</v>
@@ -17047,21 +17047,21 @@
         <v>13</v>
       </c>
       <c r="E490" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F490" t="s">
         <v>12</v>
       </c>
       <c r="G490" t="s">
+        <v>318</v>
+      </c>
+      <c r="H490" t="s">
         <v>319</v>
-      </c>
-      <c r="H490" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="491" spans="1:8">
       <c r="A491" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B491" s="18">
         <v>2.3269999999999996E-2</v>
@@ -17073,21 +17073,21 @@
         <v>13</v>
       </c>
       <c r="E491" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F491" t="s">
         <v>12</v>
       </c>
       <c r="G491" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H491" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="492" spans="1:8">
       <c r="A492" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B492" s="18">
         <f>0.01295781*43</f>
@@ -17100,21 +17100,21 @@
         <v>46</v>
       </c>
       <c r="E492" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F492" t="s">
         <v>12</v>
       </c>
       <c r="G492" t="s">
+        <v>323</v>
+      </c>
+      <c r="H492" t="s">
         <v>324</v>
-      </c>
-      <c r="H492" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="493" spans="1:8">
       <c r="A493" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B493" s="18">
         <v>7.464300000000001E-3</v>
@@ -17126,13 +17126,13 @@
         <v>19</v>
       </c>
       <c r="E493" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F493" t="s">
         <v>12</v>
       </c>
       <c r="G493" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H493" t="s">
         <v>43</v>
@@ -17140,7 +17140,7 @@
     </row>
     <row r="494" spans="1:8">
       <c r="A494" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B494" s="18">
         <v>1.9407179999999997E-3</v>
@@ -17152,13 +17152,13 @@
         <v>19</v>
       </c>
       <c r="E494" t="s">
+        <v>326</v>
+      </c>
+      <c r="F494" t="s">
+        <v>12</v>
+      </c>
+      <c r="G494" t="s">
         <v>327</v>
-      </c>
-      <c r="F494" t="s">
-        <v>12</v>
-      </c>
-      <c r="G494" t="s">
-        <v>328</v>
       </c>
       <c r="H494" t="s">
         <v>43</v>
@@ -17166,7 +17166,7 @@
     </row>
     <row r="495" spans="1:8">
       <c r="A495" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B495" s="18">
         <v>3.923859E-3</v>
@@ -17178,21 +17178,21 @@
         <v>13</v>
       </c>
       <c r="E495" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F495" t="s">
         <v>12</v>
       </c>
       <c r="G495" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H495" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="496" spans="1:8">
       <c r="A496" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B496" s="18">
         <f>17.9*(1-B478)</f>
@@ -17202,13 +17202,13 @@
         <v>46</v>
       </c>
       <c r="E496" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F496" t="s">
         <v>15</v>
       </c>
       <c r="G496" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="497" spans="1:7">
@@ -17228,12 +17228,12 @@
         <v>15</v>
       </c>
       <c r="G497" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="498" spans="1:7">
       <c r="A498" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B498" s="18">
         <f>1/(7129/10000)</f>
@@ -17249,12 +17249,12 @@
         <v>15</v>
       </c>
       <c r="G498" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="499" spans="1:7">
       <c r="A499" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B499" s="18">
         <f>1/(7129/10000)</f>
@@ -17270,12 +17270,12 @@
         <v>15</v>
       </c>
       <c r="G499" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="500" spans="1:7">
       <c r="A500" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B500" s="18">
         <f>1/(7129/10000)</f>
@@ -17291,7 +17291,7 @@
         <v>15</v>
       </c>
       <c r="G500" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="501" spans="1:7">
@@ -17311,7 +17311,7 @@
         <v>15</v>
       </c>
       <c r="G501" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="502" spans="1:7">
@@ -17331,12 +17331,12 @@
         <v>15</v>
       </c>
       <c r="G502" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="503" spans="1:7">
       <c r="A503" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B503" s="18">
         <v>1.0182310000000001E-3</v>
@@ -17351,12 +17351,12 @@
         <v>15</v>
       </c>
       <c r="G503" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="504" spans="1:7">
       <c r="A504" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B504" s="18">
         <f>B506/2</f>
@@ -17372,12 +17372,12 @@
         <v>15</v>
       </c>
       <c r="G504" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="505" spans="1:7">
       <c r="A505" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B505" s="18">
         <f>B506/2</f>
@@ -17393,12 +17393,12 @@
         <v>15</v>
       </c>
       <c r="G505" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="506" spans="1:7">
       <c r="A506" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B506" s="18">
         <v>0.95982162650602398</v>
@@ -17413,12 +17413,12 @@
         <v>15</v>
       </c>
       <c r="G506" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="507" spans="1:7">
       <c r="A507" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B507" s="18">
         <v>1.0107999999999999E-6</v>
@@ -17427,18 +17427,18 @@
         <v>13</v>
       </c>
       <c r="E507" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F507" t="s">
         <v>15</v>
       </c>
       <c r="G507" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="508" spans="1:7">
       <c r="A508" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B508" s="18">
         <v>6.1366999999999996E-7</v>
@@ -17447,18 +17447,18 @@
         <v>13</v>
       </c>
       <c r="E508" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F508" t="s">
         <v>15</v>
       </c>
       <c r="G508" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="509" spans="1:7">
       <c r="A509" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B509" s="18">
         <v>4.8131000000000003E-9</v>
@@ -17467,18 +17467,18 @@
         <v>13</v>
       </c>
       <c r="E509" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F509" t="s">
         <v>15</v>
       </c>
       <c r="G509" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="510" spans="1:7">
       <c r="A510" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B510" s="18">
         <v>6.4977000000000003E-7</v>
@@ -17487,18 +17487,18 @@
         <v>13</v>
       </c>
       <c r="E510" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F510" t="s">
         <v>15</v>
       </c>
       <c r="G510" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="511" spans="1:7">
       <c r="A511" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B511" s="18">
         <v>-1.5040999999999999E-6</v>
@@ -17507,18 +17507,18 @@
         <v>13</v>
       </c>
       <c r="E511" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F511" t="s">
         <v>15</v>
       </c>
       <c r="G511" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="512" spans="1:7">
       <c r="A512" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B512" s="18">
         <v>1.2032999999999999E-7</v>
@@ -17527,18 +17527,18 @@
         <v>13</v>
       </c>
       <c r="E512" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F512" t="s">
         <v>15</v>
       </c>
       <c r="G512" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="513" spans="1:7">
       <c r="A513" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B513" s="18">
         <v>2.4787000000000001E-6</v>
@@ -17547,18 +17547,18 @@
         <v>13</v>
       </c>
       <c r="E513" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F513" t="s">
         <v>15</v>
       </c>
       <c r="G513" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="514" spans="1:7">
       <c r="A514" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B514" s="18">
         <v>1.0829E-7</v>
@@ -17567,18 +17567,18 @@
         <v>13</v>
       </c>
       <c r="E514" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F514" t="s">
         <v>15</v>
       </c>
       <c r="G514" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="515" spans="1:7">
       <c r="A515" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B515" s="18">
         <v>1.0107999999999999E-6</v>
@@ -17587,18 +17587,18 @@
         <v>13</v>
       </c>
       <c r="E515" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F515" t="s">
         <v>15</v>
       </c>
       <c r="G515" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="516" spans="1:7">
       <c r="A516" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B516" s="18">
         <v>2.4065000000000001E-8</v>
@@ -17607,18 +17607,18 @@
         <v>13</v>
       </c>
       <c r="E516" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F516" t="s">
         <v>15</v>
       </c>
       <c r="G516" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="517" spans="1:7">
       <c r="A517" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B517" s="18">
         <v>-3.2893999999999998E-7</v>
@@ -17627,18 +17627,18 @@
         <v>13</v>
       </c>
       <c r="E517" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F517" t="s">
         <v>15</v>
       </c>
       <c r="G517" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="518" spans="1:7">
       <c r="A518" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B518" s="18">
         <v>7.9416000000000001E-7</v>
@@ -17647,18 +17647,18 @@
         <v>13</v>
       </c>
       <c r="E518" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F518" t="s">
         <v>15</v>
       </c>
       <c r="G518" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="519" spans="1:7">
       <c r="A519" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B519" s="18">
         <v>4.1393000000000003E-6</v>
@@ -17667,18 +17667,18 @@
         <v>13</v>
       </c>
       <c r="E519" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F519" t="s">
         <v>15</v>
       </c>
       <c r="G519" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="520" spans="1:7">
       <c r="A520" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B520" s="18">
         <v>5.0537999999999999E-8</v>
@@ -17687,18 +17687,18 @@
         <v>13</v>
       </c>
       <c r="E520" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F520" t="s">
         <v>15</v>
       </c>
       <c r="G520" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="521" spans="1:7">
       <c r="A521" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B521" s="18">
         <v>-5.9000999999999996E-6</v>
@@ -17707,18 +17707,18 @@
         <v>13</v>
       </c>
       <c r="E521" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F521" t="s">
         <v>15</v>
       </c>
       <c r="G521" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="522" spans="1:7">
       <c r="A522" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B522" s="18">
         <v>1.5643E-6</v>
@@ -17727,18 +17727,18 @@
         <v>13</v>
       </c>
       <c r="E522" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F522" t="s">
         <v>15</v>
       </c>
       <c r="G522" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="523" spans="1:7">
       <c r="A523" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B523" s="18">
         <v>2.6952999999999998E-6</v>
@@ -17747,18 +17747,18 @@
         <v>13</v>
       </c>
       <c r="E523" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F523" t="s">
         <v>15</v>
       </c>
       <c r="G523" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="524" spans="1:7">
       <c r="A524" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B524" s="18">
         <v>4.4454999999999997E-8</v>
@@ -17767,18 +17767,18 @@
         <v>13</v>
       </c>
       <c r="E524" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F524" t="s">
         <v>15</v>
       </c>
       <c r="G524" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="525" spans="1:7">
       <c r="A525" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B525" s="18">
         <v>3.6097999999999997E-8</v>
@@ -17787,18 +17787,18 @@
         <v>13</v>
       </c>
       <c r="E525" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F525" t="s">
         <v>15</v>
       </c>
       <c r="G525" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="526" spans="1:7">
       <c r="A526" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B526" s="18">
         <v>2.1659000000000001E-7</v>
@@ -17807,18 +17807,18 @@
         <v>13</v>
       </c>
       <c r="E526" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F526" t="s">
         <v>15</v>
       </c>
       <c r="G526" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="527" spans="1:7">
       <c r="A527" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B527" s="18">
         <v>-1.8835E-8</v>
@@ -17827,18 +17827,18 @@
         <v>13</v>
       </c>
       <c r="E527" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F527" t="s">
         <v>15</v>
       </c>
       <c r="G527" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="528" spans="1:7">
       <c r="A528" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B528" s="18">
         <v>4.2885E-5</v>
@@ -17847,18 +17847,18 @@
         <v>13</v>
       </c>
       <c r="E528" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F528" t="s">
         <v>15</v>
       </c>
       <c r="G528" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="529" spans="1:7">
       <c r="A529" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B529" s="18">
         <v>9.2460000000000006E-5</v>
@@ -17867,18 +17867,18 @@
         <v>13</v>
       </c>
       <c r="E529" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F529" t="s">
         <v>15</v>
       </c>
       <c r="G529" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="530" spans="1:7">
       <c r="A530" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B530" s="18">
         <v>5.0297000000000003E-6</v>
@@ -17887,18 +17887,18 @@
         <v>13</v>
       </c>
       <c r="E530" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F530" t="s">
         <v>15</v>
       </c>
       <c r="G530" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="531" spans="1:7">
       <c r="A531" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B531" s="18">
         <v>2.4306000000000001E-6</v>
@@ -17907,18 +17907,18 @@
         <v>13</v>
       </c>
       <c r="E531" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F531" t="s">
         <v>15</v>
       </c>
       <c r="G531" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="532" spans="1:7">
       <c r="A532" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B532" s="18">
         <v>1.7326999999999999E-6</v>
@@ -17927,18 +17927,18 @@
         <v>13</v>
       </c>
       <c r="E532" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F532" t="s">
         <v>15</v>
       </c>
       <c r="G532" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="533" spans="1:7">
       <c r="A533" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B533" s="18">
         <v>2.8878999999999998E-7</v>
@@ -17947,18 +17947,18 @@
         <v>13</v>
       </c>
       <c r="E533" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F533" t="s">
         <v>15</v>
       </c>
       <c r="G533" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="534" spans="1:7">
       <c r="A534" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B534" s="18">
         <v>1.9661999999999999E-5</v>
@@ -17967,18 +17967,18 @@
         <v>13</v>
       </c>
       <c r="E534" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F534" t="s">
         <v>15</v>
       </c>
       <c r="G534" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="535" spans="1:7">
       <c r="A535" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B535" s="18">
         <v>1.1911999999999999E-6</v>
@@ -17987,18 +17987,18 @@
         <v>13</v>
       </c>
       <c r="E535" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F535" t="s">
         <v>15</v>
       </c>
       <c r="G535" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="536" spans="1:7">
       <c r="A536" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B536" s="18">
         <v>1.9252000000000001E-7</v>
@@ -18007,18 +18007,18 @@
         <v>13</v>
       </c>
       <c r="E536" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F536" t="s">
         <v>15</v>
       </c>
       <c r="G536" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="537" spans="1:7">
       <c r="A537" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B537" s="18">
         <v>3.0442999999999998E-6</v>
@@ -18027,18 +18027,18 @@
         <v>13</v>
       </c>
       <c r="E537" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F537" t="s">
         <v>15</v>
       </c>
       <c r="G537" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="538" spans="1:7">
       <c r="A538" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B538" s="18">
         <v>4.8130999999999997E-6</v>
@@ -18047,18 +18047,18 @@
         <v>13</v>
       </c>
       <c r="E538" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F538" t="s">
         <v>15</v>
       </c>
       <c r="G538" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="539" spans="1:7">
       <c r="A539" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B539" s="18">
         <v>5.9441999999999998E-5</v>
@@ -18067,18 +18067,18 @@
         <v>13</v>
       </c>
       <c r="E539" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F539" t="s">
         <v>15</v>
       </c>
       <c r="G539" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="540" spans="1:7">
       <c r="A540" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B540" s="18">
         <v>3.3691999999999998E-7</v>
@@ -18087,18 +18087,18 @@
         <v>13</v>
       </c>
       <c r="E540" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F540" t="s">
         <v>15</v>
       </c>
       <c r="G540" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="541" spans="1:7">
       <c r="A541" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B541" s="18">
         <v>1.6846000000000001E-8</v>
@@ -18107,18 +18107,18 @@
         <v>13</v>
       </c>
       <c r="E541" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F541" t="s">
         <v>15</v>
       </c>
       <c r="G541" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="542" spans="1:7">
       <c r="A542" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B542" s="18">
         <v>5.7757E-7</v>
@@ -18127,18 +18127,18 @@
         <v>13</v>
       </c>
       <c r="E542" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F542" t="s">
         <v>15</v>
       </c>
       <c r="G542" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="543" spans="1:7">
       <c r="A543" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B543" s="18">
         <v>2.1658999999999999E-8</v>
@@ -18147,18 +18147,18 @@
         <v>13</v>
       </c>
       <c r="E543" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F543" t="s">
         <v>15</v>
       </c>
       <c r="G543" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="544" spans="1:7">
       <c r="A544" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B544" s="18">
         <v>3.6097999999999997E-8</v>
@@ -18167,18 +18167,18 @@
         <v>13</v>
       </c>
       <c r="E544" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F544" t="s">
         <v>15</v>
       </c>
       <c r="G544" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="545" spans="1:7">
       <c r="A545" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B545" s="18">
         <v>2.6472E-7</v>
@@ -18187,18 +18187,18 @@
         <v>13</v>
       </c>
       <c r="E545" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F545" t="s">
         <v>15</v>
       </c>
       <c r="G545" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="546" spans="1:7">
       <c r="A546" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B546" s="18">
         <v>1.2032999999999999E-7</v>
@@ -18207,18 +18207,18 @@
         <v>13</v>
       </c>
       <c r="E546" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F546" t="s">
         <v>15</v>
       </c>
       <c r="G546" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="547" spans="1:7">
       <c r="A547" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B547" s="18">
         <v>2.6436999999999998E-7</v>
@@ -18227,13 +18227,13 @@
         <v>13</v>
       </c>
       <c r="E547" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F547" t="s">
         <v>15</v>
       </c>
       <c r="G547" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="548" spans="1:7">
@@ -18253,7 +18253,7 @@
         <v>15</v>
       </c>
       <c r="G548" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="549" spans="1:7">
@@ -18273,7 +18273,7 @@
         <v>15</v>
       </c>
       <c r="G549" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="550" spans="1:7">
@@ -18287,18 +18287,18 @@
         <v>128</v>
       </c>
       <c r="E550" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F550" t="s">
         <v>15</v>
       </c>
       <c r="G550" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="551" spans="1:7">
       <c r="A551" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B551" s="18">
         <v>9.7541999999999995E-5</v>
@@ -18307,18 +18307,18 @@
         <v>13</v>
       </c>
       <c r="E551" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F551" t="s">
         <v>15</v>
       </c>
       <c r="G551" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="552" spans="1:7">
       <c r="A552" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B552" s="18">
         <v>7.5147999999999996E-6</v>
@@ -18327,18 +18327,18 @@
         <v>13</v>
       </c>
       <c r="E552" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F552" t="s">
         <v>15</v>
       </c>
       <c r="G552" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="553" spans="1:7">
       <c r="A553" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B553" s="18">
         <v>0</v>
@@ -18353,7 +18353,7 @@
         <v>15</v>
       </c>
       <c r="G553" s="57" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="554" spans="1:7" s="69" customFormat="1">
@@ -18364,7 +18364,7 @@
         <v>1</v>
       </c>
       <c r="B555" s="39" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="556" spans="1:7">
@@ -18448,7 +18448,7 @@
     </row>
     <row r="564" spans="1:9">
       <c r="A564" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B564" t="s">
         <v>244</v>
@@ -18584,7 +18584,7 @@
     </row>
     <row r="570" spans="1:9">
       <c r="A570" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B570" s="18" t="s">
         <v>195</v>
@@ -18596,7 +18596,7 @@
         <v>128</v>
       </c>
       <c r="G570" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H570" t="s">
         <v>12</v>
@@ -18604,10 +18604,10 @@
     </row>
     <row r="571" spans="1:9" s="41" customFormat="1">
       <c r="A571" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B571" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C571" s="65">
         <v>1</v>
@@ -18759,7 +18759,7 @@
         <v>1</v>
       </c>
       <c r="B579" s="39" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="580" spans="1:9">
@@ -18843,7 +18843,7 @@
     </row>
     <row r="588" spans="1:9">
       <c r="A588" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B588" t="s">
         <v>244</v>
@@ -18979,7 +18979,7 @@
     </row>
     <row r="594" spans="1:9">
       <c r="A594" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B594" s="18" t="s">
         <v>195</v>
@@ -18991,7 +18991,7 @@
         <v>128</v>
       </c>
       <c r="G594" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H594" t="s">
         <v>12</v>
@@ -18999,10 +18999,10 @@
     </row>
     <row r="595" spans="1:9" s="41" customFormat="1">
       <c r="A595" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B595" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C595" s="65">
         <v>1</v>
@@ -19171,10 +19171,10 @@
     </row>
     <row r="603" spans="1:9">
       <c r="A603" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B603" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B603" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C603">
         <v>1.2300000000000001E-4</v>
@@ -19194,10 +19194,10 @@
     </row>
     <row r="604" spans="1:9">
       <c r="A604" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B604" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B604" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C604">
         <v>6.9700000000000003E-4</v>
@@ -19217,10 +19217,10 @@
     </row>
     <row r="605" spans="1:9">
       <c r="A605" t="s">
+        <v>262</v>
+      </c>
+      <c r="B605" t="s">
         <v>263</v>
-      </c>
-      <c r="B605" t="s">
-        <v>264</v>
       </c>
       <c r="C605">
         <v>2.6400000000000001E-5</v>
@@ -19240,10 +19240,10 @@
     </row>
     <row r="606" spans="1:9">
       <c r="A606" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B606" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B606" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C606">
         <v>0</v>
@@ -19263,10 +19263,10 @@
     </row>
     <row r="607" spans="1:9">
       <c r="A607" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B607" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B607" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C607">
         <v>9.2899999999999995E-5</v>
@@ -19286,7 +19286,7 @@
     </row>
     <row r="608" spans="1:9">
       <c r="A608" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B608" s="47"/>
       <c r="C608">
@@ -19334,7 +19334,7 @@
         <v>1</v>
       </c>
       <c r="B611" s="39" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="612" spans="1:9">
@@ -19418,7 +19418,7 @@
     </row>
     <row r="620" spans="1:9">
       <c r="A620" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B620" t="s">
         <v>244</v>
@@ -19554,7 +19554,7 @@
     </row>
     <row r="626" spans="1:9">
       <c r="A626" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B626" s="18" t="s">
         <v>195</v>
@@ -19566,7 +19566,7 @@
         <v>128</v>
       </c>
       <c r="G626" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H626" t="s">
         <v>12</v>
@@ -19574,10 +19574,10 @@
     </row>
     <row r="627" spans="1:9" s="41" customFormat="1">
       <c r="A627" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B627" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C627" s="65">
         <v>1</v>
@@ -19746,10 +19746,10 @@
     </row>
     <row r="635" spans="1:9">
       <c r="A635" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B635" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B635" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C635">
         <v>0</v>
@@ -19769,10 +19769,10 @@
     </row>
     <row r="636" spans="1:9">
       <c r="A636" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B636" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B636" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C636">
         <v>0</v>
@@ -19792,10 +19792,10 @@
     </row>
     <row r="637" spans="1:9">
       <c r="A637" t="s">
+        <v>262</v>
+      </c>
+      <c r="B637" t="s">
         <v>263</v>
-      </c>
-      <c r="B637" t="s">
-        <v>264</v>
       </c>
       <c r="C637">
         <v>0</v>
@@ -19815,10 +19815,10 @@
     </row>
     <row r="638" spans="1:9">
       <c r="A638" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B638" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B638" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C638">
         <v>0</v>
@@ -19838,10 +19838,10 @@
     </row>
     <row r="639" spans="1:9">
       <c r="A639" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B639" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B639" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C639">
         <v>0</v>
@@ -19861,7 +19861,7 @@
     </row>
     <row r="640" spans="1:9">
       <c r="A640" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B640" s="47"/>
       <c r="C640">
@@ -19909,7 +19909,7 @@
         <v>1</v>
       </c>
       <c r="B643" s="39" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="644" spans="1:9">
@@ -19993,7 +19993,7 @@
     </row>
     <row r="652" spans="1:9">
       <c r="A652" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B652" t="s">
         <v>244</v>
@@ -20129,7 +20129,7 @@
     </row>
     <row r="658" spans="1:9">
       <c r="A658" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B658" s="18" t="s">
         <v>195</v>
@@ -20141,7 +20141,7 @@
         <v>128</v>
       </c>
       <c r="G658" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H658" t="s">
         <v>12</v>
@@ -20149,10 +20149,10 @@
     </row>
     <row r="659" spans="1:9" s="41" customFormat="1">
       <c r="A659" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B659" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C659" s="65">
         <v>1</v>
@@ -20321,10 +20321,10 @@
     </row>
     <row r="667" spans="1:9">
       <c r="A667" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B667" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B667" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C667">
         <v>2.0799999999999999E-4</v>
@@ -20344,10 +20344,10 @@
     </row>
     <row r="668" spans="1:9">
       <c r="A668" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B668" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B668" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C668">
         <v>0</v>
@@ -20367,10 +20367,10 @@
     </row>
     <row r="669" spans="1:9">
       <c r="A669" t="s">
+        <v>262</v>
+      </c>
+      <c r="B669" t="s">
         <v>263</v>
-      </c>
-      <c r="B669" t="s">
-        <v>264</v>
       </c>
       <c r="C669">
         <v>3.98E-6</v>
@@ -20390,10 +20390,10 @@
     </row>
     <row r="670" spans="1:9">
       <c r="A670" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B670" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B670" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C670">
         <v>0</v>
@@ -20413,10 +20413,10 @@
     </row>
     <row r="671" spans="1:9">
       <c r="A671" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B671" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B671" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C671">
         <v>0</v>
@@ -20436,7 +20436,7 @@
     </row>
     <row r="672" spans="1:9">
       <c r="A672" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B672" s="47"/>
       <c r="C672">
@@ -20484,7 +20484,7 @@
         <v>1</v>
       </c>
       <c r="B675" s="39" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="676" spans="1:9">
@@ -20568,7 +20568,7 @@
     </row>
     <row r="684" spans="1:9">
       <c r="A684" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B684" t="s">
         <v>244</v>
@@ -20704,7 +20704,7 @@
     </row>
     <row r="690" spans="1:9">
       <c r="A690" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B690" s="18" t="s">
         <v>195</v>
@@ -20716,7 +20716,7 @@
         <v>128</v>
       </c>
       <c r="G690" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H690" t="s">
         <v>12</v>
@@ -20724,10 +20724,10 @@
     </row>
     <row r="691" spans="1:9" s="41" customFormat="1">
       <c r="A691" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B691" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C691" s="65">
         <v>1</v>
@@ -20896,10 +20896,10 @@
     </row>
     <row r="699" spans="1:9">
       <c r="A699" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B699" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B699" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C699">
         <v>0</v>
@@ -20919,10 +20919,10 @@
     </row>
     <row r="700" spans="1:9">
       <c r="A700" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B700" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B700" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C700">
         <v>0</v>
@@ -20942,10 +20942,10 @@
     </row>
     <row r="701" spans="1:9">
       <c r="A701" t="s">
+        <v>262</v>
+      </c>
+      <c r="B701" t="s">
         <v>263</v>
-      </c>
-      <c r="B701" t="s">
-        <v>264</v>
       </c>
       <c r="C701">
         <v>0</v>
@@ -20965,10 +20965,10 @@
     </row>
     <row r="702" spans="1:9">
       <c r="A702" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B702" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B702" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C702">
         <v>0</v>
@@ -20988,10 +20988,10 @@
     </row>
     <row r="703" spans="1:9">
       <c r="A703" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B703" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B703" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C703">
         <v>0</v>
@@ -21011,7 +21011,7 @@
     </row>
     <row r="704" spans="1:9">
       <c r="A704" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B704" s="47"/>
       <c r="C704">
@@ -21059,7 +21059,7 @@
         <v>1</v>
       </c>
       <c r="B707" s="39" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="708" spans="1:9">
@@ -21143,7 +21143,7 @@
     </row>
     <row r="716" spans="1:9">
       <c r="A716" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B716" t="s">
         <v>244</v>
@@ -21279,7 +21279,7 @@
     </row>
     <row r="722" spans="1:9">
       <c r="A722" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B722" s="18" t="s">
         <v>195</v>
@@ -21291,7 +21291,7 @@
         <v>128</v>
       </c>
       <c r="G722" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H722" t="s">
         <v>12</v>
@@ -21299,10 +21299,10 @@
     </row>
     <row r="723" spans="1:9" s="41" customFormat="1">
       <c r="A723" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B723" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C723" s="65">
         <v>1</v>
@@ -21454,7 +21454,7 @@
         <v>1</v>
       </c>
       <c r="B731" s="39" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="732" spans="1:9">
@@ -21538,7 +21538,7 @@
     </row>
     <row r="740" spans="1:9">
       <c r="A740" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B740" t="s">
         <v>244</v>
@@ -21674,7 +21674,7 @@
     </row>
     <row r="746" spans="1:9">
       <c r="A746" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B746" s="18" t="s">
         <v>195</v>
@@ -21686,7 +21686,7 @@
         <v>128</v>
       </c>
       <c r="G746" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H746" t="s">
         <v>12</v>
@@ -21694,10 +21694,10 @@
     </row>
     <row r="747" spans="1:9" s="41" customFormat="1">
       <c r="A747" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B747" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C747" s="65">
         <v>1</v>
@@ -21866,10 +21866,10 @@
     </row>
     <row r="755" spans="1:8">
       <c r="A755" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B755" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B755" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C755">
         <v>1.2300000000000001E-4</v>
@@ -21889,10 +21889,10 @@
     </row>
     <row r="756" spans="1:8">
       <c r="A756" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B756" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B756" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C756">
         <v>6.9700000000000003E-4</v>
@@ -21912,10 +21912,10 @@
     </row>
     <row r="757" spans="1:8">
       <c r="A757" t="s">
+        <v>262</v>
+      </c>
+      <c r="B757" t="s">
         <v>263</v>
-      </c>
-      <c r="B757" t="s">
-        <v>264</v>
       </c>
       <c r="C757">
         <v>2.6400000000000001E-5</v>
@@ -21935,10 +21935,10 @@
     </row>
     <row r="758" spans="1:8">
       <c r="A758" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B758" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B758" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C758">
         <v>0</v>
@@ -21958,10 +21958,10 @@
     </row>
     <row r="759" spans="1:8">
       <c r="A759" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B759" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B759" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C759">
         <v>9.2899999999999995E-5</v>
@@ -21981,7 +21981,7 @@
     </row>
     <row r="760" spans="1:8">
       <c r="A760" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B760" s="47"/>
       <c r="C760">
@@ -22029,7 +22029,7 @@
         <v>1</v>
       </c>
       <c r="B763" s="39" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="764" spans="1:8">
@@ -22113,7 +22113,7 @@
     </row>
     <row r="772" spans="1:9">
       <c r="A772" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B772" t="s">
         <v>244</v>
@@ -22249,7 +22249,7 @@
     </row>
     <row r="778" spans="1:9">
       <c r="A778" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B778" s="18" t="s">
         <v>195</v>
@@ -22261,7 +22261,7 @@
         <v>128</v>
       </c>
       <c r="G778" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H778" t="s">
         <v>12</v>
@@ -22269,10 +22269,10 @@
     </row>
     <row r="779" spans="1:9" s="41" customFormat="1">
       <c r="A779" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B779" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C779" s="65">
         <v>1</v>
@@ -22441,10 +22441,10 @@
     </row>
     <row r="787" spans="1:8">
       <c r="A787" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B787" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B787" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C787">
         <v>0</v>
@@ -22464,10 +22464,10 @@
     </row>
     <row r="788" spans="1:8">
       <c r="A788" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B788" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B788" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C788">
         <v>0</v>
@@ -22487,10 +22487,10 @@
     </row>
     <row r="789" spans="1:8">
       <c r="A789" t="s">
+        <v>262</v>
+      </c>
+      <c r="B789" t="s">
         <v>263</v>
-      </c>
-      <c r="B789" t="s">
-        <v>264</v>
       </c>
       <c r="C789">
         <v>0</v>
@@ -22510,10 +22510,10 @@
     </row>
     <row r="790" spans="1:8">
       <c r="A790" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B790" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B790" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C790">
         <v>0</v>
@@ -22533,10 +22533,10 @@
     </row>
     <row r="791" spans="1:8">
       <c r="A791" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B791" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B791" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C791">
         <v>0</v>
@@ -22556,7 +22556,7 @@
     </row>
     <row r="792" spans="1:8">
       <c r="A792" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B792" s="47"/>
       <c r="C792">
@@ -22604,7 +22604,7 @@
         <v>1</v>
       </c>
       <c r="B795" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="796" spans="1:8">
@@ -22688,7 +22688,7 @@
     </row>
     <row r="804" spans="1:9">
       <c r="A804" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B804" t="s">
         <v>244</v>
@@ -22824,7 +22824,7 @@
     </row>
     <row r="810" spans="1:9">
       <c r="A810" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B810" s="18" t="s">
         <v>195</v>
@@ -22836,7 +22836,7 @@
         <v>128</v>
       </c>
       <c r="G810" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H810" t="s">
         <v>12</v>
@@ -22844,10 +22844,10 @@
     </row>
     <row r="811" spans="1:9" s="41" customFormat="1">
       <c r="A811" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B811" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C811" s="65">
         <v>1</v>
@@ -23016,10 +23016,10 @@
     </row>
     <row r="819" spans="1:9">
       <c r="A819" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B819" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B819" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C819">
         <v>2.0799999999999999E-4</v>
@@ -23039,10 +23039,10 @@
     </row>
     <row r="820" spans="1:9">
       <c r="A820" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B820" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B820" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C820">
         <v>0</v>
@@ -23062,10 +23062,10 @@
     </row>
     <row r="821" spans="1:9">
       <c r="A821" t="s">
+        <v>262</v>
+      </c>
+      <c r="B821" t="s">
         <v>263</v>
-      </c>
-      <c r="B821" t="s">
-        <v>264</v>
       </c>
       <c r="C821">
         <v>3.98E-6</v>
@@ -23085,10 +23085,10 @@
     </row>
     <row r="822" spans="1:9">
       <c r="A822" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B822" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B822" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C822">
         <v>0</v>
@@ -23108,10 +23108,10 @@
     </row>
     <row r="823" spans="1:9">
       <c r="A823" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B823" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B823" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C823">
         <v>0</v>
@@ -23131,7 +23131,7 @@
     </row>
     <row r="824" spans="1:9">
       <c r="A824" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B824" s="47"/>
       <c r="C824">
@@ -23179,7 +23179,7 @@
         <v>1</v>
       </c>
       <c r="B827" s="39" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="828" spans="1:9">
@@ -23264,7 +23264,7 @@
     </row>
     <row r="836" spans="1:9">
       <c r="A836" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B836" t="s">
         <v>244</v>
@@ -23400,7 +23400,7 @@
     </row>
     <row r="842" spans="1:9">
       <c r="A842" t="s">
-        <v>254</v>
+        <v>493</v>
       </c>
       <c r="B842" s="18" t="s">
         <v>195</v>
@@ -23412,7 +23412,7 @@
         <v>128</v>
       </c>
       <c r="G842" s="46" t="s">
-        <v>29</v>
+        <v>208</v>
       </c>
       <c r="H842" t="s">
         <v>12</v>
@@ -23420,10 +23420,10 @@
     </row>
     <row r="843" spans="1:9" s="41" customFormat="1">
       <c r="A843" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B843" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C843" s="65">
         <v>1</v>
@@ -23592,10 +23592,10 @@
     </row>
     <row r="851" spans="1:8">
       <c r="A851" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B851" s="46" t="s">
         <v>259</v>
-      </c>
-      <c r="B851" s="46" t="s">
-        <v>260</v>
       </c>
       <c r="C851">
         <v>0</v>
@@ -23615,10 +23615,10 @@
     </row>
     <row r="852" spans="1:8">
       <c r="A852" s="46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B852" s="46" t="s">
         <v>261</v>
-      </c>
-      <c r="B852" s="46" t="s">
-        <v>262</v>
       </c>
       <c r="C852">
         <v>0</v>
@@ -23638,10 +23638,10 @@
     </row>
     <row r="853" spans="1:8">
       <c r="A853" t="s">
+        <v>262</v>
+      </c>
+      <c r="B853" t="s">
         <v>263</v>
-      </c>
-      <c r="B853" t="s">
-        <v>264</v>
       </c>
       <c r="C853">
         <v>0</v>
@@ -23661,10 +23661,10 @@
     </row>
     <row r="854" spans="1:8">
       <c r="A854" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="B854" s="47" t="s">
         <v>265</v>
-      </c>
-      <c r="B854" s="47" t="s">
-        <v>266</v>
       </c>
       <c r="C854">
         <v>0</v>
@@ -23684,10 +23684,10 @@
     </row>
     <row r="855" spans="1:8">
       <c r="A855" s="46" t="s">
+        <v>266</v>
+      </c>
+      <c r="B855" s="47" t="s">
         <v>267</v>
-      </c>
-      <c r="B855" s="47" t="s">
-        <v>268</v>
       </c>
       <c r="C855">
         <v>0</v>
@@ -23707,7 +23707,7 @@
     </row>
     <row r="856" spans="1:8">
       <c r="A856" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B856" s="47"/>
       <c r="C856">
@@ -23755,7 +23755,7 @@
         <v>1</v>
       </c>
       <c r="B859" s="39" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="860" spans="1:8">
@@ -23784,7 +23784,7 @@
         <v>4</v>
       </c>
       <c r="B863" s="18" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="864" spans="1:8">
@@ -23800,7 +23800,7 @@
         <v>76</v>
       </c>
       <c r="B865" s="18" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="866" spans="1:21" ht="15.75">
@@ -23856,48 +23856,48 @@
         <v>11</v>
       </c>
       <c r="J867" s="42" t="s">
+        <v>385</v>
+      </c>
+      <c r="K867" s="42" t="s">
         <v>386</v>
       </c>
-      <c r="K867" s="42" t="s">
+      <c r="L867" s="42" t="s">
         <v>387</v>
       </c>
-      <c r="L867" s="42" t="s">
+      <c r="M867" s="42" t="s">
         <v>388</v>
       </c>
-      <c r="M867" s="42" t="s">
+      <c r="N867" s="42" t="s">
         <v>389</v>
       </c>
-      <c r="N867" s="42" t="s">
+      <c r="O867" s="42" t="s">
         <v>390</v>
       </c>
-      <c r="O867" s="42" t="s">
+      <c r="P867" s="42" t="s">
         <v>391</v>
       </c>
-      <c r="P867" s="42" t="s">
+      <c r="Q867" s="42" t="s">
         <v>392</v>
       </c>
-      <c r="Q867" s="42" t="s">
+      <c r="R867" s="42" t="s">
         <v>393</v>
       </c>
-      <c r="R867" s="42" t="s">
+      <c r="S867" s="42" t="s">
         <v>394</v>
       </c>
-      <c r="S867" s="42" t="s">
+      <c r="T867" s="42" t="s">
         <v>395</v>
       </c>
-      <c r="T867" s="42" t="s">
+      <c r="U867" s="42" t="s">
         <v>396</v>
-      </c>
-      <c r="U867" s="42" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="868" spans="1:21">
       <c r="A868" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B868" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C868">
         <v>1</v>
@@ -23912,18 +23912,18 @@
         <v>18</v>
       </c>
       <c r="I868" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="U868" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="869" spans="1:21">
       <c r="A869" t="s">
+        <v>398</v>
+      </c>
+      <c r="B869" t="s">
         <v>399</v>
-      </c>
-      <c r="B869" t="s">
-        <v>400</v>
       </c>
       <c r="C869">
         <v>2.8299989989246005E-7</v>
@@ -23938,7 +23938,7 @@
         <v>12</v>
       </c>
       <c r="I869" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J869">
         <v>2</v>
@@ -23973,10 +23973,10 @@
     </row>
     <row r="870" spans="1:21">
       <c r="A870" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B870" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C870">
         <v>1.9717499999999999</v>
@@ -23991,7 +23991,7 @@
         <v>12</v>
       </c>
       <c r="I870" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="871" spans="1:21">
@@ -24014,15 +24014,15 @@
         <v>12</v>
       </c>
       <c r="I871" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="872" spans="1:21">
       <c r="A872" t="s">
+        <v>400</v>
+      </c>
+      <c r="B872" t="s">
         <v>401</v>
-      </c>
-      <c r="B872" t="s">
-        <v>402</v>
       </c>
       <c r="C872">
         <v>5.9999993977199999E-5</v>
@@ -24037,7 +24037,7 @@
         <v>12</v>
       </c>
       <c r="I872" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J872">
         <v>2</v>
@@ -24072,10 +24072,10 @@
     </row>
     <row r="873" spans="1:21" s="41" customFormat="1">
       <c r="A873" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B873" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C873" s="65">
         <v>1</v>
@@ -24104,13 +24104,13 @@
         <v>128</v>
       </c>
       <c r="F874" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H874" t="s">
         <v>15</v>
       </c>
       <c r="I874" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="875" spans="1:21">
@@ -24131,7 +24131,7 @@
         <v>15</v>
       </c>
       <c r="I875" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="876" spans="1:21" s="69" customFormat="1">
@@ -24142,7 +24142,7 @@
         <v>1</v>
       </c>
       <c r="B877" s="39" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C877" s="40"/>
     </row>
@@ -24151,7 +24151,7 @@
         <v>11</v>
       </c>
       <c r="B878" s="41" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C878" s="40"/>
     </row>
@@ -24169,7 +24169,7 @@
         <v>4</v>
       </c>
       <c r="B880" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C880" s="40"/>
     </row>
@@ -24198,7 +24198,7 @@
         <v>76</v>
       </c>
       <c r="B883" s="41" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C883" s="40"/>
       <c r="D883" s="44"/>
@@ -24240,10 +24240,10 @@
     </row>
     <row r="886" spans="1:11" s="41" customFormat="1">
       <c r="A886" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B886" s="46" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C886" s="60">
         <v>1</v>
@@ -24265,10 +24265,10 @@
     </row>
     <row r="887" spans="1:11" s="41" customFormat="1">
       <c r="A887" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B887" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C887" s="60">
         <v>1</v>
@@ -24285,7 +24285,7 @@
         <v>12</v>
       </c>
       <c r="I887" s="46" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="J887" s="46"/>
       <c r="K887" s="46"/>
@@ -24319,10 +24319,10 @@
     </row>
     <row r="889" spans="1:11" s="41" customFormat="1">
       <c r="A889" t="s">
+        <v>258</v>
+      </c>
+      <c r="B889" t="s">
         <v>259</v>
-      </c>
-      <c r="B889" t="s">
-        <v>260</v>
       </c>
       <c r="C889" s="18">
         <v>2.8400000000000002E-4</v>
@@ -24346,10 +24346,10 @@
     </row>
     <row r="890" spans="1:11" s="41" customFormat="1">
       <c r="A890" t="s">
+        <v>406</v>
+      </c>
+      <c r="B890" t="s">
         <v>407</v>
-      </c>
-      <c r="B890" t="s">
-        <v>408</v>
       </c>
       <c r="C890" s="18">
         <v>3.0400000000000002E-4</v>
@@ -24373,10 +24373,10 @@
     </row>
     <row r="891" spans="1:11" s="41" customFormat="1">
       <c r="A891" t="s">
+        <v>260</v>
+      </c>
+      <c r="B891" t="s">
         <v>261</v>
-      </c>
-      <c r="B891" t="s">
-        <v>262</v>
       </c>
       <c r="C891" s="18">
         <v>8.2600000000000002E-5</v>
@@ -24400,10 +24400,10 @@
     </row>
     <row r="892" spans="1:11" s="41" customFormat="1">
       <c r="A892" t="s">
+        <v>408</v>
+      </c>
+      <c r="B892" t="s">
         <v>409</v>
-      </c>
-      <c r="B892" t="s">
-        <v>410</v>
       </c>
       <c r="C892" s="18">
         <v>8.2699999999999996E-11</v>
@@ -24427,10 +24427,10 @@
     </row>
     <row r="893" spans="1:11" s="41" customFormat="1">
       <c r="A893" t="s">
+        <v>410</v>
+      </c>
+      <c r="B893" t="s">
         <v>411</v>
-      </c>
-      <c r="B893" t="s">
-        <v>412</v>
       </c>
       <c r="C893" s="18">
         <v>7.4400000000000002E-10</v>
@@ -24454,10 +24454,10 @@
     </row>
     <row r="894" spans="1:11" s="41" customFormat="1">
       <c r="A894" t="s">
+        <v>412</v>
+      </c>
+      <c r="B894" t="s">
         <v>413</v>
-      </c>
-      <c r="B894" t="s">
-        <v>414</v>
       </c>
       <c r="C894" s="18">
         <v>3.3099999999999999E-10</v>
@@ -24508,10 +24508,10 @@
     </row>
     <row r="896" spans="1:11" s="41" customFormat="1">
       <c r="A896" t="s">
+        <v>414</v>
+      </c>
+      <c r="B896" t="s">
         <v>415</v>
-      </c>
-      <c r="B896" t="s">
-        <v>416</v>
       </c>
       <c r="C896" s="18">
         <v>5.7899999999999997E-10</v>
@@ -24535,10 +24535,10 @@
     </row>
     <row r="897" spans="1:11" s="41" customFormat="1">
       <c r="A897" t="s">
+        <v>416</v>
+      </c>
+      <c r="B897" t="s">
         <v>417</v>
-      </c>
-      <c r="B897" t="s">
-        <v>418</v>
       </c>
       <c r="C897" s="18">
         <v>-2.2699999999999999E-4</v>
@@ -24587,7 +24587,7 @@
     </row>
     <row r="899" spans="1:11" s="41" customFormat="1">
       <c r="A899" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B899"/>
       <c r="C899" s="18">
@@ -24612,7 +24612,7 @@
     </row>
     <row r="900" spans="1:11" s="41" customFormat="1">
       <c r="A900" s="46" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B900" s="46"/>
       <c r="C900" s="44">
@@ -24643,7 +24643,7 @@
         <v>1</v>
       </c>
       <c r="B902" s="63" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C902" s="40"/>
     </row>
@@ -24652,7 +24652,7 @@
         <v>11</v>
       </c>
       <c r="B903" s="46" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="904" spans="1:11" s="41" customFormat="1">
@@ -24669,7 +24669,7 @@
         <v>4</v>
       </c>
       <c r="B905" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C905" s="40"/>
     </row>
@@ -24698,7 +24698,7 @@
         <v>76</v>
       </c>
       <c r="B908" s="41" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C908" s="40"/>
       <c r="D908" s="44"/>
@@ -24740,10 +24740,10 @@
     </row>
     <row r="911" spans="1:11" s="41" customFormat="1">
       <c r="A911" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B911" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C911" s="60">
         <v>1</v>
@@ -24785,7 +24785,7 @@
         <v>12</v>
       </c>
       <c r="I912" s="41" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="913" spans="1:9" s="69" customFormat="1">
@@ -24796,7 +24796,7 @@
         <v>1</v>
       </c>
       <c r="B914" s="63" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C914" s="40"/>
     </row>
@@ -24805,7 +24805,7 @@
         <v>11</v>
       </c>
       <c r="B915" s="46" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="916" spans="1:9" s="41" customFormat="1">
@@ -24822,7 +24822,7 @@
         <v>4</v>
       </c>
       <c r="B917" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C917" s="40"/>
       <c r="D917" s="44"/>
@@ -24890,10 +24890,10 @@
     </row>
     <row r="923" spans="1:9" s="41" customFormat="1">
       <c r="A923" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B923" s="46" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C923" s="65">
         <v>1</v>
@@ -24913,10 +24913,10 @@
     </row>
     <row r="924" spans="1:9">
       <c r="A924" s="38" t="s">
+        <v>433</v>
+      </c>
+      <c r="B924" s="46" t="s">
         <v>434</v>
-      </c>
-      <c r="B924" s="46" t="s">
-        <v>435</v>
       </c>
       <c r="C924" s="66">
         <f>0.00593*34.72</f>
@@ -24933,7 +24933,7 @@
         <v>12</v>
       </c>
       <c r="I924" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="925" spans="1:9">
@@ -24956,7 +24956,7 @@
         <v>12</v>
       </c>
       <c r="I925" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="926" spans="1:9">
@@ -24980,7 +24980,7 @@
         <v>15</v>
       </c>
       <c r="I926" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="927" spans="1:9">
@@ -25004,7 +25004,7 @@
         <v>15</v>
       </c>
       <c r="I927" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="928" spans="1:9" s="69" customFormat="1">
@@ -25015,7 +25015,7 @@
         <v>1</v>
       </c>
       <c r="B929" s="63" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C929" s="40"/>
     </row>
@@ -25024,7 +25024,7 @@
         <v>11</v>
       </c>
       <c r="B930" s="46" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="931" spans="1:9" s="41" customFormat="1">
@@ -25041,7 +25041,7 @@
         <v>4</v>
       </c>
       <c r="B932" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C932" s="40"/>
     </row>
@@ -25110,10 +25110,10 @@
     </row>
     <row r="938" spans="1:9" s="41" customFormat="1">
       <c r="A938" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B938" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C938" s="65">
         <v>1</v>
@@ -25133,10 +25133,10 @@
     </row>
     <row r="939" spans="1:9">
       <c r="A939" s="38" t="s">
+        <v>433</v>
+      </c>
+      <c r="B939" s="46" t="s">
         <v>434</v>
-      </c>
-      <c r="B939" s="46" t="s">
-        <v>435</v>
       </c>
       <c r="C939" s="66">
         <f>0.00593*35.8</f>
@@ -25153,7 +25153,7 @@
         <v>12</v>
       </c>
       <c r="I939" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="940" spans="1:9">
@@ -25176,7 +25176,7 @@
         <v>12</v>
       </c>
       <c r="I940" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="941" spans="1:9">
@@ -25200,7 +25200,7 @@
         <v>15</v>
       </c>
       <c r="I941" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="942" spans="1:9" s="69" customFormat="1">
@@ -25211,7 +25211,7 @@
         <v>1</v>
       </c>
       <c r="B943" s="63" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C943" s="40"/>
       <c r="D943" s="41"/>
@@ -25226,7 +25226,7 @@
         <v>11</v>
       </c>
       <c r="B944" s="46" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C944" s="41"/>
       <c r="D944" s="41"/>
@@ -25353,7 +25353,7 @@
     </row>
     <row r="952" spans="1:9">
       <c r="A952" s="46" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B952" s="46" t="s">
         <v>162</v>
@@ -25375,10 +25375,10 @@
     </row>
     <row r="953" spans="1:9">
       <c r="A953" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B953" s="18" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C953">
         <v>0.1764792</v>
@@ -25393,12 +25393,12 @@
         <v>12</v>
       </c>
       <c r="I953" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="954" spans="1:9">
       <c r="A954" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B954" s="18" t="s">
         <v>162</v>
@@ -25418,7 +25418,7 @@
     </row>
     <row r="955" spans="1:9">
       <c r="A955" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B955" s="18" t="s">
         <v>162</v>
@@ -25438,7 +25438,7 @@
     </row>
     <row r="956" spans="1:9">
       <c r="A956" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B956" s="18" t="s">
         <v>162</v>
@@ -25458,7 +25458,7 @@
     </row>
     <row r="957" spans="1:9">
       <c r="A957" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B957" s="18" t="s">
         <v>162</v>
@@ -25478,7 +25478,7 @@
     </row>
     <row r="958" spans="1:9">
       <c r="A958" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B958" s="18" t="s">
         <v>162</v>
@@ -25498,7 +25498,7 @@
     </row>
     <row r="959" spans="1:9">
       <c r="A959" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B959" s="18" t="s">
         <v>162</v>
@@ -25518,7 +25518,7 @@
     </row>
     <row r="960" spans="1:9">
       <c r="A960" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B960" s="18" t="s">
         <v>162</v>
@@ -25557,7 +25557,7 @@
         <v>15</v>
       </c>
       <c r="I961" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="962" spans="1:9">
@@ -25581,12 +25581,12 @@
         <v>15</v>
       </c>
       <c r="I962" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="963" spans="1:9">
       <c r="A963" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C963" s="18">
         <v>5.74128E-5</v>
@@ -25605,7 +25605,7 @@
         <v>15</v>
       </c>
       <c r="I963" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="964" spans="1:9">
@@ -25628,7 +25628,7 @@
         <v>15</v>
       </c>
       <c r="I964" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="965" spans="1:9">
@@ -25652,7 +25652,7 @@
         <v>15</v>
       </c>
       <c r="I965" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="966" spans="1:9">
@@ -25676,7 +25676,7 @@
         <v>15</v>
       </c>
       <c r="I966" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="967" spans="1:9">
@@ -25695,7 +25695,7 @@
         <v>1</v>
       </c>
       <c r="B968" s="63" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C968" s="40"/>
       <c r="D968" s="41"/>
@@ -25710,7 +25710,7 @@
         <v>11</v>
       </c>
       <c r="B969" s="46" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C969" s="41"/>
       <c r="D969" s="41"/>
@@ -25785,7 +25785,7 @@
         <v>76</v>
       </c>
       <c r="B974" s="41" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C974" s="40"/>
       <c r="D974" s="44"/>
@@ -25839,7 +25839,7 @@
     </row>
     <row r="977" spans="1:9">
       <c r="A977" s="46" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B977" s="46" t="s">
         <v>244</v>
@@ -25861,7 +25861,7 @@
     </row>
     <row r="978" spans="1:9">
       <c r="A978" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B978" s="46" t="s">
         <v>244</v>

</xml_diff>

<commit_message>
Added pyrogasification of wood and low pressure ng market
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1312" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{444287BB-FE43-4137-874D-06C43648E757}"/>
+  <xr:revisionPtr revIDLastSave="1415" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B146A451-61E5-42FB-B882-1FB2960E6CB1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1338,9 +1338,6 @@
     <t>biomethane AD transport</t>
   </si>
   <si>
-    <t>Average transportation of biomethane from anaerobic digestion (AD) in France. Leaks are calcualted considering the average market for upgrading technologies, which remain constant over time and scenarios. While correctly representing leaks for the upgrading mix, it can udnerestimate or overestimate transportation losses of individual upgrading technologies due to the different methane purities. Transportation is added to the individual AD production pathways because of implementation easiness in the user-defined scenario markets.</t>
-  </si>
-  <si>
     <t>market for heat, central or small-scale, biomethane</t>
   </si>
   <si>
@@ -1362,9 +1359,6 @@
     <t xml:space="preserve">Production of biogas from the treatment of sewage sludge. Absorbed biogenic carbon is included to ensure carbon neutrality in </t>
   </si>
   <si>
-    <t xml:space="preserve">Production of biogas from animal manure. Absorbed biogenic carbon is included to ensure carbon neutrality in </t>
-  </si>
-  <si>
     <t xml:space="preserve">Production of biogas from agricultural residues. Absorbed biogenic carbon is included to ensure carbon neutrality in </t>
   </si>
   <si>
@@ -1485,15 +1479,9 @@
     <t>0.49%/MJ supplied (Bussa et al., 2022)</t>
   </si>
   <si>
-    <t>0.1% of emission rate (Bussa et al., 2022)</t>
-  </si>
-  <si>
     <t>market for natural gas, high pressure</t>
   </si>
   <si>
-    <t>0.49%/MJ supplied (Bussa et al., 2022). CH4 LHV = 35.8 MJ</t>
-  </si>
-  <si>
     <t>biomethane import</t>
   </si>
   <si>
@@ -1512,16 +1500,28 @@
     <t>5.93e-03 MJ heat/MJ natural gas high pressure (Faist Emmenegger et al., 2017). Biomethane LHV = 34.72 MJ considering a constant upgrading mix</t>
   </si>
   <si>
-    <t>0.019% of emission rate based on Faist Emmenegger M., Del Duce A., Moreno Ruiz E., Brunner F., (2017). Update of the European natural gas supply chains. Ecoinvent, Zürich, Switzerland. Calculated from the estimated composition of biomethane from AD in the French mix after upgrading (0.52 CH4, 0.48 CO2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.019% of emission rate based on Faist Emmenegger M., Del Duce A., Moreno Ruiz E., Brunner F., (2017). Update of the European natural gas supply chains. Ecoinvent, Zürich, Switzerland. </t>
-  </si>
-  <si>
     <t>Scaled to reference product based on ecoinvent Faist Emmenegger M., Del Duce A., Moreno Ruiz E., Brunner F., (2017). Update of the European natural gas supply chains. Ecoinvent, Zürich, Switzerland</t>
   </si>
   <si>
     <t>market for biogas</t>
+  </si>
+  <si>
+    <t>Production of biogas from animal manure. Absorbed biogenic carbon is included to respect the carbon mass balance</t>
+  </si>
+  <si>
+    <t>5.93e-03 MJ heat/MJ natural gas high pressure (Faist Emmenegger et al., 2017).LHV = 35</t>
+  </si>
+  <si>
+    <t>1.5% of losses (ADEME Transition 2050)</t>
+  </si>
+  <si>
+    <t>1.5% ADEME Transition 2050. Calculated from the estimated composition of biomethane from AD in the French mix after upgrading</t>
+  </si>
+  <si>
+    <t>Average transportation of biomethane from anaerobic digestion (AD) in France. Leaks are calcualted considering the average market for upgrading technologies, which remains constant over time and scenarios. While correctly representing leaks for the upgrading mix, it can underestimate or overestimate transportation losses of individual upgrading technologies due to the different methane purities. Transportation is added to the individual AD production pathways because of implementation easiness in the user-defined scenario markets.</t>
+  </si>
+  <si>
+    <t>Losses 1.5% ADEME Transition 2050</t>
   </si>
 </sst>
 </file>
@@ -1735,7 +1735,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1838,6 +1838,7 @@
     </xf>
     <xf numFmtId="168" fontId="14" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
@@ -2124,7 +2125,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH978"/>
+  <dimension ref="A1:AH979"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -4457,7 +4458,7 @@
     </row>
     <row r="116" spans="1:9">
       <c r="A116" s="36" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="B116" s="34">
         <v>4.3695687769999996</v>
@@ -5583,7 +5584,7 @@
     </row>
     <row r="166" spans="1:9">
       <c r="A166" s="36" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="B166" s="34">
         <v>4.3011681309999998</v>
@@ -5815,7 +5816,7 @@
         <v>11</v>
       </c>
       <c r="B181" s="41" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C181" s="40"/>
       <c r="D181" s="41"/>
@@ -6921,7 +6922,7 @@
         <v>11</v>
       </c>
       <c r="B205" s="41" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C205" s="40"/>
       <c r="D205" s="41"/>
@@ -7977,7 +7978,7 @@
         <v>11</v>
       </c>
       <c r="B228" s="41" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C228" s="40"/>
       <c r="D228" s="41"/>
@@ -9033,7 +9034,7 @@
         <v>11</v>
       </c>
       <c r="B251" s="41" t="s">
-        <v>440</v>
+        <v>488</v>
       </c>
       <c r="C251" s="40"/>
       <c r="D251" s="41"/>
@@ -9416,7 +9417,7 @@
         <v>203</v>
       </c>
       <c r="C260" s="40">
-        <v>21.366271416169667</v>
+        <v>15.692759428778107</v>
       </c>
       <c r="D260" s="41" t="s">
         <v>13</v>
@@ -10117,7 +10118,7 @@
         <v>11</v>
       </c>
       <c r="B275" s="41" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C275" s="40"/>
       <c r="D275" s="41"/>
@@ -10283,7 +10284,7 @@
         <v>220</v>
       </c>
       <c r="C284" s="47">
-        <v>8.5232248605658256</v>
+        <v>6.2600027252774755</v>
       </c>
       <c r="D284" s="41" t="s">
         <v>13</v>
@@ -10986,7 +10987,7 @@
         <v>11</v>
       </c>
       <c r="B299" s="41" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C299" s="40"/>
       <c r="D299" s="41"/>
@@ -11363,13 +11364,13 @@
     </row>
     <row r="308" spans="1:34">
       <c r="A308" s="41" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B308" s="41" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C308" s="47">
-        <v>7.1155050309249033</v>
+        <v>5.2260830394610069</v>
       </c>
       <c r="D308" s="41" t="s">
         <v>13</v>
@@ -12021,7 +12022,7 @@
         <v>11</v>
       </c>
       <c r="B323" s="41" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C323" s="40"/>
       <c r="D323" s="41"/>
@@ -12401,7 +12402,7 @@
         <v>226</v>
       </c>
       <c r="C332" s="47">
-        <v>8.3098875333373829</v>
+        <v>6.1033141160126458</v>
       </c>
       <c r="D332" s="41" t="s">
         <v>13</v>
@@ -12835,7 +12836,7 @@
         <v>11</v>
       </c>
       <c r="B347" s="41" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C347" s="40"/>
       <c r="D347" s="41"/>
@@ -13218,7 +13219,7 @@
         <v>229</v>
       </c>
       <c r="C356" s="47">
-        <v>11.869335382034194</v>
+        <v>8.7176007971510625</v>
       </c>
       <c r="D356" s="41" t="s">
         <v>13</v>
@@ -13629,7 +13630,7 @@
         <v>11</v>
       </c>
       <c r="B371" s="41" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C371" s="40"/>
       <c r="D371" s="41"/>
@@ -13882,7 +13883,7 @@
         <v>11</v>
       </c>
       <c r="B384" s="41" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C384" s="40"/>
       <c r="D384" s="41"/>
@@ -14169,7 +14170,7 @@
         <v>11</v>
       </c>
       <c r="B398" s="41" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C398" s="40"/>
       <c r="D398" s="41"/>
@@ -14429,7 +14430,7 @@
         <v>11</v>
       </c>
       <c r="B410" s="41" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C410" s="40"/>
       <c r="D410" s="41"/>
@@ -14993,7 +14994,7 @@
         <v>11</v>
       </c>
       <c r="B424" s="41" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C424" s="40"/>
       <c r="D424" s="41"/>
@@ -15267,7 +15268,7 @@
         <v>1</v>
       </c>
       <c r="B437" s="39" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C437" s="40"/>
       <c r="D437" s="41"/>
@@ -15307,7 +15308,7 @@
         <v>11</v>
       </c>
       <c r="B438" s="41" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C438" s="40"/>
       <c r="D438" s="41"/>
@@ -15387,7 +15388,7 @@
         <v>4</v>
       </c>
       <c r="B440" s="41" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C440" s="40"/>
       <c r="D440" s="41"/>
@@ -15507,7 +15508,7 @@
         <v>76</v>
       </c>
       <c r="B443" s="41" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C443" s="40"/>
       <c r="D443" s="44"/>
@@ -15636,10 +15637,10 @@
     </row>
     <row r="446" spans="1:34">
       <c r="A446" s="46" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B446" s="46" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C446" s="47">
         <v>1</v>
@@ -15738,10 +15739,10 @@
     </row>
     <row r="448" spans="1:34">
       <c r="A448" s="46" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B448" s="46" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C448" s="47">
         <v>0.14285714285714285</v>
@@ -15788,10 +15789,10 @@
     </row>
     <row r="449" spans="1:34">
       <c r="A449" s="46" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B449" s="46" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C449" s="47">
         <v>0.14285714285714285</v>
@@ -15838,10 +15839,10 @@
     </row>
     <row r="450" spans="1:34">
       <c r="A450" s="46" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B450" s="46" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C450" s="47">
         <v>0.14285714285714285</v>
@@ -15888,10 +15889,10 @@
     </row>
     <row r="451" spans="1:34">
       <c r="A451" s="46" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B451" s="46" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C451" s="47">
         <v>0.14285714285714285</v>
@@ -15938,10 +15939,10 @@
     </row>
     <row r="452" spans="1:34">
       <c r="A452" s="46" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B452" s="46" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C452" s="47">
         <v>0.14285714285714285</v>
@@ -15988,10 +15989,10 @@
     </row>
     <row r="453" spans="1:34">
       <c r="A453" s="46" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B453" s="46" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C453" s="47">
         <v>0.14285714285714285</v>
@@ -16010,7 +16011,7 @@
         <v>12</v>
       </c>
       <c r="I453" s="46" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="J453" s="46"/>
       <c r="K453" s="46"/>
@@ -16129,7 +16130,7 @@
         <v>1</v>
       </c>
       <c r="B456" s="39" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C456" s="40"/>
       <c r="D456" s="41"/>
@@ -16169,7 +16170,7 @@
         <v>11</v>
       </c>
       <c r="B457" s="41" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C457" s="40"/>
       <c r="D457" s="41"/>
@@ -16249,7 +16250,7 @@
         <v>4</v>
       </c>
       <c r="B459" s="41" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C459" s="40"/>
       <c r="D459" s="41"/>
@@ -16369,7 +16370,7 @@
         <v>76</v>
       </c>
       <c r="B462" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C462" s="40"/>
       <c r="D462" s="44"/>
@@ -16498,10 +16499,10 @@
     </row>
     <row r="465" spans="1:34">
       <c r="A465" s="46" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B465" s="46" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C465" s="47">
         <v>1</v>
@@ -18584,7 +18585,7 @@
     </row>
     <row r="570" spans="1:9">
       <c r="A570" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B570" s="18" t="s">
         <v>195</v>
@@ -18979,7 +18980,7 @@
     </row>
     <row r="594" spans="1:9">
       <c r="A594" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B594" s="18" t="s">
         <v>195</v>
@@ -19554,7 +19555,7 @@
     </row>
     <row r="626" spans="1:9">
       <c r="A626" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B626" s="18" t="s">
         <v>195</v>
@@ -20129,7 +20130,7 @@
     </row>
     <row r="658" spans="1:9">
       <c r="A658" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B658" s="18" t="s">
         <v>195</v>
@@ -20704,7 +20705,7 @@
     </row>
     <row r="690" spans="1:9">
       <c r="A690" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B690" s="18" t="s">
         <v>195</v>
@@ -21279,7 +21280,7 @@
     </row>
     <row r="722" spans="1:9">
       <c r="A722" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B722" s="18" t="s">
         <v>195</v>
@@ -21674,7 +21675,7 @@
     </row>
     <row r="746" spans="1:9">
       <c r="A746" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B746" s="18" t="s">
         <v>195</v>
@@ -22249,7 +22250,7 @@
     </row>
     <row r="778" spans="1:9">
       <c r="A778" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B778" s="18" t="s">
         <v>195</v>
@@ -22824,7 +22825,7 @@
     </row>
     <row r="810" spans="1:9">
       <c r="A810" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B810" s="18" t="s">
         <v>195</v>
@@ -23400,7 +23401,7 @@
     </row>
     <row r="842" spans="1:9">
       <c r="A842" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="B842" s="18" t="s">
         <v>195</v>
@@ -24072,10 +24073,10 @@
     </row>
     <row r="873" spans="1:21" s="41" customFormat="1">
       <c r="A873" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B873" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C873" s="65">
         <v>1</v>
@@ -24805,7 +24806,7 @@
         <v>11</v>
       </c>
       <c r="B915" s="46" t="s">
-        <v>432</v>
+        <v>492</v>
       </c>
     </row>
     <row r="916" spans="1:9" s="41" customFormat="1">
@@ -24835,7 +24836,7 @@
         <v>1</v>
       </c>
       <c r="C918" s="40"/>
-      <c r="D918" s="72"/>
+      <c r="D918" s="74"/>
     </row>
     <row r="919" spans="1:9" s="41" customFormat="1">
       <c r="A919" s="39" t="s">
@@ -24913,13 +24914,12 @@
     </row>
     <row r="924" spans="1:9">
       <c r="A924" s="38" t="s">
+        <v>432</v>
+      </c>
+      <c r="B924" s="46" t="s">
         <v>433</v>
       </c>
-      <c r="B924" s="46" t="s">
-        <v>434</v>
-      </c>
       <c r="C924" s="66">
-        <f>0.00593*34.72</f>
         <v>0.20588960000000001</v>
       </c>
       <c r="D924" s="41" t="s">
@@ -24933,7 +24933,7 @@
         <v>12</v>
       </c>
       <c r="I924" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
     </row>
     <row r="925" spans="1:9">
@@ -24956,7 +24956,7 @@
         <v>12</v>
       </c>
       <c r="I925" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
     </row>
     <row r="926" spans="1:9">
@@ -24965,7 +24965,7 @@
       </c>
       <c r="B926"/>
       <c r="C926" s="32">
-        <v>1.1448370274509817E-5</v>
+        <v>9.038187058823539E-4</v>
       </c>
       <c r="D926" t="s">
         <v>13</v>
@@ -24980,7 +24980,7 @@
         <v>15</v>
       </c>
       <c r="I926" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="927" spans="1:9">
@@ -24989,7 +24989,7 @@
       </c>
       <c r="B927"/>
       <c r="C927" s="32">
-        <v>1.3211959364705882E-4</v>
+        <v>1.0430494235294118E-2</v>
       </c>
       <c r="D927" t="s">
         <v>13</v>
@@ -25004,7 +25004,7 @@
         <v>15</v>
       </c>
       <c r="I927" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="928" spans="1:9" s="69" customFormat="1">
@@ -25015,7 +25015,7 @@
         <v>1</v>
       </c>
       <c r="B929" s="63" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C929" s="40"/>
     </row>
@@ -25024,7 +25024,7 @@
         <v>11</v>
       </c>
       <c r="B930" s="46" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="931" spans="1:9" s="41" customFormat="1">
@@ -25041,7 +25041,7 @@
         <v>4</v>
       </c>
       <c r="B932" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C932" s="40"/>
     </row>
@@ -25110,10 +25110,10 @@
     </row>
     <row r="938" spans="1:9" s="41" customFormat="1">
       <c r="A938" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B938" s="46" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C938" s="65">
         <v>1</v>
@@ -25133,10 +25133,10 @@
     </row>
     <row r="939" spans="1:9">
       <c r="A939" s="38" t="s">
+        <v>432</v>
+      </c>
+      <c r="B939" s="46" t="s">
         <v>433</v>
-      </c>
-      <c r="B939" s="46" t="s">
-        <v>434</v>
       </c>
       <c r="C939" s="66">
         <f>0.00593*35.8</f>
@@ -25153,7 +25153,7 @@
         <v>12</v>
       </c>
       <c r="I939" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
     </row>
     <row r="940" spans="1:9">
@@ -25176,7 +25176,7 @@
         <v>12</v>
       </c>
       <c r="I940" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
     </row>
     <row r="941" spans="1:9">
@@ -25185,7 +25185,7 @@
       </c>
       <c r="B941"/>
       <c r="C941" s="18">
-        <v>1.3623000000000002E-4</v>
+        <v>1.0754999999999999E-2</v>
       </c>
       <c r="D941" t="s">
         <v>13</v>
@@ -25200,7 +25200,7 @@
         <v>15</v>
       </c>
       <c r="I941" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="942" spans="1:9" s="69" customFormat="1">
@@ -25211,7 +25211,7 @@
         <v>1</v>
       </c>
       <c r="B943" s="63" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C943" s="40"/>
       <c r="D943" s="41"/>
@@ -25226,7 +25226,7 @@
         <v>11</v>
       </c>
       <c r="B944" s="46" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C944" s="41"/>
       <c r="D944" s="41"/>
@@ -25353,7 +25353,7 @@
     </row>
     <row r="952" spans="1:9">
       <c r="A952" s="46" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B952" s="46" t="s">
         <v>162</v>
@@ -25375,10 +25375,10 @@
     </row>
     <row r="953" spans="1:9">
       <c r="A953" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B953" s="18" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C953">
         <v>0.1764792</v>
@@ -25393,12 +25393,12 @@
         <v>12</v>
       </c>
       <c r="I953" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="954" spans="1:9">
       <c r="A954" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B954" s="18" t="s">
         <v>162</v>
@@ -25418,7 +25418,7 @@
     </row>
     <row r="955" spans="1:9">
       <c r="A955" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B955" s="18" t="s">
         <v>162</v>
@@ -25438,7 +25438,7 @@
     </row>
     <row r="956" spans="1:9">
       <c r="A956" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B956" s="18" t="s">
         <v>162</v>
@@ -25458,7 +25458,7 @@
     </row>
     <row r="957" spans="1:9">
       <c r="A957" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B957" s="18" t="s">
         <v>162</v>
@@ -25478,7 +25478,7 @@
     </row>
     <row r="958" spans="1:9">
       <c r="A958" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B958" s="18" t="s">
         <v>162</v>
@@ -25498,7 +25498,7 @@
     </row>
     <row r="959" spans="1:9">
       <c r="A959" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B959" s="18" t="s">
         <v>162</v>
@@ -25518,7 +25518,7 @@
     </row>
     <row r="960" spans="1:9">
       <c r="A960" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B960" s="18" t="s">
         <v>162</v>
@@ -25541,7 +25541,7 @@
         <v>113</v>
       </c>
       <c r="C961" s="18">
-        <v>6.6423599999999999E-6</v>
+        <v>9.6000000000000002E-5</v>
       </c>
       <c r="D961" s="41" t="s">
         <v>13</v>
@@ -25557,7 +25557,7 @@
         <v>15</v>
       </c>
       <c r="I961" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="962" spans="1:9">
@@ -25565,7 +25565,7 @@
         <v>40</v>
       </c>
       <c r="C962" s="18">
-        <v>2.3978160000000001E-5</v>
+        <v>3.435E-4</v>
       </c>
       <c r="D962" s="41" t="s">
         <v>13</v>
@@ -25581,15 +25581,15 @@
         <v>15</v>
       </c>
       <c r="I962" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="963" spans="1:9">
       <c r="A963" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C963" s="18">
-        <v>5.74128E-5</v>
+        <v>8.234999999999999E-4</v>
       </c>
       <c r="D963" s="41" t="s">
         <v>13</v>
@@ -25605,15 +25605,15 @@
         <v>15</v>
       </c>
       <c r="I963" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="964" spans="1:9">
       <c r="A964" t="s">
         <v>118</v>
       </c>
-      <c r="C964">
-        <v>6.9317999999999995E-4</v>
+      <c r="C964" s="18">
+        <v>9.9435000000000009E-3</v>
       </c>
       <c r="D964" s="41" t="s">
         <v>13</v>
@@ -25628,7 +25628,7 @@
         <v>15</v>
       </c>
       <c r="I964" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="965" spans="1:9">
@@ -25636,7 +25636,7 @@
         <v>216</v>
       </c>
       <c r="C965" s="18">
-        <v>4.7829600000000004E-7</v>
+        <v>7.5000000000000002E-6</v>
       </c>
       <c r="D965" s="41" t="s">
         <v>13</v>
@@ -25652,7 +25652,7 @@
         <v>15</v>
       </c>
       <c r="I965" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="966" spans="1:9">
@@ -25660,7 +25660,7 @@
         <v>123</v>
       </c>
       <c r="C966" s="18">
-        <v>1.2917519999999999E-5</v>
+        <v>1.8599999999999999E-4</v>
       </c>
       <c r="D966" s="41" t="s">
         <v>13</v>
@@ -25676,7 +25676,7 @@
         <v>15</v>
       </c>
       <c r="I966" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
     </row>
     <row r="967" spans="1:9">
@@ -25695,7 +25695,7 @@
         <v>1</v>
       </c>
       <c r="B968" s="63" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="C968" s="40"/>
       <c r="D968" s="41"/>
@@ -25710,7 +25710,7 @@
         <v>11</v>
       </c>
       <c r="B969" s="46" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="C969" s="41"/>
       <c r="D969" s="41"/>
@@ -25785,7 +25785,7 @@
         <v>76</v>
       </c>
       <c r="B974" s="41" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="C974" s="40"/>
       <c r="D974" s="44"/>
@@ -25839,7 +25839,7 @@
     </row>
     <row r="977" spans="1:9">
       <c r="A977" s="46" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="B977" s="46" t="s">
         <v>244</v>
@@ -25860,8 +25860,8 @@
       <c r="I977" s="39"/>
     </row>
     <row r="978" spans="1:9">
-      <c r="A978" t="s">
-        <v>485</v>
+      <c r="A978" s="38" t="s">
+        <v>481</v>
       </c>
       <c r="B978" s="46" t="s">
         <v>244</v>
@@ -25878,6 +25878,14 @@
       <c r="H978" t="s">
         <v>12</v>
       </c>
+    </row>
+    <row r="979" spans="1:9">
+      <c r="A979" s="46"/>
+      <c r="B979" s="46"/>
+      <c r="C979" s="41"/>
+      <c r="D979" s="41"/>
+      <c r="F979" s="39"/>
+      <c r="G979" s="46"/>
     </row>
   </sheetData>
   <phoneticPr fontId="19" type="noConversion"/>

</xml_diff>

<commit_message>
Corrected efficiency reference for AD of CIVE (supply instead of collection in the LCI)
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050-Copie.xlsx
+++ b/inventories/lci-Tr2050-Copie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1466" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B35199D4-FD63-433D-BE0A-728A11FBDF48}"/>
+  <xr:revisionPtr revIDLastSave="1468" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B83F689-C10F-4311-85F9-3E0DF88D458F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -1774,7 +1774,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1873,8 +1873,6 @@
     <xf numFmtId="168" fontId="14" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2793,7 +2791,7 @@
       <c r="B37" s="18">
         <v>1.25125</v>
       </c>
-      <c r="C37" s="70" t="s">
+      <c r="C37" t="s">
         <v>29</v>
       </c>
       <c r="D37" t="s">
@@ -4507,7 +4505,7 @@
       <c r="I115" s="34"/>
     </row>
     <row r="116" spans="1:9">
-      <c r="A116" s="71" t="s">
+      <c r="A116" s="34" t="s">
         <v>472</v>
       </c>
       <c r="B116" s="34">
@@ -5633,7 +5631,7 @@
       <c r="I165" s="34"/>
     </row>
     <row r="166" spans="1:9">
-      <c r="A166" s="71" t="s">
+      <c r="A166" s="34" t="s">
         <v>472</v>
       </c>
       <c r="B166" s="34">
@@ -16779,1688 +16777,1688 @@
         <v>242</v>
       </c>
     </row>
-    <row r="471" spans="1:34" s="74" customFormat="1">
-      <c r="A471" s="72"/>
-      <c r="B471" s="72"/>
-      <c r="C471" s="73"/>
-      <c r="D471" s="72"/>
-      <c r="E471" s="72"/>
-      <c r="F471" s="72"/>
-      <c r="G471" s="72"/>
-      <c r="H471" s="72"/>
-      <c r="I471" s="72"/>
-      <c r="J471" s="72"/>
-      <c r="K471" s="72"/>
-      <c r="L471" s="72"/>
-      <c r="M471" s="72"/>
-      <c r="N471" s="72"/>
-      <c r="O471" s="72"/>
-      <c r="P471" s="72"/>
-      <c r="Q471" s="72"/>
-      <c r="R471" s="72"/>
-      <c r="S471" s="72"/>
-      <c r="T471" s="72"/>
-      <c r="U471" s="72"/>
-      <c r="V471" s="72"/>
-      <c r="W471" s="72"/>
-      <c r="X471" s="72"/>
-      <c r="Y471" s="72"/>
-      <c r="Z471" s="72"/>
-      <c r="AA471" s="72"/>
-      <c r="AB471" s="72"/>
-      <c r="AC471" s="72"/>
-      <c r="AD471" s="72"/>
-      <c r="AE471" s="72"/>
-      <c r="AF471" s="72"/>
-      <c r="AG471" s="72"/>
-      <c r="AH471" s="72"/>
-    </row>
-    <row r="472" spans="1:34" s="74" customFormat="1">
-      <c r="A472" s="75" t="s">
+    <row r="471" spans="1:34" s="72" customFormat="1">
+      <c r="A471" s="70"/>
+      <c r="B471" s="70"/>
+      <c r="C471" s="71"/>
+      <c r="D471" s="70"/>
+      <c r="E471" s="70"/>
+      <c r="F471" s="70"/>
+      <c r="G471" s="70"/>
+      <c r="H471" s="70"/>
+      <c r="I471" s="70"/>
+      <c r="J471" s="70"/>
+      <c r="K471" s="70"/>
+      <c r="L471" s="70"/>
+      <c r="M471" s="70"/>
+      <c r="N471" s="70"/>
+      <c r="O471" s="70"/>
+      <c r="P471" s="70"/>
+      <c r="Q471" s="70"/>
+      <c r="R471" s="70"/>
+      <c r="S471" s="70"/>
+      <c r="T471" s="70"/>
+      <c r="U471" s="70"/>
+      <c r="V471" s="70"/>
+      <c r="W471" s="70"/>
+      <c r="X471" s="70"/>
+      <c r="Y471" s="70"/>
+      <c r="Z471" s="70"/>
+      <c r="AA471" s="70"/>
+      <c r="AB471" s="70"/>
+      <c r="AC471" s="70"/>
+      <c r="AD471" s="70"/>
+      <c r="AE471" s="70"/>
+      <c r="AF471" s="70"/>
+      <c r="AG471" s="70"/>
+      <c r="AH471" s="70"/>
+    </row>
+    <row r="472" spans="1:34" s="72" customFormat="1">
+      <c r="A472" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B472" s="76" t="s">
+      <c r="B472" s="74" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="473" spans="1:34" s="74" customFormat="1">
-      <c r="A473" s="75" t="s">
+    <row r="473" spans="1:34" s="72" customFormat="1">
+      <c r="A473" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B473" s="77" t="s">
+      <c r="B473" s="75" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="474" spans="1:34" s="74" customFormat="1">
-      <c r="A474" s="75" t="s">
+    <row r="474" spans="1:34" s="72" customFormat="1">
+      <c r="A474" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="B474" s="77">
+      <c r="B474" s="75">
         <v>1</v>
       </c>
     </row>
-    <row r="475" spans="1:34" s="74" customFormat="1" ht="15.75">
-      <c r="A475" s="75" t="s">
+    <row r="475" spans="1:34" s="72" customFormat="1" ht="15.75">
+      <c r="A475" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="B475" s="78" t="s">
+      <c r="B475" s="76" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="476" spans="1:34" s="74" customFormat="1">
-      <c r="A476" s="75" t="s">
+    <row r="476" spans="1:34" s="72" customFormat="1">
+      <c r="A476" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="B476" s="77" t="s">
+      <c r="B476" s="75" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="477" spans="1:34" s="74" customFormat="1">
-      <c r="A477" s="75" t="s">
+    <row r="477" spans="1:34" s="72" customFormat="1">
+      <c r="A477" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="B477" s="77" t="s">
+      <c r="B477" s="75" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="478" spans="1:34" s="74" customFormat="1">
-      <c r="A478" s="75" t="s">
+    <row r="478" spans="1:34" s="72" customFormat="1">
+      <c r="A478" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="B478" s="77" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="479" spans="1:34" s="74" customFormat="1">
-      <c r="A479" s="75" t="s">
+      <c r="B478" s="75" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="479" spans="1:34" s="72" customFormat="1">
+      <c r="A479" s="73" t="s">
         <v>299</v>
       </c>
-      <c r="B479" s="79">
+      <c r="B479" s="77">
         <f>14.9/(1-B480)</f>
         <v>17.325581395348838</v>
       </c>
     </row>
-    <row r="480" spans="1:34" s="74" customFormat="1">
-      <c r="A480" s="75" t="s">
+    <row r="480" spans="1:34" s="72" customFormat="1">
+      <c r="A480" s="73" t="s">
         <v>300</v>
       </c>
-      <c r="B480" s="80">
+      <c r="B480" s="78">
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="481" spans="1:8" s="74" customFormat="1" ht="15.75">
-      <c r="A481" s="81" t="s">
+    <row r="481" spans="1:8" s="72" customFormat="1" ht="15.75">
+      <c r="A481" s="79" t="s">
         <v>7</v>
       </c>
-      <c r="B481" s="77"/>
-    </row>
-    <row r="482" spans="1:8" s="82" customFormat="1">
-      <c r="A482" s="82" t="s">
+      <c r="B481" s="75"/>
+    </row>
+    <row r="482" spans="1:8" s="80" customFormat="1">
+      <c r="A482" s="80" t="s">
         <v>8</v>
       </c>
-      <c r="B482" s="82" t="s">
+      <c r="B482" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="C482" s="82" t="s">
+      <c r="C482" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="D482" s="82" t="s">
+      <c r="D482" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="E482" s="82" t="s">
+      <c r="E482" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="F482" s="82" t="s">
+      <c r="F482" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="G482" s="82" t="s">
+      <c r="G482" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="H482" s="82" t="s">
+      <c r="H482" s="80" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="483" spans="1:8" s="74" customFormat="1" ht="15.75">
-      <c r="A483" s="74" t="s">
+    <row r="483" spans="1:8" s="72" customFormat="1" ht="15.75">
+      <c r="A483" s="72" t="s">
         <v>381</v>
       </c>
-      <c r="B483" s="77">
+      <c r="B483" s="75">
         <v>1</v>
       </c>
-      <c r="C483" s="74" t="s">
+      <c r="C483" s="72" t="s">
         <v>49</v>
       </c>
-      <c r="D483" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E483" s="74" t="s">
+      <c r="D483" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E483" s="72" t="s">
         <v>301</v>
       </c>
-      <c r="F483" s="74" t="s">
+      <c r="F483" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="G483" s="74" t="s">
+      <c r="G483" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="H483" s="78" t="s">
+      <c r="H483" s="76" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="484" spans="1:8" s="74" customFormat="1">
-      <c r="A484" s="74" t="s">
+    <row r="484" spans="1:8" s="72" customFormat="1">
+      <c r="A484" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="B484" s="77">
+      <c r="B484" s="75">
         <v>7.5716999999999994E-4</v>
       </c>
-      <c r="D484" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E484" s="74" t="s">
+      <c r="D484" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E484" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="F484" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G484" s="74" t="s">
+      <c r="F484" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G484" s="72" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="485" spans="1:8" s="74" customFormat="1">
-      <c r="A485" s="74" t="s">
+    <row r="485" spans="1:8" s="72" customFormat="1">
+      <c r="A485" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="B485" s="77">
+      <c r="B485" s="75">
         <v>1.7899999999999998E-6</v>
       </c>
-      <c r="D485" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E485" s="74" t="s">
+      <c r="D485" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E485" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="F485" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G485" s="74" t="s">
+      <c r="F485" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G485" s="72" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="486" spans="1:8" s="74" customFormat="1">
-      <c r="A486" s="74" t="s">
+    <row r="486" spans="1:8" s="72" customFormat="1">
+      <c r="A486" s="72" t="s">
         <v>304</v>
       </c>
-      <c r="B486" s="77">
+      <c r="B486" s="75">
         <v>8.9499999999999996E-3</v>
       </c>
-      <c r="C486" s="74" t="s">
+      <c r="C486" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D486" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E486" s="74" t="s">
+      <c r="D486" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E486" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F486" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G486" s="74" t="s">
+      <c r="F486" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G486" s="72" t="s">
         <v>306</v>
       </c>
-      <c r="H486" s="74" t="s">
+      <c r="H486" s="72" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="487" spans="1:8" s="74" customFormat="1">
-      <c r="A487" s="74" t="s">
+    <row r="487" spans="1:8" s="72" customFormat="1">
+      <c r="A487" s="72" t="s">
         <v>308</v>
       </c>
-      <c r="B487" s="77">
+      <c r="B487" s="75">
         <v>3.382384E-3</v>
       </c>
-      <c r="C487" s="74" t="s">
+      <c r="C487" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D487" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E487" s="74" t="s">
+      <c r="D487" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E487" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F487" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G487" s="74" t="s">
+      <c r="F487" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G487" s="72" t="s">
         <v>309</v>
       </c>
-      <c r="H487" s="74" t="s">
+      <c r="H487" s="72" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="488" spans="1:8" s="74" customFormat="1">
-      <c r="A488" s="74" t="s">
+    <row r="488" spans="1:8" s="72" customFormat="1">
+      <c r="A488" s="72" t="s">
         <v>243</v>
       </c>
-      <c r="B488" s="77">
+      <c r="B488" s="75">
         <v>1.9689999999999999E-2</v>
       </c>
-      <c r="C488" s="74" t="s">
+      <c r="C488" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="D488" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E488" s="74" t="s">
+      <c r="D488" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E488" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F488" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G488" s="74" t="s">
+      <c r="F488" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G488" s="72" t="s">
         <v>311</v>
       </c>
-      <c r="H488" s="74" t="s">
+      <c r="H488" s="72" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="489" spans="1:8" s="74" customFormat="1">
-      <c r="A489" s="74" t="s">
+    <row r="489" spans="1:8" s="72" customFormat="1">
+      <c r="A489" s="72" t="s">
         <v>295</v>
       </c>
-      <c r="B489" s="77">
+      <c r="B489" s="75">
         <f>0.00179/1000</f>
         <v>1.79E-6</v>
       </c>
-      <c r="C489" s="74" t="s">
+      <c r="C489" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D489" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E489" s="74" t="s">
+      <c r="D489" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E489" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F489" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G489" s="74" t="s">
+      <c r="F489" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G489" s="72" t="s">
         <v>312</v>
       </c>
-      <c r="H489" s="74" t="s">
+      <c r="H489" s="72" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="490" spans="1:8" s="74" customFormat="1">
-      <c r="A490" s="74" t="s">
+    <row r="490" spans="1:8" s="72" customFormat="1">
+      <c r="A490" s="72" t="s">
         <v>313</v>
       </c>
-      <c r="B490" s="77">
+      <c r="B490" s="75">
         <f>986/1000000</f>
         <v>9.859999999999999E-4</v>
       </c>
-      <c r="C490" s="74" t="s">
+      <c r="C490" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D490" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="F490" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G490" s="74" t="s">
+      <c r="D490" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="F490" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G490" s="72" t="s">
         <v>314</v>
       </c>
-      <c r="H490" s="74" t="s">
+      <c r="H490" s="72" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="491" spans="1:8" s="74" customFormat="1">
-      <c r="A491" s="74" t="s">
+    <row r="491" spans="1:8" s="72" customFormat="1">
+      <c r="A491" s="72" t="s">
         <v>293</v>
       </c>
-      <c r="B491" s="77">
+      <c r="B491" s="75">
         <v>5.3699999999999989E-3</v>
       </c>
-      <c r="C491" s="74" t="s">
+      <c r="C491" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="D491" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E491" s="74" t="s">
+      <c r="D491" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E491" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F491" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G491" s="74" t="s">
+      <c r="F491" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G491" s="72" t="s">
         <v>316</v>
       </c>
-      <c r="H491" s="74" t="s">
+      <c r="H491" s="72" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="492" spans="1:8" s="74" customFormat="1">
-      <c r="A492" s="74" t="s">
+    <row r="492" spans="1:8" s="72" customFormat="1">
+      <c r="A492" s="72" t="s">
         <v>317</v>
       </c>
-      <c r="B492" s="77">
+      <c r="B492" s="75">
         <v>5.3699999999999989E-3</v>
       </c>
-      <c r="C492" s="74" t="s">
+      <c r="C492" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="D492" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E492" s="74" t="s">
+      <c r="D492" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E492" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F492" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G492" s="74" t="s">
+      <c r="F492" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G492" s="72" t="s">
         <v>318</v>
       </c>
-      <c r="H492" s="74" t="s">
+      <c r="H492" s="72" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="493" spans="1:8" s="74" customFormat="1">
-      <c r="A493" s="74" t="s">
+    <row r="493" spans="1:8" s="72" customFormat="1">
+      <c r="A493" s="72" t="s">
         <v>320</v>
       </c>
-      <c r="B493" s="77">
+      <c r="B493" s="75">
         <v>2.3269999999999996E-2</v>
       </c>
-      <c r="C493" s="74" t="s">
+      <c r="C493" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D493" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E493" s="74" t="s">
+      <c r="D493" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E493" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F493" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G493" s="74" t="s">
+      <c r="F493" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G493" s="72" t="s">
         <v>311</v>
       </c>
-      <c r="H493" s="74" t="s">
+      <c r="H493" s="72" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="494" spans="1:8" s="74" customFormat="1">
-      <c r="A494" s="74" t="s">
+    <row r="494" spans="1:8" s="72" customFormat="1">
+      <c r="A494" s="72" t="s">
         <v>322</v>
       </c>
-      <c r="B494" s="77">
+      <c r="B494" s="75">
         <f>0.01295781*43</f>
         <v>0.55718582999999999</v>
       </c>
-      <c r="C494" s="74" t="s">
+      <c r="C494" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="D494" s="74" t="s">
+      <c r="D494" s="72" t="s">
         <v>46</v>
       </c>
-      <c r="E494" s="74" t="s">
+      <c r="E494" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F494" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G494" s="74" t="s">
+      <c r="F494" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G494" s="72" t="s">
         <v>323</v>
       </c>
-      <c r="H494" s="74" t="s">
+      <c r="H494" s="72" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="495" spans="1:8" s="74" customFormat="1">
-      <c r="A495" s="74" t="s">
+    <row r="495" spans="1:8" s="72" customFormat="1">
+      <c r="A495" s="72" t="s">
         <v>325</v>
       </c>
-      <c r="B495" s="77">
+      <c r="B495" s="75">
         <v>7.464300000000001E-3</v>
       </c>
-      <c r="C495" s="74" t="s">
+      <c r="C495" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="D495" s="74" t="s">
+      <c r="D495" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="E495" s="74" t="s">
+      <c r="E495" s="72" t="s">
         <v>326</v>
       </c>
-      <c r="F495" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G495" s="74" t="s">
+      <c r="F495" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G495" s="72" t="s">
         <v>309</v>
       </c>
-      <c r="H495" s="74" t="s">
+      <c r="H495" s="72" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="496" spans="1:8" s="74" customFormat="1">
-      <c r="A496" s="74" t="s">
+    <row r="496" spans="1:8" s="72" customFormat="1">
+      <c r="A496" s="72" t="s">
         <v>325</v>
       </c>
-      <c r="B496" s="77">
+      <c r="B496" s="75">
         <v>1.9407179999999997E-3</v>
       </c>
-      <c r="C496" s="74" t="s">
+      <c r="C496" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="D496" s="74" t="s">
+      <c r="D496" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="E496" s="74" t="s">
+      <c r="E496" s="72" t="s">
         <v>326</v>
       </c>
-      <c r="F496" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G496" s="74" t="s">
+      <c r="F496" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G496" s="72" t="s">
         <v>327</v>
       </c>
-      <c r="H496" s="74" t="s">
+      <c r="H496" s="72" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="497" spans="1:8" s="74" customFormat="1">
-      <c r="A497" s="74" t="s">
+    <row r="497" spans="1:8" s="72" customFormat="1">
+      <c r="A497" s="72" t="s">
         <v>328</v>
       </c>
-      <c r="B497" s="77">
+      <c r="B497" s="75">
         <v>3.923859E-3</v>
       </c>
-      <c r="C497" s="74" t="s">
+      <c r="C497" s="72" t="s">
         <v>49</v>
       </c>
-      <c r="D497" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E497" s="74" t="s">
+      <c r="D497" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E497" s="72" t="s">
         <v>305</v>
       </c>
-      <c r="F497" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="G497" s="74" t="s">
+      <c r="F497" s="72" t="s">
+        <v>12</v>
+      </c>
+      <c r="G497" s="72" t="s">
         <v>309</v>
       </c>
-      <c r="H497" s="74" t="s">
+      <c r="H497" s="72" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="498" spans="1:8" s="74" customFormat="1">
-      <c r="A498" s="74" t="s">
+    <row r="498" spans="1:8" s="72" customFormat="1">
+      <c r="A498" s="72" t="s">
         <v>285</v>
       </c>
-      <c r="B498" s="77">
+      <c r="B498" s="75">
         <f>17.9*(1-B480)</f>
         <v>15.393999999999998</v>
       </c>
-      <c r="D498" s="74" t="s">
+      <c r="D498" s="72" t="s">
         <v>46</v>
       </c>
-      <c r="E498" s="74" t="s">
+      <c r="E498" s="72" t="s">
         <v>286</v>
       </c>
-      <c r="F498" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G498" s="74" t="s">
+      <c r="F498" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G498" s="72" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="499" spans="1:8" s="74" customFormat="1">
-      <c r="A499" s="74" t="s">
+    <row r="499" spans="1:8" s="72" customFormat="1">
+      <c r="A499" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="B499" s="77">
+      <c r="B499" s="75">
         <v>0</v>
       </c>
-      <c r="D499" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E499" s="74" t="s">
+      <c r="D499" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E499" s="72" t="s">
         <v>198</v>
       </c>
-      <c r="F499" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G499" s="74" t="s">
+      <c r="F499" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G499" s="72" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="500" spans="1:8" s="74" customFormat="1">
-      <c r="A500" s="74" t="s">
+    <row r="500" spans="1:8" s="72" customFormat="1">
+      <c r="A500" s="72" t="s">
         <v>289</v>
       </c>
-      <c r="B500" s="77">
+      <c r="B500" s="75">
         <f>1/(7129/10000)</f>
         <v>1.4027212792818067</v>
       </c>
-      <c r="D500" s="74" t="s">
+      <c r="D500" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="E500" s="74" t="s">
+      <c r="E500" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F500" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G500" s="74" t="s">
+      <c r="F500" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G500" s="72" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="501" spans="1:8" s="74" customFormat="1">
-      <c r="A501" s="74" t="s">
+    <row r="501" spans="1:8" s="72" customFormat="1">
+      <c r="A501" s="72" t="s">
         <v>332</v>
       </c>
-      <c r="B501" s="77">
+      <c r="B501" s="75">
         <f>1/(7129/10000)</f>
         <v>1.4027212792818067</v>
       </c>
-      <c r="D501" s="74" t="s">
+      <c r="D501" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="E501" s="74" t="s">
+      <c r="E501" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F501" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G501" s="74" t="s">
+      <c r="F501" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G501" s="72" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="502" spans="1:8" s="74" customFormat="1">
-      <c r="A502" s="74" t="s">
+    <row r="502" spans="1:8" s="72" customFormat="1">
+      <c r="A502" s="72" t="s">
         <v>292</v>
       </c>
-      <c r="B502" s="77">
+      <c r="B502" s="75">
         <f>1/(7129/10000)</f>
         <v>1.4027212792818067</v>
       </c>
-      <c r="D502" s="74" t="s">
+      <c r="D502" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="E502" s="74" t="s">
+      <c r="E502" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F502" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G502" s="74" t="s">
+      <c r="F502" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G502" s="72" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="503" spans="1:8" s="74" customFormat="1">
-      <c r="A503" s="74" t="s">
+    <row r="503" spans="1:8" s="72" customFormat="1">
+      <c r="A503" s="72" t="s">
         <v>130</v>
       </c>
-      <c r="B503" s="77">
+      <c r="B503" s="75">
         <v>0.17007192792102799</v>
       </c>
-      <c r="D503" s="74" t="s">
+      <c r="D503" s="72" t="s">
         <v>128</v>
       </c>
-      <c r="E503" s="74" t="s">
+      <c r="E503" s="72" t="s">
         <v>25</v>
       </c>
-      <c r="F503" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G503" s="74" t="s">
+      <c r="F503" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G503" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="504" spans="1:8" s="74" customFormat="1">
-      <c r="A504" s="74" t="s">
+    <row r="504" spans="1:8" s="72" customFormat="1">
+      <c r="A504" s="72" t="s">
         <v>119</v>
       </c>
-      <c r="B504" s="77">
+      <c r="B504" s="75">
         <v>8.3517419999999996E-5</v>
       </c>
-      <c r="D504" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E504" s="74" t="s">
+      <c r="D504" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E504" s="72" t="s">
         <v>183</v>
       </c>
-      <c r="F504" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G504" s="74" t="s">
+      <c r="F504" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G504" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="505" spans="1:8" s="74" customFormat="1">
-      <c r="A505" s="74" t="s">
+    <row r="505" spans="1:8" s="72" customFormat="1">
+      <c r="A505" s="72" t="s">
         <v>268</v>
       </c>
-      <c r="B505" s="77">
+      <c r="B505" s="75">
         <v>1.0182310000000001E-3</v>
       </c>
-      <c r="D505" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E505" s="74" t="s">
+      <c r="D505" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E505" s="72" t="s">
         <v>183</v>
       </c>
-      <c r="F505" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G505" s="74" t="s">
+      <c r="F505" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G505" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="506" spans="1:8" s="74" customFormat="1">
-      <c r="A506" s="74" t="s">
+    <row r="506" spans="1:8" s="72" customFormat="1">
+      <c r="A506" s="72" t="s">
         <v>335</v>
       </c>
-      <c r="B506" s="77">
+      <c r="B506" s="75">
         <f>B508/2</f>
         <v>0.47991081325301199</v>
       </c>
-      <c r="D506" s="74" t="s">
+      <c r="D506" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="E506" s="74" t="s">
+      <c r="E506" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F506" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G506" s="74" t="s">
+      <c r="F506" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G506" s="72" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="507" spans="1:8" s="74" customFormat="1">
-      <c r="A507" s="74" t="s">
+    <row r="507" spans="1:8" s="72" customFormat="1">
+      <c r="A507" s="72" t="s">
         <v>337</v>
       </c>
-      <c r="B507" s="77">
+      <c r="B507" s="75">
         <f>B508/2</f>
         <v>0.47991081325301199</v>
       </c>
-      <c r="D507" s="74" t="s">
+      <c r="D507" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="E507" s="74" t="s">
+      <c r="E507" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F507" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G507" s="74" t="s">
+      <c r="F507" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G507" s="72" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="508" spans="1:8" s="74" customFormat="1">
-      <c r="A508" s="74" t="s">
+    <row r="508" spans="1:8" s="72" customFormat="1">
+      <c r="A508" s="72" t="s">
         <v>338</v>
       </c>
-      <c r="B508" s="77">
+      <c r="B508" s="75">
         <v>0.95982162650602398</v>
       </c>
-      <c r="D508" s="74" t="s">
+      <c r="D508" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="E508" s="74" t="s">
+      <c r="E508" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="F508" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G508" s="74" t="s">
+      <c r="F508" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G508" s="72" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="509" spans="1:8" s="74" customFormat="1">
-      <c r="A509" s="74" t="s">
+    <row r="509" spans="1:8" s="72" customFormat="1">
+      <c r="A509" s="72" t="s">
         <v>340</v>
       </c>
-      <c r="B509" s="77">
+      <c r="B509" s="75">
         <v>1.0107999999999999E-6</v>
       </c>
-      <c r="D509" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E509" s="74" t="s">
+      <c r="D509" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E509" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F509" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G509" s="74" t="s">
+      <c r="F509" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G509" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="510" spans="1:8" s="74" customFormat="1">
-      <c r="A510" s="74" t="s">
+    <row r="510" spans="1:8" s="72" customFormat="1">
+      <c r="A510" s="72" t="s">
         <v>341</v>
       </c>
-      <c r="B510" s="77">
+      <c r="B510" s="75">
         <v>6.1366999999999996E-7</v>
       </c>
-      <c r="D510" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E510" s="74" t="s">
+      <c r="D510" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E510" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F510" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G510" s="74" t="s">
+      <c r="F510" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G510" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="511" spans="1:8" s="74" customFormat="1">
-      <c r="A511" s="74" t="s">
+    <row r="511" spans="1:8" s="72" customFormat="1">
+      <c r="A511" s="72" t="s">
         <v>342</v>
       </c>
-      <c r="B511" s="77">
+      <c r="B511" s="75">
         <v>4.8131000000000003E-9</v>
       </c>
-      <c r="D511" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E511" s="74" t="s">
+      <c r="D511" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E511" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F511" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G511" s="74" t="s">
+      <c r="F511" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G511" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="512" spans="1:8" s="74" customFormat="1">
-      <c r="A512" s="74" t="s">
+    <row r="512" spans="1:8" s="72" customFormat="1">
+      <c r="A512" s="72" t="s">
         <v>343</v>
       </c>
-      <c r="B512" s="77">
+      <c r="B512" s="75">
         <v>6.4977000000000003E-7</v>
       </c>
-      <c r="D512" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E512" s="74" t="s">
+      <c r="D512" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E512" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F512" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G512" s="74" t="s">
+      <c r="F512" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G512" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="513" spans="1:7" s="74" customFormat="1">
-      <c r="A513" s="74" t="s">
+    <row r="513" spans="1:7" s="72" customFormat="1">
+      <c r="A513" s="72" t="s">
         <v>344</v>
       </c>
-      <c r="B513" s="77">
+      <c r="B513" s="75">
         <v>-1.5040999999999999E-6</v>
       </c>
-      <c r="D513" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E513" s="74" t="s">
+      <c r="D513" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E513" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F513" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G513" s="74" t="s">
+      <c r="F513" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G513" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="514" spans="1:7" s="74" customFormat="1">
-      <c r="A514" s="74" t="s">
+    <row r="514" spans="1:7" s="72" customFormat="1">
+      <c r="A514" s="72" t="s">
         <v>345</v>
       </c>
-      <c r="B514" s="77">
+      <c r="B514" s="75">
         <v>1.2032999999999999E-7</v>
       </c>
-      <c r="D514" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E514" s="74" t="s">
+      <c r="D514" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E514" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F514" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G514" s="74" t="s">
+      <c r="F514" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G514" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="515" spans="1:7" s="74" customFormat="1">
-      <c r="A515" s="74" t="s">
+    <row r="515" spans="1:7" s="72" customFormat="1">
+      <c r="A515" s="72" t="s">
         <v>346</v>
       </c>
-      <c r="B515" s="77">
+      <c r="B515" s="75">
         <v>2.4787000000000001E-6</v>
       </c>
-      <c r="D515" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E515" s="74" t="s">
+      <c r="D515" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E515" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F515" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G515" s="74" t="s">
+      <c r="F515" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G515" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="516" spans="1:7" s="74" customFormat="1">
-      <c r="A516" s="74" t="s">
+    <row r="516" spans="1:7" s="72" customFormat="1">
+      <c r="A516" s="72" t="s">
         <v>347</v>
       </c>
-      <c r="B516" s="77">
+      <c r="B516" s="75">
         <v>1.0829E-7</v>
       </c>
-      <c r="D516" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E516" s="74" t="s">
+      <c r="D516" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E516" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F516" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G516" s="74" t="s">
+      <c r="F516" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G516" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="517" spans="1:7" s="74" customFormat="1">
-      <c r="A517" s="74" t="s">
+    <row r="517" spans="1:7" s="72" customFormat="1">
+      <c r="A517" s="72" t="s">
         <v>348</v>
       </c>
-      <c r="B517" s="77">
+      <c r="B517" s="75">
         <v>1.0107999999999999E-6</v>
       </c>
-      <c r="D517" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E517" s="74" t="s">
+      <c r="D517" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E517" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F517" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G517" s="74" t="s">
+      <c r="F517" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G517" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="518" spans="1:7" s="74" customFormat="1">
-      <c r="A518" s="74" t="s">
+    <row r="518" spans="1:7" s="72" customFormat="1">
+      <c r="A518" s="72" t="s">
         <v>349</v>
       </c>
-      <c r="B518" s="77">
+      <c r="B518" s="75">
         <v>2.4065000000000001E-8</v>
       </c>
-      <c r="D518" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E518" s="74" t="s">
+      <c r="D518" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E518" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F518" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G518" s="74" t="s">
+      <c r="F518" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G518" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="519" spans="1:7" s="74" customFormat="1">
-      <c r="A519" s="74" t="s">
+    <row r="519" spans="1:7" s="72" customFormat="1">
+      <c r="A519" s="72" t="s">
         <v>350</v>
       </c>
-      <c r="B519" s="77">
+      <c r="B519" s="75">
         <v>-3.2893999999999998E-7</v>
       </c>
-      <c r="D519" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E519" s="74" t="s">
+      <c r="D519" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E519" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F519" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G519" s="74" t="s">
+      <c r="F519" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G519" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="520" spans="1:7" s="74" customFormat="1">
-      <c r="A520" s="74" t="s">
+    <row r="520" spans="1:7" s="72" customFormat="1">
+      <c r="A520" s="72" t="s">
         <v>351</v>
       </c>
-      <c r="B520" s="77">
+      <c r="B520" s="75">
         <v>7.9416000000000001E-7</v>
       </c>
-      <c r="D520" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E520" s="74" t="s">
+      <c r="D520" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E520" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F520" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G520" s="74" t="s">
+      <c r="F520" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G520" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="521" spans="1:7" s="74" customFormat="1">
-      <c r="A521" s="74" t="s">
+    <row r="521" spans="1:7" s="72" customFormat="1">
+      <c r="A521" s="72" t="s">
         <v>352</v>
       </c>
-      <c r="B521" s="77">
+      <c r="B521" s="75">
         <v>4.1393000000000003E-6</v>
       </c>
-      <c r="D521" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E521" s="74" t="s">
+      <c r="D521" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E521" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F521" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G521" s="74" t="s">
+      <c r="F521" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G521" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="522" spans="1:7" s="74" customFormat="1">
-      <c r="A522" s="74" t="s">
+    <row r="522" spans="1:7" s="72" customFormat="1">
+      <c r="A522" s="72" t="s">
         <v>353</v>
       </c>
-      <c r="B522" s="77">
+      <c r="B522" s="75">
         <v>5.0537999999999999E-8</v>
       </c>
-      <c r="D522" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E522" s="74" t="s">
+      <c r="D522" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E522" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F522" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G522" s="74" t="s">
+      <c r="F522" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G522" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="523" spans="1:7" s="74" customFormat="1">
-      <c r="A523" s="74" t="s">
+    <row r="523" spans="1:7" s="72" customFormat="1">
+      <c r="A523" s="72" t="s">
         <v>354</v>
       </c>
-      <c r="B523" s="77">
+      <c r="B523" s="75">
         <v>-5.9000999999999996E-6</v>
       </c>
-      <c r="D523" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E523" s="74" t="s">
+      <c r="D523" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E523" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F523" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G523" s="74" t="s">
+      <c r="F523" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G523" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="524" spans="1:7" s="74" customFormat="1">
-      <c r="A524" s="74" t="s">
+    <row r="524" spans="1:7" s="72" customFormat="1">
+      <c r="A524" s="72" t="s">
         <v>355</v>
       </c>
-      <c r="B524" s="77">
+      <c r="B524" s="75">
         <v>1.5643E-6</v>
       </c>
-      <c r="D524" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E524" s="74" t="s">
+      <c r="D524" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E524" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F524" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G524" s="74" t="s">
+      <c r="F524" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G524" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="525" spans="1:7" s="74" customFormat="1">
-      <c r="A525" s="74" t="s">
+    <row r="525" spans="1:7" s="72" customFormat="1">
+      <c r="A525" s="72" t="s">
         <v>356</v>
       </c>
-      <c r="B525" s="77">
+      <c r="B525" s="75">
         <v>2.6952999999999998E-6</v>
       </c>
-      <c r="D525" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E525" s="74" t="s">
+      <c r="D525" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E525" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F525" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G525" s="74" t="s">
+      <c r="F525" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G525" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="526" spans="1:7" s="74" customFormat="1">
-      <c r="A526" s="74" t="s">
+    <row r="526" spans="1:7" s="72" customFormat="1">
+      <c r="A526" s="72" t="s">
         <v>357</v>
       </c>
-      <c r="B526" s="77">
+      <c r="B526" s="75">
         <v>4.4454999999999997E-8</v>
       </c>
-      <c r="D526" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E526" s="74" t="s">
+      <c r="D526" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E526" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F526" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G526" s="74" t="s">
+      <c r="F526" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G526" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="527" spans="1:7" s="74" customFormat="1">
-      <c r="A527" s="74" t="s">
+    <row r="527" spans="1:7" s="72" customFormat="1">
+      <c r="A527" s="72" t="s">
         <v>358</v>
       </c>
-      <c r="B527" s="77">
+      <c r="B527" s="75">
         <v>3.6097999999999997E-8</v>
       </c>
-      <c r="D527" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E527" s="74" t="s">
+      <c r="D527" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E527" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F527" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G527" s="74" t="s">
+      <c r="F527" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G527" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="528" spans="1:7" s="74" customFormat="1">
-      <c r="A528" s="74" t="s">
+    <row r="528" spans="1:7" s="72" customFormat="1">
+      <c r="A528" s="72" t="s">
         <v>359</v>
       </c>
-      <c r="B528" s="77">
+      <c r="B528" s="75">
         <v>2.1659000000000001E-7</v>
       </c>
-      <c r="D528" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E528" s="74" t="s">
+      <c r="D528" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E528" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F528" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G528" s="74" t="s">
+      <c r="F528" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G528" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="529" spans="1:7" s="74" customFormat="1">
-      <c r="A529" s="74" t="s">
+    <row r="529" spans="1:7" s="72" customFormat="1">
+      <c r="A529" s="72" t="s">
         <v>360</v>
       </c>
-      <c r="B529" s="77">
+      <c r="B529" s="75">
         <v>-1.8835E-8</v>
       </c>
-      <c r="D529" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E529" s="74" t="s">
+      <c r="D529" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E529" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F529" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G529" s="74" t="s">
+      <c r="F529" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G529" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="530" spans="1:7" s="74" customFormat="1">
-      <c r="A530" s="74" t="s">
+    <row r="530" spans="1:7" s="72" customFormat="1">
+      <c r="A530" s="72" t="s">
         <v>288</v>
       </c>
-      <c r="B530" s="77">
+      <c r="B530" s="75">
         <v>4.2885E-5</v>
       </c>
-      <c r="D530" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E530" s="74" t="s">
+      <c r="D530" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E530" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F530" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G530" s="74" t="s">
+      <c r="F530" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G530" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="531" spans="1:7" s="74" customFormat="1">
-      <c r="A531" s="74" t="s">
+    <row r="531" spans="1:7" s="72" customFormat="1">
+      <c r="A531" s="72" t="s">
         <v>282</v>
       </c>
-      <c r="B531" s="77">
+      <c r="B531" s="75">
         <v>9.2460000000000006E-5</v>
       </c>
-      <c r="D531" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E531" s="74" t="s">
+      <c r="D531" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E531" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F531" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G531" s="74" t="s">
+      <c r="F531" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G531" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="532" spans="1:7" s="74" customFormat="1">
-      <c r="A532" s="74" t="s">
+    <row r="532" spans="1:7" s="72" customFormat="1">
+      <c r="A532" s="72" t="s">
         <v>361</v>
       </c>
-      <c r="B532" s="77">
+      <c r="B532" s="75">
         <v>5.0297000000000003E-6</v>
       </c>
-      <c r="D532" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E532" s="74" t="s">
+      <c r="D532" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E532" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F532" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G532" s="74" t="s">
+      <c r="F532" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G532" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="533" spans="1:7" s="74" customFormat="1">
-      <c r="A533" s="74" t="s">
+    <row r="533" spans="1:7" s="72" customFormat="1">
+      <c r="A533" s="72" t="s">
         <v>362</v>
       </c>
-      <c r="B533" s="77">
+      <c r="B533" s="75">
         <v>2.4306000000000001E-6</v>
       </c>
-      <c r="D533" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E533" s="74" t="s">
+      <c r="D533" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E533" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F533" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G533" s="74" t="s">
+      <c r="F533" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G533" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="534" spans="1:7" s="74" customFormat="1">
-      <c r="A534" s="74" t="s">
+    <row r="534" spans="1:7" s="72" customFormat="1">
+      <c r="A534" s="72" t="s">
         <v>363</v>
       </c>
-      <c r="B534" s="77">
+      <c r="B534" s="75">
         <v>1.7326999999999999E-6</v>
       </c>
-      <c r="D534" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E534" s="74" t="s">
+      <c r="D534" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E534" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F534" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G534" s="74" t="s">
+      <c r="F534" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G534" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="535" spans="1:7" s="74" customFormat="1">
-      <c r="A535" s="74" t="s">
+    <row r="535" spans="1:7" s="72" customFormat="1">
+      <c r="A535" s="72" t="s">
         <v>364</v>
       </c>
-      <c r="B535" s="77">
+      <c r="B535" s="75">
         <v>2.8878999999999998E-7</v>
       </c>
-      <c r="D535" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E535" s="74" t="s">
+      <c r="D535" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E535" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F535" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G535" s="74" t="s">
+      <c r="F535" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G535" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="536" spans="1:7" s="74" customFormat="1">
-      <c r="A536" s="74" t="s">
+    <row r="536" spans="1:7" s="72" customFormat="1">
+      <c r="A536" s="72" t="s">
         <v>287</v>
       </c>
-      <c r="B536" s="77">
+      <c r="B536" s="75">
         <v>1.9661999999999999E-5</v>
       </c>
-      <c r="D536" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E536" s="74" t="s">
+      <c r="D536" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E536" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F536" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G536" s="74" t="s">
+      <c r="F536" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G536" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="537" spans="1:7" s="74" customFormat="1">
-      <c r="A537" s="74" t="s">
+    <row r="537" spans="1:7" s="72" customFormat="1">
+      <c r="A537" s="72" t="s">
         <v>365</v>
       </c>
-      <c r="B537" s="77">
+      <c r="B537" s="75">
         <v>1.1911999999999999E-6</v>
       </c>
-      <c r="D537" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E537" s="74" t="s">
+      <c r="D537" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E537" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F537" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G537" s="74" t="s">
+      <c r="F537" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G537" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="538" spans="1:7" s="74" customFormat="1">
-      <c r="A538" s="74" t="s">
+    <row r="538" spans="1:7" s="72" customFormat="1">
+      <c r="A538" s="72" t="s">
         <v>366</v>
       </c>
-      <c r="B538" s="77">
+      <c r="B538" s="75">
         <v>1.9252000000000001E-7</v>
       </c>
-      <c r="D538" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E538" s="74" t="s">
+      <c r="D538" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E538" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F538" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G538" s="74" t="s">
+      <c r="F538" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G538" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="539" spans="1:7" s="74" customFormat="1">
-      <c r="A539" s="74" t="s">
+    <row r="539" spans="1:7" s="72" customFormat="1">
+      <c r="A539" s="72" t="s">
         <v>367</v>
       </c>
-      <c r="B539" s="77">
+      <c r="B539" s="75">
         <v>3.0442999999999998E-6</v>
       </c>
-      <c r="D539" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E539" s="74" t="s">
+      <c r="D539" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E539" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F539" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G539" s="74" t="s">
+      <c r="F539" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G539" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="540" spans="1:7" s="74" customFormat="1">
-      <c r="A540" s="74" t="s">
+    <row r="540" spans="1:7" s="72" customFormat="1">
+      <c r="A540" s="72" t="s">
         <v>368</v>
       </c>
-      <c r="B540" s="77">
+      <c r="B540" s="75">
         <v>4.8130999999999997E-6</v>
       </c>
-      <c r="D540" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E540" s="74" t="s">
+      <c r="D540" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E540" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F540" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G540" s="74" t="s">
+      <c r="F540" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G540" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="541" spans="1:7" s="74" customFormat="1">
-      <c r="A541" s="74" t="s">
+    <row r="541" spans="1:7" s="72" customFormat="1">
+      <c r="A541" s="72" t="s">
         <v>369</v>
       </c>
-      <c r="B541" s="77">
+      <c r="B541" s="75">
         <v>5.9441999999999998E-5</v>
       </c>
-      <c r="D541" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E541" s="74" t="s">
+      <c r="D541" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E541" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F541" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G541" s="74" t="s">
+      <c r="F541" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G541" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="542" spans="1:7" s="74" customFormat="1">
-      <c r="A542" s="74" t="s">
+    <row r="542" spans="1:7" s="72" customFormat="1">
+      <c r="A542" s="72" t="s">
         <v>370</v>
       </c>
-      <c r="B542" s="77">
+      <c r="B542" s="75">
         <v>3.3691999999999998E-7</v>
       </c>
-      <c r="D542" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E542" s="74" t="s">
+      <c r="D542" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E542" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F542" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G542" s="74" t="s">
+      <c r="F542" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G542" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="543" spans="1:7" s="74" customFormat="1">
-      <c r="A543" s="74" t="s">
+    <row r="543" spans="1:7" s="72" customFormat="1">
+      <c r="A543" s="72" t="s">
         <v>371</v>
       </c>
-      <c r="B543" s="77">
+      <c r="B543" s="75">
         <v>1.6846000000000001E-8</v>
       </c>
-      <c r="D543" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E543" s="74" t="s">
+      <c r="D543" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E543" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F543" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G543" s="74" t="s">
+      <c r="F543" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G543" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="544" spans="1:7" s="74" customFormat="1">
-      <c r="A544" s="74" t="s">
+    <row r="544" spans="1:7" s="72" customFormat="1">
+      <c r="A544" s="72" t="s">
         <v>372</v>
       </c>
-      <c r="B544" s="77">
+      <c r="B544" s="75">
         <v>5.7757E-7</v>
       </c>
-      <c r="D544" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E544" s="74" t="s">
+      <c r="D544" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E544" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F544" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G544" s="74" t="s">
+      <c r="F544" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G544" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="545" spans="1:7" s="74" customFormat="1">
-      <c r="A545" s="74" t="s">
+    <row r="545" spans="1:7" s="72" customFormat="1">
+      <c r="A545" s="72" t="s">
         <v>373</v>
       </c>
-      <c r="B545" s="77">
+      <c r="B545" s="75">
         <v>2.1658999999999999E-8</v>
       </c>
-      <c r="D545" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E545" s="74" t="s">
+      <c r="D545" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E545" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F545" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G545" s="74" t="s">
+      <c r="F545" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G545" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="546" spans="1:7" s="74" customFormat="1">
-      <c r="A546" s="74" t="s">
+    <row r="546" spans="1:7" s="72" customFormat="1">
+      <c r="A546" s="72" t="s">
         <v>374</v>
       </c>
-      <c r="B546" s="77">
+      <c r="B546" s="75">
         <v>3.6097999999999997E-8</v>
       </c>
-      <c r="D546" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E546" s="74" t="s">
+      <c r="D546" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E546" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F546" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G546" s="74" t="s">
+      <c r="F546" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G546" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="547" spans="1:7" s="74" customFormat="1">
-      <c r="A547" s="74" t="s">
+    <row r="547" spans="1:7" s="72" customFormat="1">
+      <c r="A547" s="72" t="s">
         <v>375</v>
       </c>
-      <c r="B547" s="77">
+      <c r="B547" s="75">
         <v>2.6472E-7</v>
       </c>
-      <c r="D547" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E547" s="74" t="s">
+      <c r="D547" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E547" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F547" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G547" s="74" t="s">
+      <c r="F547" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G547" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="548" spans="1:7" s="74" customFormat="1">
-      <c r="A548" s="74" t="s">
+    <row r="548" spans="1:7" s="72" customFormat="1">
+      <c r="A548" s="72" t="s">
         <v>376</v>
       </c>
-      <c r="B548" s="77">
+      <c r="B548" s="75">
         <v>1.2032999999999999E-7</v>
       </c>
-      <c r="D548" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E548" s="74" t="s">
+      <c r="D548" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E548" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F548" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G548" s="74" t="s">
+      <c r="F548" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G548" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="549" spans="1:7" s="74" customFormat="1">
-      <c r="A549" s="74" t="s">
+    <row r="549" spans="1:7" s="72" customFormat="1">
+      <c r="A549" s="72" t="s">
         <v>377</v>
       </c>
-      <c r="B549" s="77">
+      <c r="B549" s="75">
         <v>2.6436999999999998E-7</v>
       </c>
-      <c r="D549" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E549" s="74" t="s">
+      <c r="D549" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E549" s="72" t="s">
         <v>283</v>
       </c>
-      <c r="F549" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G549" s="74" t="s">
+      <c r="F549" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G549" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="550" spans="1:7" s="74" customFormat="1">
-      <c r="A550" s="74" t="s">
+    <row r="550" spans="1:7" s="72" customFormat="1">
+      <c r="A550" s="72" t="s">
         <v>130</v>
       </c>
-      <c r="B550" s="77">
+      <c r="B550" s="75">
         <v>5.9736877488796199E-2</v>
       </c>
-      <c r="D550" s="74" t="s">
+      <c r="D550" s="72" t="s">
         <v>128</v>
       </c>
-      <c r="E550" s="74" t="s">
+      <c r="E550" s="72" t="s">
         <v>241</v>
       </c>
-      <c r="F550" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G550" s="74" t="s">
+      <c r="F550" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G550" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="551" spans="1:7" s="74" customFormat="1">
-      <c r="A551" s="74" t="s">
+    <row r="551" spans="1:7" s="72" customFormat="1">
+      <c r="A551" s="72" t="s">
         <v>240</v>
       </c>
-      <c r="B551" s="77">
+      <c r="B551" s="75">
         <v>1.1639108E-2</v>
       </c>
-      <c r="D551" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E551" s="74" t="s">
+      <c r="D551" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E551" s="72" t="s">
         <v>241</v>
       </c>
-      <c r="F551" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G551" s="74" t="s">
+      <c r="F551" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G551" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="552" spans="1:7" s="74" customFormat="1">
-      <c r="A552" s="74" t="s">
+    <row r="552" spans="1:7" s="72" customFormat="1">
+      <c r="A552" s="72" t="s">
         <v>130</v>
       </c>
-      <c r="B552" s="77">
+      <c r="B552" s="75">
         <v>1.4934219372198999E-2</v>
       </c>
-      <c r="D552" s="74" t="s">
+      <c r="D552" s="72" t="s">
         <v>128</v>
       </c>
-      <c r="E552" s="74" t="s">
+      <c r="E552" s="72" t="s">
         <v>284</v>
       </c>
-      <c r="F552" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G552" s="74" t="s">
+      <c r="F552" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G552" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="553" spans="1:7" s="74" customFormat="1">
-      <c r="A553" s="74" t="s">
+    <row r="553" spans="1:7" s="72" customFormat="1">
+      <c r="A553" s="72" t="s">
         <v>291</v>
       </c>
-      <c r="B553" s="77">
+      <c r="B553" s="75">
         <v>9.7541999999999995E-5</v>
       </c>
-      <c r="D553" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E553" s="74" t="s">
+      <c r="D553" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E553" s="72" t="s">
         <v>284</v>
       </c>
-      <c r="F553" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G553" s="74" t="s">
+      <c r="F553" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G553" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="554" spans="1:7" s="74" customFormat="1">
-      <c r="A554" s="74" t="s">
+    <row r="554" spans="1:7" s="72" customFormat="1">
+      <c r="A554" s="72" t="s">
         <v>290</v>
       </c>
-      <c r="B554" s="77">
+      <c r="B554" s="75">
         <v>7.5147999999999996E-6</v>
       </c>
-      <c r="D554" s="74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E554" s="74" t="s">
+      <c r="D554" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="E554" s="72" t="s">
         <v>284</v>
       </c>
-      <c r="F554" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G554" s="74" t="s">
+      <c r="F554" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G554" s="72" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="555" spans="1:7" s="74" customFormat="1">
-      <c r="A555" s="74" t="s">
+    <row r="555" spans="1:7" s="72" customFormat="1">
+      <c r="A555" s="72" t="s">
         <v>378</v>
       </c>
-      <c r="B555" s="77">
+      <c r="B555" s="75">
         <v>0</v>
       </c>
-      <c r="D555" s="74" t="s">
+      <c r="D555" s="72" t="s">
         <v>128</v>
       </c>
-      <c r="E555" s="74" t="s">
+      <c r="E555" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="F555" s="74" t="s">
-        <v>15</v>
-      </c>
-      <c r="G555" s="83" t="s">
+      <c r="F555" s="72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G555" s="81" t="s">
         <v>379</v>
       </c>
     </row>
@@ -18479,7 +18477,7 @@
       <c r="A558" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B558" s="70" t="s">
+      <c r="B558" t="s">
         <v>496</v>
       </c>
     </row>
@@ -18876,7 +18874,7 @@
       <c r="A582" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B582" s="70" t="s">
+      <c r="B582" t="s">
         <v>497</v>
       </c>
     </row>
@@ -19453,7 +19451,7 @@
       <c r="A614" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B614" s="70" t="s">
+      <c r="B614" t="s">
         <v>498</v>
       </c>
     </row>
@@ -20030,7 +20028,7 @@
       <c r="A646" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B646" s="70" t="s">
+      <c r="B646" t="s">
         <v>499</v>
       </c>
     </row>
@@ -20607,7 +20605,7 @@
       <c r="A678" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B678" s="70" t="s">
+      <c r="B678" t="s">
         <v>500</v>
       </c>
     </row>
@@ -21184,7 +21182,7 @@
       <c r="A710" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B710" s="70" t="s">
+      <c r="B710" t="s">
         <v>501</v>
       </c>
     </row>
@@ -21581,7 +21579,7 @@
       <c r="A734" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B734" s="70" t="s">
+      <c r="B734" t="s">
         <v>502</v>
       </c>
     </row>
@@ -22158,7 +22156,7 @@
       <c r="A766" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B766" s="70" t="s">
+      <c r="B766" t="s">
         <v>503</v>
       </c>
     </row>
@@ -22735,7 +22733,7 @@
       <c r="A798" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B798" s="70" t="s">
+      <c r="B798" t="s">
         <v>504</v>
       </c>
     </row>
@@ -23312,7 +23310,7 @@
       <c r="A830" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B830" s="70" t="s">
+      <c r="B830" t="s">
         <v>505</v>
       </c>
     </row>

</xml_diff>